<commit_message>
Corrige les dates de 5 philosophes orientaux
Vivekananda (1863–1902) et Sri Aurobindo (1872–1950) affichaient les dates
d'autres penseurs ; Mirabai (1498–1547), Lu Xiangshan (1139–1193) et
Huang Zongxi (1610–1695) avaient des dates erronées. Corrigé dans le xlsx
(cellules modifiées une à une) et les données régénérées.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -5187,15 +5187,15 @@
       </c>
     </row>
     <row r="76" ht="157.5" customHeight="1" s="25">
-      <c r="A76" s="30" t="n">
-        <v>1130</v>
-      </c>
-      <c r="B76" s="30" t="n">
-        <v>1200</v>
+      <c r="A76" s="30">
+        <v>1139</v>
+      </c>
+      <c r="B76" s="30">
+        <v>1193</v>
       </c>
       <c r="C76" s="30" t="inlineStr">
         <is>
-          <t>1130 — 1200</t>
+          <t>1139 — 1193</t>
         </is>
       </c>
       <c r="D76" s="31" t="inlineStr">
@@ -6234,15 +6234,15 @@
       </c>
     </row>
     <row r="93" ht="338.25" customHeight="1" s="25">
-      <c r="A93" s="30" t="n">
-        <v>1440</v>
-      </c>
-      <c r="B93" s="30" t="n">
-        <v>1518</v>
+      <c r="A93" s="30">
+        <v>1498</v>
+      </c>
+      <c r="B93" s="30">
+        <v>1547</v>
       </c>
       <c r="C93" s="30" t="inlineStr">
         <is>
-          <t>1440 - 1518</t>
+          <t>1498 – 1547</t>
         </is>
       </c>
       <c r="D93" s="31" t="inlineStr">
@@ -6792,15 +6792,15 @@
       </c>
     </row>
     <row r="102" ht="255.75" customHeight="1" s="25">
-      <c r="A102" s="23" t="n">
-        <v>1633</v>
-      </c>
-      <c r="B102" s="23" t="n">
-        <v>1682</v>
+      <c r="A102" s="23">
+        <v>1610</v>
+      </c>
+      <c r="B102" s="23">
+        <v>1695</v>
       </c>
       <c r="C102" s="23" t="inlineStr">
         <is>
-          <t>1633 — 1682</t>
+          <t>1610 — 1695</t>
         </is>
       </c>
       <c r="D102" s="24" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="C114" s="23" t="inlineStr">
         <is>
-          <t>1238 — 1317</t>
+          <t>1863 — 1902</t>
         </is>
       </c>
       <c r="D114" s="24" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="C117" s="23" t="inlineStr">
         <is>
-          <t>1895 — 1986</t>
+          <t>1872 — 1950</t>
         </is>
       </c>
       <c r="D117" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Ajoute 20 fiches du Proche-Orient ancien
Égypte : Kagemni, Hordjédef, Enseignement pour Mérikarê, Dialogue du
désespéré avec son ba, Ipou-our, Akhenaton, Amenemopet, Ânkhsheshonqy.
Mésopotamie : Shuruppak, Enheduanna, Hammurabi, Ludlul bel nemeqi,
Dialogue du pessimisme, Ahiqar, Bérose. Perse : Zarathoustra. Phénicie :
Sanchoniathon. Sagesse biblique et syriaque : Livre de Job, Qohélet,
Bardesane. Dates vérifiées sur Wikipédia ; groupe orient-ancien (le
couloir passe de 8 à 28 penseurs). Images et vidéos à venir.

xlsx_cellules.py crée désormais une ligne absente (avec les attributs de
la précédente) et agrandit la zone déclarée <dimension> du classeur.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N139"/>
+  <dimension ref="A1:P159"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9.869999999999999" customWidth="1" style="23" min="1" max="1"/>
@@ -9917,41 +9917,992 @@
       </c>
     </row>
     <row r="140" ht="128.25" customHeight="1" s="25">
-      <c r="D140" s="23" t="n"/>
-      <c r="E140" s="23" t="n"/>
-      <c r="K140" s="23" t="n"/>
-      <c r="L140" s="23" t="n"/>
-      <c r="M140" s="23" t="n"/>
+      <c r="A140" s="23">
+        <v>-2600</v>
+      </c>
+      <c r="B140" s="23">
+        <v>-2540</v>
+      </c>
+      <c r="C140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 2600 A JC</t>
+        </is>
+      </c>
+      <c r="D140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KAGEMNI</t>
+        </is>
+      </c>
+      <c r="E140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Kagemni_(vizir_de_Snéfrou)"  title=" Wikipedia"&gt;KAGEMNI&lt;/a&gt; était un vizir de l'Ancien Empire égyptien, au service du pharaon Snéfrou (vers 2613-2589 avant J.-C.), fondateur de la IVe dynastie. Son nom reste attaché à l'&lt;em&gt;Enseignement pour Kagemni&lt;/em&gt;, un court texte de sagesse conservé sur le célèbre papyrus Prisse, le même manuscrit qui contient les maximes de Ptahhotep.&lt;/p&gt; &lt;p&gt;Comme beaucoup d'enseignements égyptiens, ce texte a sans doute été rédigé plus tard, au Moyen Empire, puis placé sous l'autorité d'un sage du passé. Il se présente comme les conseils d'un père à ses enfants : on y loue la modestie, la maîtrise de soi et la retenue à table comme dans les paroles, et l'on met en garde contre l'orgueil et la gloutonnerie.&lt;/p&gt; &lt;p&gt;L'enseignement commence par une phrase restée célèbre : « L'homme respectueux prospère, le modeste est loué ; la tente est ouverte au silencieux ». Le silence, la discrétion et la politesse y sont présentés comme des vertus sociales, qui protègent contre les conflits et attirent la faveur des supérieurs. La gourmandise est vue comme un manque de maîtrise : celui qui se jette sur la nourriture se laisse gouverner par ses désirs au lieu de se gouverner lui-même.&lt;/p&gt; &lt;p&gt;Ce type de texte, appelé &lt;em&gt;sebayt&lt;/em&gt; (« enseignement »), était copié et recopié par les apprentis scribes. Il servait à la fois à apprendre à écrire et à former le caractère des futurs fonctionnaires de l'État égyptien. La sagesse n'y est pas une spéculation abstraite, mais une éducation pratique à la vie en société.&lt;/p&gt; &lt;p&gt;Derrière ces règles de conduite se dessine une idée centrale de la pensée égyptienne : l'homme sage est celui qui sait se tenir à sa place et préserver l'harmonie de l'ordre social, reflet de la Maât, l'ordre juste du monde.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique</t>
+        </is>
+      </c>
+      <c r="L140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M140" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vizir égyptien à qui est attribué l'un des plus anciens enseignements de sagesse.</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="25">
-      <c r="D141" s="23" t="n"/>
-      <c r="K141" s="23" t="n"/>
-      <c r="L141" s="23" t="n"/>
-      <c r="M141" s="23" t="n"/>
+      <c r="A141" s="23">
+        <v>-2550</v>
+      </c>
+      <c r="B141" s="23">
+        <v>-2480</v>
+      </c>
+      <c r="C141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 2550 A JC</t>
+        </is>
+      </c>
+      <c r="D141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HORDJÉDEF</t>
+        </is>
+      </c>
+      <c r="E141" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hordjédef"  title=" Wikipedia"&gt;HORDJÉDEF&lt;/a&gt; était un prince de la IVe dynastie égyptienne, fils du pharaon Khéops, qui vécut vers 2550 avant J.-C. Les Égyptiens eux-mêmes le tenaient pour l'un des plus grands sages de leur histoire : son nom est cité avec admiration jusqu'à l'époque romaine.&lt;/p&gt; &lt;p&gt;On lui attribue un &lt;em&gt;Enseignement&lt;/em&gt; adressé à son fils Aouibrê, dont il ne subsiste que des fragments. Le texte, sans doute composé au Moyen Empire, conseille de fonder un foyer, d'élever un fils et de préparer dignement sa tombe : la sagesse y est d'abord une manière de bien vivre pour bien mourir, en assurant sa mémoire et la continuité de sa lignée.&lt;/p&gt; &lt;p&gt;La célébrité d'Hordjédef dépasse largement ce texte. Un papyrus raconte qu'il fit venir à la cour de son père le magicien Djédi, et le Livre des morts lui attribue la découverte de certaines formules sacrées. Plus tard, les Égyptiens le rangèrent parmi les grands sages du passé, aux côtés d'Imhotep et de Ptahhotep, dont « les noms durent à cause de leurs livres ».&lt;/p&gt; &lt;p&gt;Cette idée est essentielle dans la culture égyptienne : l'écrit est une forme d'immortalité. Plus sûrement qu'une pyramide ou une tombe, le livre transmet le nom et la pensée de son auteur aux générations futures. Hordjédef devient ainsi le symbole du sage dont la parole survit au temps.&lt;/p&gt; &lt;p&gt;Hordjédef illustre une figure typique de la pensée égyptienne : le sage n'est pas un penseur solitaire mais un homme de rang qui transmet à ses descendants un art de vivre conforme à l'ordre du monde.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique;spiritualite</t>
+        </is>
+      </c>
+      <c r="L141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M141" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prince égyptien, fils de Khéops, auteur présumé de l'un des plus anciens enseignements de sagesse.</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="25">
-      <c r="D142" s="23" t="n"/>
-      <c r="K142" s="23" t="n"/>
-      <c r="L142" s="23" t="n"/>
-      <c r="M142" s="23" t="n"/>
+      <c r="A142" s="23">
+        <v>-2500</v>
+      </c>
+      <c r="B142" s="23">
+        <v>-2400</v>
+      </c>
+      <c r="C142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 2500 A JC</t>
+        </is>
+      </c>
+      <c r="D142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHURUPPAK</t>
+        </is>
+      </c>
+      <c r="E142" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Les &lt;a href="https://fr.wikipedia.org/wiki/Instructions_de_Shuruppak"  title=" Wikipedia"&gt;Instructions de SHURUPPAK&lt;/a&gt; sont l'un des plus anciens textes de sagesse de l'humanité : leurs premières versions, rédigées en sumérien, remontent à environ 2500 avant J.-C. Elles mettent en scène Shuruppak, sage et roi légendaire, qui transmet ses conseils à son fils Ziusudra, le héros sumérien du Déluge.&lt;/p&gt; &lt;p&gt;Les préceptes couvrent tous les domaines de la vie : ne pas voler, ne pas commettre de violence, respecter ses parents, se méfier des paroles imprudentes, choisir avec soin ses terres et ses alliances, et gouverner avec mesure. On y trouve déjà la forme qui fera le succès de la littérature de sagesse du Proche-Orient : des maximes brèves, faciles à retenir, fondées sur l'expérience.&lt;/p&gt; &lt;p&gt;Le texte a été retrouvé sous plusieurs formes, du site d'Abu Salabikh à des copies plus tardives de l'époque paléo-babylonienne, signe qu'il a été enseigné et recopié pendant des siècles dans les écoles de scribes, les « maisons des tablettes ». Certains conseils paraissent très concrets, comme ne pas construire sa maison près d'une place publique ou ne pas acheter un âne qui braie ; d'autres ont une portée morale plus générale, comme ne pas proférer de mensonges ou ne pas se montrer arrogant.&lt;/p&gt; &lt;p&gt;La figure de Ziusudra, le fils qui reçoit ces instructions, est celle du survivant du Déluge dans la tradition sumérienne, l'équivalent d'Uta-napishti dans l'Épopée de Gilgamesh et de Noé dans la Bible. La sagesse est ainsi placée à l'origine même de l'humanité, comme un savoir transmis depuis les temps les plus anciens.&lt;/p&gt; &lt;p&gt;Ce texte montre qu'une réflexion morale structurée existait en Mésopotamie bien avant la philosophie grecque, et qu'elle a nourri toute une tradition, jusqu'aux Proverbes de la Bible.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique;politique</t>
+        </is>
+      </c>
+      <c r="L142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M142" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sage légendaire de Sumer, à qui sont attribuées les plus anciennes instructions de sagesse connues.</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="128.25" customHeight="1" s="25">
-      <c r="D143" s="23" t="n"/>
-      <c r="K143" s="23" t="n"/>
-      <c r="L143" s="23" t="n"/>
-      <c r="M143" s="23" t="n"/>
+      <c r="A143" s="23">
+        <v>-2285</v>
+      </c>
+      <c r="B143" s="23">
+        <v>-2250</v>
+      </c>
+      <c r="C143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 2285 A JC - 2250 A JC</t>
+        </is>
+      </c>
+      <c r="D143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENHEDUANNA</t>
+        </is>
+      </c>
+      <c r="E143" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Enheduana"  title=" Wikipedia"&gt;ENHEDUANNA&lt;/a&gt; était la fille du roi Sargon d'Akkad et la grande prêtresse du dieu-lune Nanna dans la ville d'Ur, au XXIIIe siècle avant J.-C. Elle est la plus ancienne personne connue à nous avoir laissé une œuvre littéraire signée de son nom.&lt;/p&gt; &lt;p&gt;On lui attribue des hymnes majeurs, dont &lt;em&gt;L'Exaltation d'Inanna&lt;/em&gt;, où elle raconte à la première personne son exil et sa détresse avant son retour en grâce, et un recueil de quarante-deux &lt;em&gt;Hymnes aux temples&lt;/em&gt; de Sumer et d'Akkad. Par ces textes, elle contribua à unifier les croyances des Sumériens et des Akkadiens autour de divinités communes.&lt;/p&gt; &lt;p&gt;Sa nomination comme grande prêtresse d'Ur n'était pas seulement religieuse : en plaçant sa fille au cœur du culte sumérien, Sargon, roi akkadien, consolidait son pouvoir sur les cités de Sumer. Enheduanna fut ainsi à la fois une autorité spirituelle et un acteur politique. Lors d'une révolte, elle fut chassée de son temple, épisode qu'elle évoque dans ses hymnes avant d'être rétablie dans ses fonctions.&lt;/p&gt; &lt;p&gt;Ses textes furent recopiés pendant des siècles dans les écoles de scribes, bien après sa mort, ce qui montre l'importance qu'on leur accordait. Redécouverte au XXe siècle grâce aux fouilles d'Ur menées par l'archéologue Leonard Woolley, qui mit au jour un disque de calcite la représentant, elle est aujourd'hui étudiée comme la première autrice de l'histoire et une grande voix de la poésie religieuse.&lt;/p&gt; &lt;p&gt;Son œuvre mêle théologie, poésie et expérience personnelle : la relation au divin y devient une méditation sur le pouvoir, la souffrance et la fidélité, ce qui fait d'Enheduanna une figure fondatrice de la pensée religieuse et de la littérature.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite;esthetique</t>
+        </is>
+      </c>
+      <c r="L143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M143" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grande prêtresse d'Ur, fille de Sargon d'Akkad, premier auteur de l'histoire connu par son nom.</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P143">
+        <v>2</v>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="25">
-      <c r="D144" s="23" t="n"/>
-      <c r="K144" s="23" t="n"/>
-      <c r="L144" s="23" t="n"/>
-      <c r="M144" s="23" t="n"/>
+      <c r="A144" s="23">
+        <v>-2000</v>
+      </c>
+      <c r="B144" s="23">
+        <v>-1950</v>
+      </c>
+      <c r="C144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 2000 A JC</t>
+        </is>
+      </c>
+      <c r="D144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enseignement pour MÉRIKARÊ</t>
+        </is>
+      </c>
+      <c r="E144" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;L'&lt;a href="https://fr.wikipedia.org/wiki/Enseignement_pour_Mérikarê"  title=" Wikipedia"&gt;Enseignement pour MÉRIKARÊ&lt;/a&gt; est un texte égyptien composé vers 2000 avant J.-C., durant la Première Période intermédiaire, une époque de divisions et de troubles. Il se présente comme le testament d'un roi de la dynastie d'Héracléopolis adressé à son fils, le futur pharaon Mérikarê.&lt;/p&gt; &lt;p&gt;C'est un véritable traité sur l'art de gouverner : le roi doit être éloquent, car « la parole est plus forte que le combat », juste envers ses sujets, prudent face aux rebelles et attentif aux dieux. Le texte a ceci de remarquable qu'il reconnaît les fautes du père et confronte l'idéal de la royauté à la réalité du pouvoir.&lt;/p&gt; &lt;p&gt;Le texte est l'un des rares à évoquer les déchirements de son temps. Le roi y avoue avoir laissé ses troupes saccager des tombeaux dans la région d'Abydos, et reconnaît que ce crime lui a été rendu : « un coup est payé par un coup semblable ». L'aveu d'une faute royale est exceptionnel dans une civilisation où le pharaon était censé incarner l'ordre parfait.&lt;/p&gt; &lt;p&gt;La fin de l'enseignement contient un hymne au dieu créateur, qui a fait le ciel et la terre « à cause des hommes », leur a donné le souffle, la nourriture et la lumière, et veille sur eux « comme un berger sur son troupeau ». On y trouve l'une des premières expressions d'une providence divine bienveillante envers l'humanité tout entière, et non seulement envers le roi.&lt;/p&gt; &lt;p&gt;On y trouve aussi une réflexion morale d'une grande profondeur : le dieu préfère la vertu du juste au sacrifice du méchant, et chacun sera jugé sur ses actes après la mort.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique;ethique</t>
+        </is>
+      </c>
+      <c r="L144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M144" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">texte de sagesse égyptien sur l'art de gouverner, testament d'un roi à son fils.</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="25">
-      <c r="D145" s="23" t="n"/>
-      <c r="K145" s="23" t="n"/>
-      <c r="L145" s="23" t="n"/>
-      <c r="M145" s="23" t="n"/>
+      <c r="A145" s="23">
+        <v>-1860</v>
+      </c>
+      <c r="B145" s="23">
+        <v>-1814</v>
+      </c>
+      <c r="C145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1860 A JC - 1814 A JC</t>
+        </is>
+      </c>
+      <c r="D145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dialogue du DÉSESPÉRÉ avec son ba</t>
+        </is>
+      </c>
+      <c r="E145" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://en.wikipedia.org/wiki/Dispute_between_a_man_and_his_Ba"  title=" Wikipedia"&gt;Dialogue du DÉSESPÉRÉ avec son ba&lt;/a&gt; est un texte égyptien du Moyen Empire, daté du règne d'Amenemhat III (vers 1860-1814 avant J.-C.). Un homme accablé par la souffrance et l'injustice y dialogue avec son &lt;em&gt;ba&lt;/em&gt;, une part de son âme.&lt;/p&gt; &lt;p&gt;L'homme songe à mourir et vante la mort comme une délivrance ; son ba lui oppose d'abord la joie de vivre, puis menace de l'abandonner. La discussion, faite de poèmes d'une grande beauté (« La mort est devant moi aujourd'hui comme la guérison d'un malade »), aborde le sens de la vie, la valeur des rites funéraires et la solitude dans un monde où « il n'y a plus de juste ».&lt;/p&gt; &lt;p&gt;Le texte, conservé sur un papyrus aujourd'hui à Berlin dont le début est perdu, est d'une forme très élaborée. Il alterne des passages en prose, où l'homme et le ba argumentent, et quatre poèmes, construits sur des refrains : « Vois, mon nom est méprisé », « À qui parler aujourd'hui ? », « La mort est devant moi aujourd'hui », « Certes, celui qui est là-bas sera un dieu vivant ».&lt;/p&gt; &lt;p&gt;Le ba, pour sa part, rappelle que les tombeaux les plus somptueux finissent en ruine, comme ceux des pauvres, et invite l'homme à « suivre le jour heureux » et à oublier ses soucis. Les spécialistes discutent encore de la conclusion : le ba accepte-t-il de rester avec l'homme jusqu'à sa mort naturelle, ou consent-il à le suivre ? Cette ambiguïté fait toute la richesse du texte.&lt;/p&gt; &lt;p&gt;Souvent présenté comme le premier texte philosophique sur le suicide et le sens de l'existence, ce dialogue montre que la pensée égyptienne savait aussi douter et s'interroger.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;ethique</t>
+        </is>
+      </c>
+      <c r="L145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M145" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">texte égyptien où un homme désespéré débat de la vie et de la mort avec son âme.</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="15" customHeight="1" s="25">
+      <c r="A146" s="23">
+        <v>-1850</v>
+      </c>
+      <c r="B146" s="23">
+        <v>-1650</v>
+      </c>
+      <c r="C146" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1850 A JC</t>
+        </is>
+      </c>
+      <c r="D146" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IPOU-OUR</t>
+        </is>
+      </c>
+      <c r="E146" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Les &lt;a href="https://en.wikipedia.org/wiki/Ipuwer_Papyrus"  title=" Wikipedia"&gt;Lamentations d’IPOU-OUR&lt;/a&gt; sont un texte égyptien composé au plus tôt à la fin de la XIIe dynastie (vers 1850 avant J.-C.). Le sage Ipou-our s'y adresse au roi pour lui décrire un pays sens dessus dessous : les pauvres sont devenus riches, les nobles sont dans la misère, les lois ne sont plus respectées et le Nil lui-même semble ensanglanté.&lt;/p&gt; &lt;p&gt;Ce tableau d'un monde en chaos est moins une chronique historique qu'une réflexion sur ce qui arrive quand l'ordre juste, la Maât, n'est plus garanti. Ipou-our reproche même au dieu créateur de laisser faire le mal, et appelle un pouvoir fort à rétablir l'harmonie.&lt;/p&gt; &lt;p&gt;Le texte nous est parvenu sur un seul papyrus, conservé aujourd'hui au musée de Leyde, aux Pays-Bas, dont le début et la fin manquent. Il se compose de longues séries de lamentations commençant par le même refrain, « En vérité… », qui décrivent tour à tour la violence, la famine, le pillage des tombes, la fuite des serviteurs et l'effondrement de l'administration.&lt;/p&gt; &lt;p&gt;Certains y ont vu le témoignage d'une révolution sociale réelle, d'autres un écho des plaies d'Égypte du livre de l'Exode ; les égyptologues y lisent plutôt un genre littéraire, celui des « lamentations », qui montre l'image inversée de l'ordre idéal pour mieux en faire sentir la valeur. Le désordre décrit n'est pas seulement politique : c'est tout l'équilibre entre les hommes, la nature et les dieux qui semble rompu.&lt;/p&gt; &lt;p&gt;Le texte pose ainsi, très tôt, la question du mal et de la responsabilité des dirigeants et des dieux face au désordre du monde.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J146" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K146" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique;ethique</t>
+        </is>
+      </c>
+      <c r="L146" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M146" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sage égyptien dont les Lamentations décrivent un monde en chaos et interrogent le mal.</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="15" customHeight="1" s="25">
+      <c r="A147" s="23">
+        <v>-1792</v>
+      </c>
+      <c r="B147" s="23">
+        <v>-1750</v>
+      </c>
+      <c r="C147" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1792 A JC - 1750 A JC (règne)</t>
+        </is>
+      </c>
+      <c r="D147" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HAMMURABI</t>
+        </is>
+      </c>
+      <c r="E147" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hammurabi"  title=" Wikipedia"&gt;HAMMURABI&lt;/a&gt; fut roi de Babylone de 1792 à 1750 avant J.-C. (chronologie moyenne). Par ses conquêtes, il fit de sa cité la capitale d'un grand royaume mésopotamien.&lt;/p&gt; &lt;p&gt;Il est surtout connu pour le &lt;em&gt;Code de Hammurabi&lt;/em&gt;, gravé vers la fin de son règne sur une stèle de basalte aujourd'hui conservée au musée du Louvre. Ce recueil de près de trois cents décisions de justice règle la vie économique, familiale et sociale, avec le célèbre principe de la loi du talion (« œil pour œil »).&lt;/p&gt; &lt;p&gt;Le code ne se présente pas comme une législation abstraite mais comme une liste de cas : « si un homme a fait ceci, alors il lui sera fait cela ». Les peines varient selon le rang social de la victime et du coupable, homme libre, dépendant ou esclave, ce qui reflète une société très hiérarchisée. Le code traite des prix, des salaires, des prêts, du mariage, du divorce, de l'héritage, des soins médicaux et même de la responsabilité des architectes dont la maison s'effondre.&lt;/p&gt; &lt;p&gt;La loi du talion, qui paraît brutale aujourd'hui, avait aussi pour but de limiter la vengeance : la peine doit être proportionnée au dommage, et non illimitée. Le code affirme enfin que tout homme lésé peut venir lire la stèle pour connaître ses droits, idée d'une justice publique et accessible qui marque une étape importante dans l'histoire du droit.&lt;/p&gt; &lt;p&gt;Le prologue en donne la philosophie : le roi a reçu des dieux la mission de « faire apparaître la justice dans le pays, détruire le méchant et le pervers, afin que le fort n'opprime pas le faible ». L'idée que le pouvoir se justifie par la protection des plus faibles traversera toute l'histoire de la pensée politique.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J147" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K147" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">politique;ethique</t>
+        </is>
+      </c>
+      <c r="L147" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M147" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">roi de Babylone, auteur du célèbre code de lois, réflexion sur la justice et l'ordre social.</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P147">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148" ht="15" customHeight="1" s="25">
+      <c r="A148" s="23">
+        <v>-1370</v>
+      </c>
+      <c r="B148" s="23">
+        <v>-1337</v>
+      </c>
+      <c r="C148" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1370 A JC - 1337 A JC</t>
+        </is>
+      </c>
+      <c r="D148" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AKHENATON</t>
+        </is>
+      </c>
+      <c r="E148" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Akhenaton"  title=" Wikipedia"&gt;AKHENATON&lt;/a&gt;, d'abord nommé Amenhotep IV, fut pharaon d'Égypte de 1355 à 1337 avant J.-C. environ. Époux de Néfertiti et sans doute père de Toutânkhamon, il bouleversa la religion égyptienne en imposant le culte exclusif d'Aton, le disque solaire.&lt;/p&gt; &lt;p&gt;Il fit fermer les temples des autres dieux, fonda une nouvelle capitale, Akhetaton (Amarna), et composa ou inspira le &lt;em&gt;Grand Hymne à Aton&lt;/em&gt;, qui célèbre un dieu unique, créateur bienveillant de tous les êtres et de tous les peuples. On y voit souvent le premier monothéisme exclusif connu de l'histoire.&lt;/p&gt; &lt;p&gt;La révolution d'Akhenaton ne fut pas seulement religieuse. L'art de son règne, dit « amarnien », rompt avec les conventions séculaires : le roi est représenté avec un visage allongé et un corps aux formes étranges, dans des scènes de vie familiale intimes, entouré de Néfertiti et de leurs filles, sous les rayons du disque solaire terminés par des mains qui tendent la vie.&lt;/p&gt; &lt;p&gt;Le Grand Hymne à Aton, gravé dans une tombe d'Amarna, célèbre la lumière qui fait vivre toute la création : les hommes, les animaux, les plantes et même les pays étrangers, dont le dieu a fait les langues différentes. Certains passages présentent de fortes ressemblances avec le psaume 104 de la Bible. Freud, dans &lt;em&gt;Moïse et le monothéisme&lt;/em&gt;, alla jusqu'à supposer un lien entre la réforme d'Akhenaton et la religion de Moïse, hypothèse très discutée.&lt;/p&gt; &lt;p&gt;Sa réforme fut effacée après sa mort, mais elle pose une question philosophique durable : celle d'un principe unique à l'origine du monde, et du lien entre la vérité religieuse et le pouvoir politique.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J148" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K148" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite;metaphysique</t>
+        </is>
+      </c>
+      <c r="L148" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monothéisme</t>
+        </is>
+      </c>
+      <c r="M148" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pharaon égyptien qui imposa le culte du dieu unique Aton, parfois vu comme le premier monothéisme.</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P148">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149" ht="15" customHeight="1" s="25">
+      <c r="A149" s="23">
+        <v>-1300</v>
+      </c>
+      <c r="B149" s="23">
+        <v>-1100</v>
+      </c>
+      <c r="C149" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1300 A JC - 1100 A JC</t>
+        </is>
+      </c>
+      <c r="D149" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUDLUL bel nemeqi</t>
+        </is>
+      </c>
+      <c r="E149" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://fr.wikipedia.org/wiki/Ludlul_bēl_nēmeqi"  title=" Wikipedia"&gt;LUDLUL bel nemeqi&lt;/a&gt;, ou &lt;em&gt;Poème du juste souffrant&lt;/em&gt;, est un texte babylonien de la seconde moitié du IIe millénaire avant J.-C. Son titre signifie « Je veux louer le Seigneur de la sagesse », c'est-à-dire le dieu Marduk.&lt;/p&gt; &lt;p&gt;Un homme pieux, Shubshi-meshre-Shakkan, raconte comment il a tout perdu : son rang, ses amis, sa santé, alors qu'il avait toujours honoré les dieux. Il s'interroge : les hommes peuvent-ils comprendre la volonté divine, quand ce qui leur semble bon déplaît aux dieux ? Finalement, Marduk le rétablit dans sa prospérité.&lt;/p&gt; &lt;p&gt;Le poème compte environ cinq cents vers répartis sur quatre tablettes. Sa description de la maladie est d'un réalisme saisissant : le juste souffrant perd le sommeil, l'appétit et la vue, ses membres se paralysent, ses proches l'abandonnent et ses ennemis se réjouissent. Les devins et les exorcistes ne trouvent aucune explication à son malheur, car il n'a commis aucune faute rituelle.&lt;/p&gt; &lt;p&gt;La guérison survient à la suite de rêves où apparaissent des envoyés de Marduk, qui purifient le malade et chassent les démons. Le poème se termine par une célébration de la puissance du dieu, capable de frapper comme de guérir. La leçon n'est pas que la souffrance a une raison compréhensible, mais que les voies divines dépassent la raison humaine et que l'homme doit garder confiance malgré tout.&lt;/p&gt; &lt;p&gt;Ce poème pose, bien avant le livre biblique de Job, la grande question de la souffrance de l'innocent et de la justice divine, un problème que la philosophie appellera plus tard la théodicée.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J149" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K149" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;spiritualite</t>
+        </is>
+      </c>
+      <c r="L149" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M149" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poème babylonien du « juste souffrant », méditation sur le mal et la justice divine.</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="15" customHeight="1" s="25">
+      <c r="A150" s="23">
+        <v>-1200</v>
+      </c>
+      <c r="B150" s="23">
+        <v>-1100</v>
+      </c>
+      <c r="C150" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1200 A JC</t>
+        </is>
+      </c>
+      <c r="D150" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMENEMOPET</t>
+        </is>
+      </c>
+      <c r="E150" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Enseignement_d'Aménémopé"  title=" Wikipedia"&gt;AMENEMOPET&lt;/a&gt;, fils de Kanakht, était un scribe égyptien de l'époque ramesside (vers 1300-1075 avant J.-C.). Il composa pour son fils un &lt;em&gt;Enseignement&lt;/em&gt; en trente chapitres, l'un des plus beaux textes de sagesse de l'Égypte ancienne.&lt;/p&gt; &lt;p&gt;Il y oppose l'homme « silencieux », calme, honnête et maître de lui, à l'homme « emporté », colérique et avide. Il recommande de ne pas déplacer les bornes des champs, de ne pas se moquer des faibles, de ne pas s'enrichir par la fraude, et rappelle que l'homme ne connaît pas l'avenir : « l'homme est argile et paille, le dieu est son bâtisseur ».&lt;/p&gt; &lt;p&gt;L'enseignement est connu principalement par un papyrus conservé au British Museum, et par de nombreux fragments sur des tablettes d'écoliers, signe qu'il servait à la formation des scribes. Il se distingue des enseignements plus anciens par la place qu'il accorde à la vie intérieure : la vraie valeur de l'homme ne réside pas dans sa réussite sociale mais dans son calme, sa droiture et sa confiance en la divinité.&lt;/p&gt; &lt;p&gt;Le rapprochement avec la Bible est particulièrement frappant pour un passage des Proverbes (22,17 à 24,22), qui reprend souvent de très près les conseils d'Amenemopet, jusqu'à la mention de « trente » sentences. Cette parenté montre que les sages d'Israël connaissaient la littérature de sagesse égyptienne et s'en inspiraient, en l'adaptant à leur propre foi.&lt;/p&gt; &lt;p&gt;Plusieurs passages ont été rapprochés du livre biblique des Proverbes, ce qui montre la circulation des idées de sagesse dans tout le Proche-Orient ancien.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J150" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K150" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique</t>
+        </is>
+      </c>
+      <c r="L150" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M150" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scribe égyptien, auteur d'un enseignement de sagesse proche du livre biblique des Proverbes.</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15" customHeight="1" s="25">
+      <c r="A151" s="23">
+        <v>-1200</v>
+      </c>
+      <c r="B151" s="23">
+        <v>-1150</v>
+      </c>
+      <c r="C151" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1200 A JC (?)</t>
+        </is>
+      </c>
+      <c r="D151" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SANCHONIATHON</t>
+        </is>
+      </c>
+      <c r="E151" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sanchoniathon"  title=" Wikipedia"&gt;SANCHONIATHON&lt;/a&gt; est un auteur phénicien dont l'&lt;em&gt;Histoire phénicienne&lt;/em&gt; ne nous est connue que par les extraits traduits en grec par Philon de Byblos (Ier-IIe siècle), puis cités par Eusèbe de Césarée. Selon la tradition, il aurait vécu avant la guerre de Troie ; d'autres le placent bien plus tard, et son existence même est discutée.&lt;/p&gt; &lt;p&gt;Ces fragments constituent la principale source écrite sur la religion phénicienne. Ils proposent une cosmogonie, un récit de l'origine du monde à partir d'un chaos primitif et d'un souffle, puis l'apparition des dieux et des inventions humaines.&lt;/p&gt; &lt;p&gt;Selon Philon de Byblos, Sanchoniathon aurait rédigé son œuvre à partir d'archives conservées dans les temples et d'inscriptions sacrées. Son récit commence par un air sombre et venteux et un chaos trouble, d'où naît, par le désir du souffle pour ses propres principes, une matière originelle appelée &lt;em&gt;Môt&lt;/em&gt;, source de toutes les créatures. Viennent ensuite des générations de dieux et de héros civilisateurs qui inventent le feu, la pêche, la navigation ou l'écriture.&lt;/p&gt; &lt;p&gt;Longtemps, les savants ont douté de l'authenticité de ces fragments, qu'ils attribuaient à l'imagination de Philon. Mais la découverte, au XXe siècle, des textes mythologiques d'Ougarit, cité de la côte syrienne, a montré que plusieurs de ses récits correspondaient à d'authentiques traditions cananéennes, ce qui a redonné du crédit à Sanchoniathon.&lt;/p&gt; &lt;p&gt;Sanchoniathon témoigne de l'effort des anciens pour ordonner leurs mythes en une histoire du monde, et de la manière dont ces récits ont été relus par les philosophes grecs et chrétiens.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J151" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénicienne</t>
+        </is>
+      </c>
+      <c r="K151" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;spiritualite</t>
+        </is>
+      </c>
+      <c r="L151" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Polythéisme</t>
+        </is>
+      </c>
+      <c r="M151" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auteur phénicien d'une histoire des origines du monde et des dieux, connue par Philon de Byblos.</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="15" customHeight="1" s="25">
+      <c r="A152" s="23">
+        <v>-1000</v>
+      </c>
+      <c r="B152" s="23">
+        <v>-930</v>
+      </c>
+      <c r="C152" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1000 A JC</t>
+        </is>
+      </c>
+      <c r="D152" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZARATHOUSTRA</t>
+        </is>
+      </c>
+      <c r="E152" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Zarathoustra"  title=" Wikipedia"&gt;ZARATHOUSTRA&lt;/a&gt;, ou Zoroastre, est le prophète fondateur du zoroastrisme, la religion de l'Iran ancien. Ses dates sont très discutées : l'analyse de la langue des &lt;em&gt;Gathas&lt;/em&gt;, les hymnes qui lui sont attribués, conduit aujourd'hui la plupart des spécialistes à le situer vers l'an 1000 avant J.-C.&lt;/p&gt; &lt;p&gt;Sa pensée repose sur l'opposition entre deux principes : l'esprit du bien, lié à Ahura Mazda, le « Seigneur sage », et l'esprit du mal et du mensonge. Chaque être humain est libre de choisir son camp par ses pensées, ses paroles et ses actions, et sera jugé selon ce choix.&lt;/p&gt; &lt;p&gt;Selon la tradition, Zarathoustra reçut sa révélation vers l'âge de trente ans, lors d'une vision au bord d'une rivière. Il dut affronter l'hostilité des prêtres de l'ancienne religion avant de trouver un protecteur, le roi Vishtaspa, qui se convertit à son enseignement. Ses &lt;em&gt;Gathas&lt;/em&gt;, dix-sept hymnes écrits dans une langue très archaïque, forment la partie la plus ancienne de l'Avesta, le livre sacré du zoroastrisme.&lt;/p&gt; &lt;p&gt;Le zoroastrisme devint plus tard la religion des grands empires perses, des Achéménides aux Sassanides, jusqu'à la conquête arabe au VIIe siècle. Il survit aujourd'hui dans de petites communautés en Iran et chez les Parsis de l'Inde. Le feu, symbole de la vérité et de la pureté, y occupe une place centrale, ce qui a valu aux zoroastriens le nom, inexact, d'« adorateurs du feu ».&lt;/p&gt; &lt;p&gt;Cette vision d'un combat cosmique entre le bien et le mal, de la responsabilité morale individuelle et d'un jugement final a profondément influencé le judaïsme, le christianisme et l'islam. Nietzsche a repris son nom dans &lt;em&gt;Ainsi parlait Zarathoustra&lt;/em&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J152" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perse</t>
+        </is>
+      </c>
+      <c r="K152" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spiritualite;ethique;metaphysique</t>
+        </is>
+      </c>
+      <c r="L152" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zoroastrisme</t>
+        </is>
+      </c>
+      <c r="M152" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prophète iranien, fondateur du zoroastrisme, penseur du combat entre le bien et le mal.</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P152">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="153" ht="15" customHeight="1" s="25">
+      <c r="A153" s="23">
+        <v>-1000</v>
+      </c>
+      <c r="B153" s="23">
+        <v>-900</v>
+      </c>
+      <c r="C153" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 1000 A JC</t>
+        </is>
+      </c>
+      <c r="D153" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dialogue du PESSIMISME</t>
+        </is>
+      </c>
+      <c r="E153" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://en.wikipedia.org/wiki/Dialogue_of_Pessimism"  title=" Wikipedia"&gt;Dialogue du PESSIMISME&lt;/a&gt; est un court texte akkadien composé peu après l'an 1000 avant J.-C. en Mésopotamie. Il met en scène un maître et son esclave.&lt;/p&gt; &lt;p&gt;Le maître annonce tour à tour qu'il va aller au palais, festoyer, aimer une femme, faire un sacrifice, prêter de l'argent ou servir son pays ; à chaque fois l'esclave l'approuve avec de bonnes raisons, puis, quand le maître change d'avis, l'approuve encore avec des raisons tout aussi bonnes. À la fin, le maître demande ce qui est bon : l'esclave répond qu'il vaut mieux mourir.&lt;/p&gt; &lt;p&gt;Chaque échange suit le même schéma : « Esclave, obéis-moi ! — Oui, mon maître, oui. » Le maître propose une action, l'esclave en vante les avantages ; le maître y renonce, l'esclave en montre aussitôt les dangers. Ainsi, faire l'amour à une femme fait oublier le chagrin, mais la femme est « un piège, un trou, un fossé » ; faire le bien de son pays est louable, mais personne ne distingue, parmi les crânes des morts, le bienfaiteur du malfaiteur.&lt;/p&gt; &lt;p&gt;Les spécialistes hésitent sur le sens du texte : satire comique du maître capricieux et de l'esclave flatteur, ou méditation sérieuse sur l'absence de valeur sûre ? Dans les deux cas, il met en évidence une idée troublante : pour chaque choix, on peut trouver des raisons aussi convaincantes que pour le choix contraire, de sorte que la raison seule ne permet pas de décider comment vivre.&lt;/p&gt; &lt;p&gt;Ironique ou désespéré, ce dialogue interroge la valeur de toute action humaine et annonce les grandes réflexions sceptiques et pessimistes, de Qohélet à Schopenhauer.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J153" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K153" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique;metaphysique</t>
+        </is>
+      </c>
+      <c r="L153" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M153" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dialogue babylonien entre un maître et son esclave sur la vanité de toute action humaine.</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="15" customHeight="1" s="25">
+      <c r="A154" s="23">
+        <v>-700</v>
+      </c>
+      <c r="B154" s="23">
+        <v>-640</v>
+      </c>
+      <c r="C154" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIIe siècle A JC</t>
+        </is>
+      </c>
+      <c r="D154" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AHIQAR</t>
+        </is>
+      </c>
+      <c r="E154" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar"  title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup concernent la parole : « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs connaissaient Ahiqar : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une diffusion aussi large à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J154" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K154" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique</t>
+        </is>
+      </c>
+      <c r="L154" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M154" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sage assyrien semi-légendaire, dont l'histoire et les maximes circulèrent dans tout le Proche-Orient.</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="15" customHeight="1" s="25">
+      <c r="A155" s="23">
+        <v>-550</v>
+      </c>
+      <c r="B155" s="23">
+        <v>-400</v>
+      </c>
+      <c r="C155" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIe - IVe siècle A JC</t>
+        </is>
+      </c>
+      <c r="D155" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Livre de JOB</t>
+        </is>
+      </c>
+      <c r="E155" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://fr.wikipedia.org/wiki/Livre_de_Job"  title=" Wikipedia"&gt;Livre de JOB&lt;/a&gt; est un livre de la Bible hébraïque rédigé entre le VIe et le début du IVe siècle avant J.-C. Il raconte l'histoire de Job, un homme juste et prospère que Dieu laisse éprouver par Satan : il perd ses biens, ses enfants et sa santé.&lt;/p&gt; &lt;p&gt;Ses amis soutiennent qu'il doit avoir péché pour souffrir ainsi ; Job refuse cette explication, proclame son innocence et demande des comptes à Dieu. Dieu lui répond enfin du milieu de la tempête, non par une justification, mais en lui montrant l'immensité et le mystère de la création.&lt;/p&gt; &lt;p&gt;Le livre est construit comme une œuvre littéraire complexe : un prologue et un épilogue en prose, où Job est un modèle de patience (« Le Seigneur a donné, le Seigneur a repris »), encadrent de longs discours poétiques où Job, au contraire, se révolte, maudit le jour de sa naissance et accuse Dieu d'injustice. Trois amis, Éliphaz, Bildad et Tsophar, puis un jeune homme, Élihou, tentent en vain de le convaincre qu'il est puni pour ses fautes.&lt;/p&gt; &lt;p&gt;Le livre refuse ainsi la doctrine de la rétribution, selon laquelle le bonheur récompense les justes et le malheur punit les méchants. Dieu donne finalement tort aux amis et raison à Job, qui a parlé avec franchise. La souffrance n'est pas expliquée : elle reste un mystère que l'homme doit affronter sans réponse, dans une relation directe et exigeante avec Dieu.&lt;/p&gt; &lt;p&gt;Ce chef-d'œuvre poétique pose avec une force inégalée la question de la souffrance de l'innocent et des limites de la raison humaine face au mal. Il a inspiré de nombreux philosophes, de Kierkegaard à Levinas.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J155" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Juive</t>
+        </is>
+      </c>
+      <c r="K155" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;spiritualite</t>
+        </is>
+      </c>
+      <c r="L155" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Herméneutique juive</t>
+        </is>
+      </c>
+      <c r="M155" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">livre biblique sur la souffrance du juste et le silence de Dieu.</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P155">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="156" ht="15" customHeight="1" s="25">
+      <c r="A156" s="23">
+        <v>-340</v>
+      </c>
+      <c r="B156" s="23">
+        <v>-270</v>
+      </c>
+      <c r="C156" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 340 A JC - 270 A JC</t>
+        </is>
+      </c>
+      <c r="D156" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BÉROSE</t>
+        </is>
+      </c>
+      <c r="E156" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bérose"  title=" Wikipedia"&gt;BÉROSE&lt;/a&gt; était un prêtre du dieu Bêl à Babylone, astronome et historien, né vers 340 avant J.-C. Il vécut après la conquête de la Mésopotamie par Alexandre le Grand, à l'époque des rois séleucides.&lt;/p&gt; &lt;p&gt;Il rédigea en grec, entre 290 et 279 avant J.-C., une &lt;em&gt;Histoire de Babylone&lt;/em&gt; (&lt;em&gt;Babyloniaca&lt;/em&gt;) dédiée au roi Antiochos Ier. Il y présentait aux Grecs le savoir babylonien : la création du monde, les rois d'avant le Déluge, le récit du Déluge lui-même et l'histoire des grands empires mésopotamiens.&lt;/p&gt; &lt;p&gt;L'œuvre de Bérose est perdue : nous n'en connaissons que des fragments cités par des auteurs plus tardifs, comme l'historien juif Flavius Josèphe ou l'évêque Eusèbe de Césarée. Elle était divisée en trois livres : le premier sur la géographie de la Babylonie et la création du monde, où apparaît le monstre marin Oannès, maître civilisateur qui enseigne aux hommes l'écriture, les lois et les arts ; les deux autres sur les rois et l'histoire jusqu'à Alexandre.&lt;/p&gt; &lt;p&gt;Selon la tradition, Bérose se serait ensuite installé sur l'île grecque de Cos, où il aurait fondé une école d'astrologie, et les Athéniens lui auraient élevé une statue en l'honneur de ses prédictions. Réelle ou légendaire, cette figure du prêtre babylonien enseignant les Grecs résume bien le rôle de passeur que lui attribue l'histoire.&lt;/p&gt; &lt;p&gt;Bérose est l'un des premiers passeurs entre deux mondes : il transmit à la culture grecque une partie de la sagesse et de l'astronomie chaldéennes, à la fin de la longue histoire de la pensée mésopotamienne.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J156" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamienne</t>
+        </is>
+      </c>
+      <c r="K156" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">epistemologie;spiritualite</t>
+        </is>
+      </c>
+      <c r="L156" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme</t>
+        </is>
+      </c>
+      <c r="M156" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prêtre et astronome babylonien qui fit connaître aux Grecs l'histoire et le savoir de Babylone.</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="15" customHeight="1" s="25">
+      <c r="A157" s="23">
+        <v>-250</v>
+      </c>
+      <c r="B157" s="23">
+        <v>-220</v>
+      </c>
+      <c r="C157" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vers 250 A JC</t>
+        </is>
+      </c>
+      <c r="D157" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QOHÉLET (l’Ecclésiaste)</t>
+        </is>
+      </c>
+      <c r="E157" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ecclésiaste"  title=" Wikipedia"&gt;QOHÉLET&lt;/a&gt;, ou l'&lt;em&gt;Ecclésiaste&lt;/em&gt;, est un livre de sagesse de la Bible hébraïque écrit vers 250 avant J.-C., à Jérusalem, à l'époque du Second Temple. Son auteur se présente comme « Qohélet », un fils de David, roi à Jérusalem.&lt;/p&gt; &lt;p&gt;Il s'ouvre sur une formule restée célèbre : « Vanité des vanités, tout est vanité ». Qohélet observe que la richesse, le travail, le plaisir et même la sagesse ne mettent pas l'homme à l'abri de la mort, qui frappe le sage comme l'insensé ; « rien de nouveau sous le soleil » et « il y a un temps pour tout ».&lt;/p&gt; &lt;p&gt;Le mot hébreu traduit par « vanité », &lt;em&gt;hèvèl&lt;/em&gt;, signifie d'abord « buée » ou « souffle » : ce qui est léger, insaisissable et passager. Qohélet l'applique à tout ce que l'homme entreprend sous le soleil. Il observe aussi l'injustice du monde : le juste peut périr dans sa justice et le méchant prolonger sa vie dans sa méchanceté, et l'homme ne peut pas comprendre l'œuvre de Dieu du début à la fin.&lt;/p&gt; &lt;p&gt;La tradition a attribué le livre au roi Salomon, ce qui a sans doute facilité son entrée dans la Bible malgré ses idées audacieuses. Son ton désabusé a souvent été rapproché de la philosophie grecque, du scepticisme et de l'épicurisme, sans qu'une influence directe soit certaine. Montaigne, Pascal ou Camus y ont trouvé un écho à leur propre réflexion sur la condition humaine.&lt;/p&gt; &lt;p&gt;Plutôt que de désespérer, il invite à profiter avec simplicité des joies de la vie, du pain et du vin, fruits du travail, comme d'un don de Dieu. Par son regard lucide et presque sceptique, Qohélet est l'un des textes les plus philosophiques de la Bible.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J157" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Juive</t>
+        </is>
+      </c>
+      <c r="K157" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;ethique</t>
+        </is>
+      </c>
+      <c r="L157" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Herméneutique juive</t>
+        </is>
+      </c>
+      <c r="M157" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">livre de sagesse biblique, méditation lucide sur la vanité et le sens de la vie.</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="P157">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158" ht="15" customHeight="1" s="25">
+      <c r="A158" s="23">
+        <v>-250</v>
+      </c>
+      <c r="B158" s="23">
+        <v>-100</v>
+      </c>
+      <c r="C158" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IIIe - Ier siècle A JC</t>
+        </is>
+      </c>
+      <c r="D158" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ÂNKHSHESHONQY</t>
+        </is>
+      </c>
+      <c r="E158" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;L'&lt;a href="https://en.wikipedia.org/wiki/Instruction_of_Ankhsheshonq"  title=" Wikipedia"&gt;Enseignement d’ÂNKHSHESHONQY&lt;/a&gt; est un texte égyptien rédigé en démotique, daté de l'époque ptolémaïque (après 305 avant J.-C.), mais dont le contenu est peut-être plus ancien.&lt;/p&gt; &lt;p&gt;Un récit raconte qu'Ânkhsheshonqy, prêtre d'Héliopolis, fut jeté en prison pour n'avoir pas dénoncé un complot contre le pharaon ; ne pouvant plus éduquer son fils, il écrivit pour lui ses conseils sur des tessons de poterie. Suit une longue série de maximes brèves, souvent ironiques et pleines de bon sens, sur le travail, la famille, l'amitié, la prudence et les revers de la fortune.&lt;/p&gt; &lt;p&gt;Les maximes sont écrites sur un seul papyrus conservé au British Museum. Elles se succèdent sans ordre apparent, une par ligne, dans un style direct et imagé : « Ne dis pas : c'est l'été, il y a l'hiver aussi », « Celui qui envoie des épines récoltera des épines », « Ne fais pas confiance au feu tant qu'il brûle », ou encore « La femme sage ne quitte pas sa maison ». On y trouve aussi une réflexion sur la fortune et le destin, qui peuvent frapper chacun sans prévenir.&lt;/p&gt; &lt;p&gt;Le récit qui les introduit, avec son pharaon trompé, son complot et son sage emprisonné, rappelle l'histoire d'Ahiqar, ce qui montre les échanges entre les traditions égyptienne et araméenne. Contrairement aux enseignements anciens destinés aux fonctionnaires, celui d'Ânkhsheshonqy s'adresse à tous, paysans, artisans ou marchands : c'est une sagesse populaire, tournée vers la vie de tous les jours.&lt;/p&gt; &lt;p&gt;Ce texte, l'un des derniers grands enseignements égyptiens, montre la vitalité d'une sagesse pratique qui a traversé trois millénaires d'histoire.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J158" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Égyptienne</t>
+        </is>
+      </c>
+      <c r="K158" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ethique</t>
+        </is>
+      </c>
+      <c r="L158" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egypte antique</t>
+        </is>
+      </c>
+      <c r="M158" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prêtre égyptien d'époque ptolémaïque, auteur d'un recueil de maximes écrit en prison pour son fils.</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="15" customHeight="1" s="25">
+      <c r="A159" s="23">
+        <v>154</v>
+      </c>
+      <c r="B159" s="23">
+        <v>222</v>
+      </c>
+      <c r="C159" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">154 - 222</t>
+        </is>
+      </c>
+      <c r="D159" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BARDESANE</t>
+        </is>
+      </c>
+      <c r="E159" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bardesane"  title=" Wikipedia"&gt;BARDESANE&lt;/a&gt; (154-222) est un philosophe, poète et astronome né à Édesse, en Mésopotamie du Nord (aujourd'hui Şanlıurfa, en Turquie). Il fut l'un des premiers grands auteurs de langue syriaque et un proche de la cour du roi Abgar VIII.&lt;/p&gt; &lt;p&gt;Son œuvre principale, le &lt;em&gt;Livre des lois des pays&lt;/em&gt;, retrouvé en 1845, est un dialogue sur le destin et la liberté. Bardesane y combat l'idée que les astres déterminent entièrement la vie humaine : il montre que les peuples, soumis aux mêmes astres, ont des lois et des mœurs très différentes, preuve que l'homme reste libre de ses choix.&lt;/p&gt; &lt;p&gt;Le &lt;em&gt;Livre des lois des pays&lt;/em&gt; fut en réalité rédigé par un disciple, Philippe, qui rapporte la conversation de son maître avec un certain Awida. Bardesane y distingue trois niveaux dans l'existence humaine : la nature, commune à tous et qui règle la naissance, la croissance et la mort ; le destin, lié aux astres, qui explique la richesse, la maladie ou les accidents ; et la liberté, qui dépend de l'homme seul et fait de lui un être moral, responsable de ses actes.&lt;/p&gt; &lt;p&gt;Bardesane composa aussi des hymnes en syriaque, si populaires que saint Éphrem, un siècle plus tard, écrivit ses propres hymnes sur les mêmes mélodies pour combattre les idées de Bardesane. Son fils Harmonios poursuivit son œuvre poétique. Bardesane occupe ainsi une place importante dans les débuts de la littérature syriaque, qui sera plus tard un pont entre la philosophie grecque et le monde arabe.&lt;/p&gt; &lt;p&gt;Chrétien aux idées originales, marquées par l'astrologie et des influences gnostiques, il fut ensuite jugé hérétique. Il reste un témoin de la rencontre entre la sagesse orientale, la philosophie grecque et le christianisme naissant.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J159" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Syrienne</t>
+        </is>
+      </c>
+      <c r="K159" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique;ethique</t>
+        </is>
+      </c>
+      <c r="L159" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gnosticisme</t>
+        </is>
+      </c>
+      <c r="M159" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe syriaque d'Édesse, penseur du destin et de la liberté humaine.</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="1048572" ht="12.75" customHeight="1" s="25"/>
     <row r="1048573" ht="12.75" customHeight="1" s="25"/>

</xml_diff>

<commit_message>
Ipou-Our : identifiant de la vidéo et crédit corrigés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -315,10 +315,10 @@
     <t xml:space="preserve">&lt;p&gt;Les &lt;a href="https://fr.wikipedia.org/wiki/Papyrus_d%27Ipou-Our"  title=" Wikipedia"&gt;Lamentations d’IPOU-OUR&lt;/a&gt; sont un texte égyptien composé au plus tôt à la fin de la XIIe dynastie. Le sage Ipou-our s'y adresse au roi pour lui décrire un pays sens dessus dessous : les pauvres sont devenus riches, les nobles sont dans la misère, les lois ne sont plus respectées et le Nil lui-même semble ensanglanté.&lt;/p&gt; &lt;p&gt;Ce tableau d'un monde en chaos est moins une chronique historique qu'une réflexion sur ce qui arrive quand l'ordre juste, la Maât, n'est plus garanti. Il reproche même au dieu créateur de laisser faire le mal, et appelle un pouvoir fort à rétablir l'harmonie.&lt;/p&gt; &lt;p&gt;Le texte nous est parvenu sur un seul papyrus, conservé aujourd'hui au musée de Leyde, aux Pays-Bas, dont le début et la fin manquent. Il se compose de longues séries de lamentations commençant par le même refrain, « En vérité… », qui décrivent tour à tour la violence, la famine, le pillage des tombes, la fuite des serviteurs et l'effondrement de l'administration.&lt;/p&gt; &lt;p&gt;Certains y ont vu le témoignage d'une révolution sociale réelle, d'autres un écho des plaies d'Égypte du livre de l'Exode ; les égyptologues y lisent plutôt un genre littéraire, celui   &lt;a href="https://www.worldhistory.org/trans/fr/2-981/lamentations-dipou-our/"   title="lamentations d’Ipou-Our par worldhistory"&gt;des « lamentations »,&lt;/a&gt;  qui montre l'image inversée de l'ordre idéal pour mieux en faire sentir la valeur. Le désordre décrit n'est pas seulement politique : c'est tout l'équilibre entre les hommes, la nature et les dieux qui semble rompu.&lt;/p&gt; &lt;p&gt;Le texte pose ainsi, très tôt, la question du mal et de la responsabilité des dirigeants et des dieux face au désordre du monde.&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">VL-OWz8Awm0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Ipuwer Payrus par Evidence 4 faith</t>
+    <t xml:space="preserve">vL-OWz8Awm0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Ipuwer Papyrus par Evidence 4 faith</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.laphilo.fr/pho/iour-mini.webp</t>

</xml_diff>

<commit_message>
1er test formulaire - Laroui
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -12756,14 +12756,33 @@
       <c r="D154" s="2" t="s">
         <v>1288</v>
       </c>
-      <c r="E154" s="10" t="s">
-        <v>1289</v>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://fr.wikipedia.org/wiki/Dialogue_du_pessimisme" title=" Wikipedia"&gt;Dialogue du PESSIMISME&lt;/a&gt; est un court texte akkadien composé en Mésopotamie qui met en scène un maître et son esclave.&lt;/p&gt; &lt;p&gt;Le maître &lt;a href="http://www.aroumah.net/seminar/Dialogue%20of%20Pessimism.pdf"&gt;annonce tour à tour &lt;/a&gt;qu'il va aller au palais, festoyer, aimer une femme, faire un sacrifice, prêter de l'argent ou servir son pays ; à chaque fois l'esclave l'approuve avec de bonnes raisons, puis, quand le maître change d'avis, l'approuve encore avec des raisons tout aussi bonnes. À la fin, le maître demande ce qui est bon : l'esclave répond qu'il vaut mieux mourir.&lt;/p&gt; &lt;p&gt;Chaque échange suit le même schéma : « Esclave, obéis-moi ! — Oui, mon maître, oui. » Le maître propose une action, l'esclave en vante les avantages ; le maître y renonce, l'esclave en montre aussitôt les dangers. Ainsi, faire l'amour à une femme fait oublier le chagrin, mais la femme est « un piège, un trou, un fossé » ; faire le bien de son pays est louable, mais personne ne distingue, parmi les crânes des morts, le bienfaiteur du malfaiteur.&lt;/p&gt; &lt;p&gt;Les spécialistes hésitent sur le sens du texte : satire comique du maître capricieux et de l'esclave flatteur, ou méditation sérieuse sur l'absence de valeur sûre ? Dans les deux cas, il met en évidence une idée troublante : pour chaque choix, on peut trouver des raisons aussi convaincantes que pour le choix contraire, de sorte que la raison seule ne permet pas de décider comment vivre.&lt;/p&gt; &lt;p&gt;Ironique ou désespéré, ce dialogue interroge la valeur de toute action humaine et annonce les grandes réflexions sceptiques et pessimistes, de Qohélet à Schopenhauer.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0aawol43UdU</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The Dialogue of Pessimism (Full Audiobook)" par abitof_ane_rd</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/dialoguedupessimisme-mini.webp</t>
+        </is>
       </c>
       <c r="J154" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K154" s="2" t="s">
-        <v>1290</v>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique</t>
+        </is>
       </c>
       <c r="L154" s="2" t="s">
         <v>53</v>
@@ -12788,8 +12807,25 @@
       <c r="D155" s="2" t="s">
         <v>1293</v>
       </c>
-      <c r="E155" s="10" t="s">
-        <v>1294</v>
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar" title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup&lt;a href="https://www.persee.fr/doc/ethio_0066-2127_1978_num_11_1_912" title="L'histoire d'Ahiqar en éthiopien par persée"&gt; concernent la parole &lt;/a&gt;: « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs le connaissaient : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une &lt;a href="https://www.youtube.com/watch?v=3HCHSrvEwuc" title="Sage Ahiqar Quotes Ancient Assyrian Wisdom par mir allround"&gt;diffusion aussi large &lt;/a&gt;à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AX9Hmh5qJ9U</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The Story of Ahikar" par Study of Antiquity and the Middle Ages</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ahiqar-mini.webp</t>
+        </is>
       </c>
       <c r="J155" s="1" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Textes enrichis (~1 600 car.) : Jaimini, Kapila, Yajnavalkya, Brihaspati, Buddhaghosa, Kanada, Makkhali Gosala ; portrait Khatibi ; éditeur : longueur des textes, filtres, colonne élargissable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -7256,8 +7256,10 @@
       <c r="D25" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>202</v>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Y%C4%81j%C3%B1avalkya" title=" Wikipedia"&gt;Yâjñavalkya&lt;/a&gt; est l’un des grands sages (&lt;em&gt;ṛṣi&lt;/em&gt;) des Upanishads, figure centrale de la &lt;a href="https://fr.wikipedia.org/wiki/Brihadaranyaka_Upanishad" title=" Wikipedia"&gt;&lt;em&gt;Brihadâranyaka Upanishad&lt;/em&gt;&lt;/a&gt;. La tradition lui attribue aussi la révélation du Yajur-Véda « blanc », le &lt;em&gt;Shatapatha Brâhmana&lt;/em&gt; et, bien plus tardivement, un célèbre traité de droit. Dans l’Upanishad, il développe une réflexion fondatrice sur l’identité entre le Soi individuel (&lt;em&gt;ātman&lt;/em&gt;) et le principe universel (&lt;em&gt;brahman&lt;/em&gt;), posant les bases philosophiques du brahmanisme et, plus tard, du Vedânta.&lt;/p&gt; &lt;p&gt;L’Upanishad le montre à la cour du roi Janaka de Videha, où il remporte un grand tournoi de questions contre les brahmanes les plus savants, dont la philosophe Gârgî. Celle-ci l’interroge sur la trame de l’univers : tout est tissé sur l’espace, répond-il, et l’espace lui-même sur l’Impérissable (&lt;em&gt;akṣara&lt;/em&gt;), sous le commandement duquel se tiennent le soleil et la lune. Il y enseigne que le Soi ne peut être saisi comme un objet : « On ne peut voir le voyant de la vue, ni entendre l’entendeur de l’audition. » On ne peut le décrire que négativement : « Il n’est ni ceci, ni cela » (&lt;em&gt;neti neti&lt;/em&gt;). Insaisissable, il échappe au changement, à la souffrance et à la mort.&lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=tdfdWUqQrwE"  title="a masterpiece of indian philosophy par BharatVerse"&gt; Ses dialogues, &lt;/a&gt; notamment avec son épouse &lt;a href="https://fr.wikipedia.org/wiki/Maitreyi" title=" Wikipedia"&gt;Maitreyî&lt;/a&gt; sur la nature du désir et de la connaissance, comptent parmi les textes fondateurs de la métaphysique indienne. Sur le point de partir pour la vie d’ascète, il veut partager ses biens entre ses deux épouses ; Maitreyî lui demande si la richesse rend immortel, et il lui répond : « Ce n’est pas pour l’amour de l’époux que l’époux est cher, mais pour l’amour du Soi. » Ce passage a nourri toute la tradition du Vedânta.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F25" s="1" t="s">
         <v>203</v>
@@ -7384,8 +7386,10 @@
       <c r="D28" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>227</v>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Kanada" title=" Wikipedia"&gt;Kanada&lt;/a&gt; (ou Kaṇāda) est le fondateur traditionnel de l’école Vaisheshika, l’une des six écoles orthodoxes de la philosophie indienne. Son nom signifie « mangeur de grains » : la légende raconte qu’il vivait des grains glanés dans les champs, mais on y voit aussi une allusion aux particules infimes au cœur de sa doctrine.&lt;/p&gt; &lt;p&gt;Auteur des &lt;em&gt;Vaisheshika-sûtras&lt;/em&gt;, il développe une physique atomiste : la réalité est composée de substances élémentaires indivisibles (&lt;em&gt;paramāṇu&lt;/em&gt;) combinées selon des catégories logiques précises. Les atomes de terre, d’eau, de feu et d’air sont éternels et invisibles ; ils s’unissent par deux, puis par trois, pour former les corps perceptibles. À ces quatre éléments s’ajoutent l’éther, le temps, l’espace, l’âme et le mental, soit neuf substances. Le réel se répartit en six catégories : la substance, la qualité, l’action, le général, le particulier et l’inhérence. C’est la « particularité » (&lt;em&gt;viśeṣa&lt;/em&gt;), qui distingue chaque atome et chaque âme, qui a donné son nom à l’école. On compare souvent cet &lt;a href="https://fr.wikipedia.org/wiki/Atomisme" title=" Wikipedia"&gt;atomisme&lt;/a&gt; à celui de Démocrite, mais ses atomes diffèrent par leurs qualités et sont mis en mouvement par une force invisible, liée aux actes des êtres.&lt;/p&gt; &lt;p&gt;Les sûtras s’ouvrent sur le &lt;em&gt;dharma&lt;/em&gt;, « ce qui procure la prospérité et le bien suprême » : connaître exactement les catégories du réel conduit à la délivrance. Cette approche fait du &lt;a href="https://www.youtube.com/watch?v=WDTGhajiZyo"  title="sage Kanada Vaisesika par Maynka Vadya"&gt; Vaisheshika &lt;/a&gt; l’une des premières tentatives systématiques de philosophie de la nature en Inde, plus tard fusionnée avec le &lt;a href="https://fr.wikipedia.org/wiki/Ny%C3%A2ya" title=" Wikipedia"&gt;Nyâya&lt;/a&gt;. Ses commentateurs, à commencer par Prashastapada vers le VIe siècle, systématisèrent la doctrine, et les auteurs ultérieurs ajoutèrent une septième catégorie : la non-existence.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F28" s="1" t="s">
         <v>228</v>
@@ -7425,8 +7429,10 @@
       <c r="D29" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>236</v>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Kapila" title=" Wikipedia"&gt;Kapila&lt;/a&gt; est le sage fondateur traditionnel du Sâmkhya, l’une des plus anciennes écoles de philosophie indienne. Sa figure appartient à la légende : la &lt;em&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bhagavad-G%C4%ABt%C4%81" title=" Wikipedia"&gt;Bhagavad-Gîtâ&lt;/a&gt;&lt;/em&gt; le nomme parmi les sages accomplis, et les Purânas en font une incarnation de Vishnou enseignant la délivrance à sa mère. Aucun de ses écrits ne nous est parvenu ; le plus ancien exposé conservé de la doctrine, les &lt;em&gt;Sâmkhya-kârikâ&lt;/em&gt; d’Îshvarakrishna, date des premiers siècles de notre ère.&lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=PcOxBi1VRL4"  title="kapila and sankhya par foolish musings"&gt;Le Sâmkhya &lt;/a&gt; propose un dualisme radical entre la conscience pure (&lt;em&gt;puruṣa&lt;/em&gt;) et la matière primordiale (&lt;em&gt;prakṛti&lt;/em&gt;), dont l’évolution engendre l’ensemble du monde phénoménal. La matière est faite de trois qualités (&lt;em&gt;guṇa&lt;/em&gt;) : la clarté, l’énergie et l’inertie ; de leur déséquilibre naissent successivement l’intellect, le sens du moi, le mental, les sens et les éléments, soit vingt-cinq principes en tout : le mot &lt;em&gt;sâmkhya&lt;/em&gt; signifie d’ailleurs « dénombrement ». L’effet préexiste dans sa cause, comme l’huile dans la graine de sésame. Ce dualisme de l’âme et de la matière rappelle celui du &lt;a href="https://www.youtube.com/watch?v=Q0AR1mxTME4&amp;t=106s&amp;ab_channel=Ja%C3%AFnisme-Uneintroduction"  title="Jaïnisme Introduction par Jaïnisme Université de Gent "&gt;jaïnisme &lt;/a&gt;, qui distingue lui aussi les âmes de la matière inerte.&lt;/p&gt; &lt;p&gt;La souffrance vient de ce que la conscience se confond avec les activités de la matière ; la délivrance (&lt;em&gt;kaivalya&lt;/em&gt;) est leur discernement, l’« isolement » de la conscience, spectatrice immobile. Contrairement au Vedânta, le Sâmkhya admet une infinité de consciences distinctes, une pour chaque être. Les &lt;em&gt;Sâmkhya-kârikâ&lt;/em&gt; comparent la matière à une danseuse qui se retire une fois qu’elle s’est montrée au spectateur. Cette cosmologie, indépendante de toute divinité créatrice, a profondément marqué l’hindouisme classique et sert de socle théorique aux &lt;a href="https://fr.wikipedia.org/wiki/Yoga_s%C5%ABtra" title=" Wikipedia"&gt;&lt;em&gt;Yoga-sûtras&lt;/em&gt; de Patañjali&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F29" s="1" t="s">
         <v>237</v>
@@ -7466,8 +7472,10 @@
       <c r="D30" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>243</v>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Brihaspati" title=" Wikipedia"&gt;Brihaspati&lt;/a&gt; est le sage auquel la tradition attribue  &lt;a href="https://www.wisdomlib.org/fr/concept/brihaspati"  title="Brihaspati par wisdom library"&gt;la fondation du Lokâyata&lt;/a&gt;  (ou &lt;a href="https://fr.wikipedia.org/wiki/Ch%C3%A2rv%C3%A2ka" title=" Wikipedia"&gt;Cârvâka&lt;/a&gt;), école matérialiste et athée de la philosophie indienne. Le nom est aussi celui du précepteur des dieux, et un récit des Purânas prétend qu’il aurait enseigné le matérialisme aux démons pour les égarer. Ses &lt;em&gt;Bârhaspatya-sûtras&lt;/em&gt; sont perdus : la doctrine n’est connue que par les citations de ses adversaires, notamment le &lt;em&gt;Sarva-darshana-samgraha&lt;/em&gt; de Mâdhava, au XIVe siècle.&lt;/p&gt; &lt;p&gt;Rejetant l’autorité des Védas, la réincarnation et toute réalité suprasensible, ce courant ne reconnaît comme source de connaissance valide que la perception directe. L’inférence est incertaine, car on ne peut jamais avoir observé tous les cas : une critique qui annonce le problème de l’induction. Le monde est fait de quatre éléments, terre, eau, feu et air, et la conscience naît de leur combinaison dans le corps, comme le pouvoir enivrant naît du mélange de certains ingrédients. Il n’y a donc pas d’âme qui survive à la mort, et le bonheur comme le malheur s’expliquent par la nature des choses, sans qu’il soit besoin d’invoquer le karma.&lt;/p&gt; &lt;p&gt;Le Lokâyata prône une éthique hédoniste centrée sur le plaisir dans cette vie : « Tant que tu vis, vis heureux ; une fois le corps réduit en cendres, comment reviendrait-il ? » Il raille les prêtres, qui vivraient des rites qu’ils prescrivent : si la victime sacrifiée monte au ciel, pourquoi le sacrifiant n’y envoie-t-il pas son propre père ? Et si les offrandes nourrissent les morts, pourquoi les voyageurs emportent-ils des provisions ? Le Lokâyata demeure la voix la plus radicalement sceptique de la pensée indienne classique.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F30" s="1" t="s">
         <v>244</v>
@@ -7771,8 +7779,10 @@
       <c r="D37" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>309</v>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ajivika" title=" Wikipedia"&gt;Makkhali Gosala&lt;/a&gt; est le principal fondateur de l’Ajîvika, courant hétérodoxe (&lt;em&gt;nâstika&lt;/em&gt;) contemporain du Bouddha et de &lt;a href="https://fr.wikipedia.org/wiki/Mah%C4%81v%C4%ABra" title=" Wikipedia"&gt;Mahâvîra&lt;/a&gt;. Ses écrits sont perdus, et on ne le connaît que par les textes de ses rivaux bouddhistes et jaïns, peu bienveillants. Son surnom de Gosala (« étable ») viendrait de ce qu’il y serait né. Selon les sources jaïnes, il fut pendant six ans le compagnon d’ascèse de Mahâvîra, avant une rupture violente : Gosala se proclamait lui aussi « vainqueur » (&lt;em&gt;jina&lt;/em&gt;) des passions, ce que Mahâvîra lui contestait. Il mourut à Shrâvastî dans l’atelier d’une potière qui le soutenait.&lt;/p&gt; &lt;p&gt;Il défend un déterminisme absolu (&lt;em&gt;niyati&lt;/em&gt;) : tout événement, y compris le destin de chaque âme à travers ses réincarnations, est fixé d’avance, rendant vain tout effort moral ou ascétique pour infléchir son sort. Les sages comme les sots traversent un nombre fixe de grands cycles avant de voir leur souffrance prendre fin, comme une pelote de fil lancée se déroule jusqu’à son terme. Tout dépend de la destinée, des circonstances et de la nature propre de chaque être, sans que les actes y changent rien. Le Bouddha jugeait cette doctrine la pire de toutes, car elle ôte à l’homme toute raison d’agir.&lt;/p&gt; &lt;p&gt;Les Ajîvikas étaient pourtant des ascètes rigoureux, vivant nus, mendiant leur nourriture et pratiquant le jeûne. L’empereur Ashoka et son petit-fils leur offrirent les &lt;a href="https://fr.wikipedia.org/wiki/Grottes_de_Barabar" title=" Wikipedia"&gt;grottes de Barabar&lt;/a&gt;, au Bihar, parmi les plus anciennes grottes artificielles de l’Inde. Bien que  &lt;a href="https://www.youtube.com/watch?v=4_LtAMsQgMM"   title="who were the ajjivika par jay Vardhan Singh"&gt; l’Ajîvika ait disparu &lt;/a&gt; vers le XIVe siècle, il constitue un jalon important de la pensée indienne sur le déterminisme et le libre arbitre.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F37" s="1" t="s">
         <v>310</v>
@@ -7902,8 +7912,10 @@
       <c r="D40" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>333</v>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jaimini" title=" Wikipedia"&gt;Jaimini&lt;/a&gt; est l’auteur traditionnel des &lt;em&gt;Mîmâmsâ-sûtras&lt;/em&gt;, texte fondateur de l’école &lt;a href="https://fr.wikipedia.org/wiki/Mimamsa" title=" Wikipedia"&gt;Mimamsa&lt;/a&gt; (ou Pûrva-Mîmâmsâ, « première investigation »), l’une des six écoles orthodoxes de la philosophie indienne. On ne sait presque rien de sa vie : la tradition en fait un disciple de Vyâsa, le compilateur légendaire des Védas.&lt;/p&gt; &lt;p&gt;Les &lt;em&gt;Mîmâmsâ-sûtras&lt;/em&gt;, environ 2 700 aphorismes répartis en douze livres, s’ouvrent sur ces mots : « Maintenant, donc, le désir de connaître le &lt;em&gt;dharma&lt;/em&gt; ». Le &lt;em&gt;dharma&lt;/em&gt;, c’est-à-dire le devoir rituel et moral, ne se connaît ni par la perception ni par le raisonnement, mais seulement par l’injonction védique : le Véda ne décrit pas le monde, il ordonne, comme dans la formule « que celui qui désire le ciel accomplisse le sacrifice ». Le Véda n’a pas d’auteur, ni humain ni divin : il est éternel, et le lien entre les mots et leur sens l’est aussi. Cette école orthodoxe se consacre donc à l’interprétation rigoureuse des textes védiques et de leurs prescriptions rituelles, en fixant des règles pour distinguer l’ordre principal du détail, lever les contradictions apparentes et déterminer qui doit accomplir quel rite.&lt;/p&gt; &lt;p&gt;Elle développe au passage une théorie du langage et de l’herméneutique parmi les plus sophistiquées de l’Inde ancienne, fondée sur l’autorité intrinsèque et éternelle du Véda. Commentée par Shabara, puis au VIIe siècle par &lt;a href="https://fr.wikipedia.org/wiki/Kumarila_Bhatta" title=" Wikipedia"&gt;Kumârila Bhatta&lt;/a&gt; et Prabhâkara, qui fondèrent deux écoles rivales, la Mîmâmsâ inspira durablement le droit hindou et prépara la voie au Vedânta, sa « seconde investigation ». Pour la Mîmâmsâ ancienne, nul dieu créateur n’est nécessaire : le rite produit ses fruits par sa propre force.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F40" s="1" t="s">
         <v>334</v>
@@ -8674,8 +8686,10 @@
       <c r="D58" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="E58" s="2" t="s">
-        <v>489</v>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Buddhaghosa" title=" Wikipedia"&gt;Buddhaghosa&lt;/a&gt; est le plus grand commentateur et systématisateur du bouddhisme &lt;a href="https://fr.wikipedia.org/wiki/Therav%C4%81da" title=" Wikipedia"&gt;Theravâda&lt;/a&gt;. Selon les chroniques de Ceylan, il naquit dans une famille de brahmanes près de Bodh-Gaya, au Ve siècle, et se convertit après avoir été vaincu dans un débat par un moine bouddhiste. Une tradition birmane en fait au contraire un moine de Thaton, en Birmanie.&lt;/p&gt; &lt;p&gt;Moine originaire d’Inde établi au Sri Lanka, au grand monastère (&lt;em&gt;Mahâvihâra&lt;/em&gt;) d’Anurâdhapura, &lt;a href="https://www.babelio.com/auteur/-Buddhaghosa/231082/citations"   title="citations de Buddhaghosa par babelio"&gt;il rédige &lt;/a&gt; en pâli le &lt;a href="https://fr.wikipedia.org/wiki/Visuddhimagga" title=" Wikipedia"&gt;&lt;em&gt;Visuddhimagga&lt;/em&gt;&lt;/a&gt; (« Chemin de la pureté »), somme doctrinale qui organise l’ensemble de l’enseignement du Bouddha ancien autour de la discipline morale (&lt;em&gt;sīla&lt;/em&gt;), de la concentration (&lt;em&gt;samādhi&lt;/em&gt;) et de la sagesse (&lt;em&gt;paññā&lt;/em&gt;). Selon la légende, les moines l’avaient mis à l’épreuve avec deux strophes à commenter ; les dieux cachèrent deux fois son manuscrit, et il le récrivit à l’identique, si bien que les trois versions concordaient mot pour mot. L’ouvrage décrit avec précision quarante sujets de méditation et les sept étapes de la purification, de la conduite à la vision libératrice. Il y articule la méditation de quiétude (&lt;em&gt;samatha&lt;/em&gt;), qui apaise l’esprit, et celle de vision pénétrante (&lt;em&gt;vipassanā&lt;/em&gt;), qui en saisit l’impermanence.&lt;/p&gt; &lt;p&gt;Il traduisit aussi en pâli les anciens commentaires conservés en cinghalais et commenta la discipline monastique et les grands recueils de sermons. Fidèle à l’Abhidhamma, il analyse la personne en phénomènes momentanés, sans soi permanent. Son œuvre fixa l’interprétation orthodoxe des textes et demeure aujourd’hui encore la référence doctrinale du bouddhisme Theravâda, au Sri Lanka comme en Asie du Sud-Est.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F58" s="1" t="s">
         <v>490</v>
@@ -12776,402 +12790,416 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="n">
-        <v>1940</v>
+        <v>1938</v>
       </c>
       <c r="B153" s="1" t="n">
-        <v>2015</v>
+        <v>2009</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>1459</v>
+        <v>1453</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="E153" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fatima_Mernissi" title=" Wikipedia"&gt;Fatima MERNISSI&lt;/a&gt; est une sociologue et écrivaine marocaine qui grandit dans une grande maison familiale où les femmes vivent à l'écart, enfance qu'elle racontera dans &lt;em&gt;Rêves de femmes&lt;/em&gt; (1994). Appartenant à la première génération de Marocaines scolarisées, elle étudie à Rabat, à Paris, puis aux États-Unis, où elle obtient un doctorat, avant d'enseigner la sociologie à l'université Mohammed V de Rabat.&lt;/p&gt; &lt;p&gt;Son premier livre, &lt;em&gt;Sexe, idéologie, islam&lt;/em&gt; (1975), étudie la&lt;a href="https://scienceetbiencommun.pressbooks.pub/citoyennes/chapter/__unknown__/" title="Fatima Mernissi, sociologue, écrivaine et féministe marocaine par esbc"&gt; place faite aux femmes&lt;/a&gt; dans la société marocaine. Mais c'est &lt;em&gt;Le Harem politique&lt;/em&gt; (1987) qui la rend célèbre, et qui fut interdit dans son pays. Traduite dans de nombreuses langues, son œuvre a ouvert la voie à ce que l'on a appelé le féminisme islamique.&lt;/p&gt; &lt;p&gt;Elle y mène une &lt;a href="https://www.youtube.com/watch?v=Qb6iaPFs-ZI" title="Une vie : Fatima Mernissi par Brut"&gt;enquête d'historienne&lt;/a&gt; sur les paroles attribuées au Prophète qui servent à écarter les femmes de la vie publique. En utilisant les règles mêmes de la science religieuse traditionnelle, elle examine qui les a rapportées, à quel moment et dans quel intérêt, et montre leur fragilité. Pour elle, le message du Prophète était favorable à l'égalité ; ce sont les hommes de pouvoir qui, après lui, ont imposé une lecture hostile aux femmes.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Sultanes oubliées&lt;/em&gt;, elle rappelle les femmes qui ont gouverné en terre d'islam. Elle a aussi retourné le regard vers l'Europe : &lt;em&gt;Le Harem et l'Occident&lt;/em&gt; montre que les femmes occidentales sont enfermées, elles, par la tyrannie de l'image et de la minceur. Elle a animé au Maroc de nombreux ateliers d'écriture et reçu en 2003 le prix Prince des Asturies. L'année suivante, le prix Érasme lui fut décerné en même temps qu'au philosophe iranien Abdolkarim Soroush.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abdelk%C3%A9bir_Khatibi" title=" Wikipedia"&gt;Abdelkébir KHATIBI&lt;/a&gt; est un écrivain, sociologue et penseur marocain né à El Jadida. Il étudie la sociologie à la Sorbonne, où il soutient la première thèse consacrée au roman maghrébin, puis dirige à Rabat l'Institut de sociologie, et ensuite l'Institut universitaire de la recherche scientifique. Il a &lt;a href="https://www.contretemps.eu/abdelkebir-khatibi-principe-revolution/" title="Abdelkebir Khatibi, le principe révolution par contretemps"&gt;également animé &lt;/a&gt;pendant de longues années la principale revue marocaine de sciences sociales.&lt;/p&gt; &lt;p&gt;Son œuvre, écrite en français, mêle le roman, la poésie et l'essai. &lt;em&gt;La Mémoire tatouée&lt;/em&gt; (1971), sous-titrée « autobiographie d'un décolonisé », raconte son enfance entre deux langues et deux cultures. Il étudie aussi les signes de la culture populaire et savante du Maghreb : le tatouage, la calligraphie, le conte, le tapis. Roland Barthes lui rendit hommage dans un texte intitulé « Ce que je dois à Khatibi ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Maghreb pluriel&lt;/em&gt; (1983), il formule son idée centrale, la « double critique ». Pour décoloniser la pensée, il ne suffit pas de critiquer l'Occident et sa prétention à l'universel ; il faut critiquer en même temps son propre héritage, la théologie et le pouvoir patriarcal, sans quoi l'on ne fait que retourner le discours du maître. Il appelle &lt;a href="https://www.persee.fr/doc/horma_0984-2616_2009_num_60_1_2725" title="hommage à Abdelkébir Khatibi par persée"&gt;« pensée-autre » &lt;/a&gt;cette pensée qui ne se réfugie ni dans l'identité ni dans l'imitation.&lt;/p&gt; &lt;p&gt;Avec &lt;em&gt;Amour bilingue&lt;/em&gt;, il médite sur la « bi-langue » : écrire dans la langue de l'autre, habitée en secret par la langue maternelle, n'est pas une perte mais une chance. Jacques Derrida dialogue avec lui dans &lt;em&gt;Le Monolinguisme de l'autre&lt;/em&gt;. Il a aussi forgé le mot « aimance » pour désigner une relation d'affinité et d'hospitalité entre les êtres, les langues et les cultures.&lt;/p&gt;  &lt;audio controls title="Les arabes immigrés, traditions et racines par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/27050-16.09.2026-ITEMA_24673584-2023C3372E0379-NET_MFC_351639A3-9329-4471-B711-76D39FE2EEF5-25-c35cc310ff8a2a782c2f9f8d9928d6e9.m4a" type="audio/mp4" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t xml:space="preserve">UQab1UXbrM4</t>
+          <t xml:space="preserve">f8Kms-rwdIc</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Fatima Mernissi : Islam et Féminisme" par ​L'Art de Comprendre</t>
+          <t xml:space="preserve">"Marc Gontard - Abdelkébir Khatibi de Selegan au déconstructivisme" par سلسلة لقاء مع الموجه</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/fatimamernissi-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/abdelkebirkhatibi-mini.webp</t>
         </is>
       </c>
       <c r="J153" s="1" t="s">
         <v>1250</v>
       </c>
       <c r="K153" s="2" t="s">
-        <v>1043</v>
+        <v>1456</v>
       </c>
       <c r="L153" s="2" t="s">
-        <v>1462</v>
+        <v>1457</v>
       </c>
       <c r="M153" s="2" t="s">
-        <v>1463</v>
+        <v>1458</v>
       </c>
       <c r="N153" s="1" t="s">
-        <v>72</v>
+        <v>660</v>
       </c>
       <c r="O153" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P153" s="1" t="n">
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A154" s="1" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B154" s="1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fatima_Mernissi" title=" Wikipedia"&gt;Fatima MERNISSI&lt;/a&gt; est une sociologue et écrivaine marocaine qui grandit dans une grande maison familiale où les femmes vivent à l'écart, enfance qu'elle racontera dans &lt;em&gt;Rêves de femmes&lt;/em&gt; (1994). Appartenant à la première génération de Marocaines scolarisées, elle étudie à Rabat, à Paris, puis aux États-Unis, où elle obtient un doctorat, avant d'enseigner la sociologie à l'université Mohammed V de Rabat.&lt;/p&gt; &lt;p&gt;Son premier livre, &lt;em&gt;Sexe, idéologie, islam&lt;/em&gt; (1975), étudie la&lt;a href="https://scienceetbiencommun.pressbooks.pub/citoyennes/chapter/__unknown__/" title="Fatima Mernissi, sociologue, écrivaine et féministe marocaine par esbc"&gt; place faite aux femmes&lt;/a&gt; dans la société marocaine. Mais c'est &lt;em&gt;Le Harem politique&lt;/em&gt; (1987) qui la rend célèbre, et qui fut interdit dans son pays. Traduite dans de nombreuses langues, son œuvre a ouvert la voie à ce que l'on a appelé le féminisme islamique.&lt;/p&gt; &lt;p&gt;Elle y mène une &lt;a href="https://www.youtube.com/watch?v=Qb6iaPFs-ZI" title="Une vie : Fatima Mernissi par Brut"&gt;enquête d'historienne&lt;/a&gt; sur les paroles attribuées au Prophète qui servent à écarter les femmes de la vie publique. En utilisant les règles mêmes de la science religieuse traditionnelle, elle examine qui les a rapportées, à quel moment et dans quel intérêt, et montre leur fragilité. Pour elle, le message du Prophète était favorable à l'égalité ; ce sont les hommes de pouvoir qui, après lui, ont imposé une lecture hostile aux femmes.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Sultanes oubliées&lt;/em&gt;, elle rappelle les femmes qui ont gouverné en terre d'islam. Elle a aussi retourné le regard vers l'Europe : &lt;em&gt;Le Harem et l'Occident&lt;/em&gt; montre que les femmes occidentales sont enfermées, elles, par la tyrannie de l'image et de la minceur. Elle a animé au Maroc de nombreux ateliers d'écriture et reçu en 2003 le prix Prince des Asturies. L'année suivante, le prix Érasme lui fut décerné en même temps qu'au philosophe iranien Abdolkarim Soroush.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UQab1UXbrM4</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Fatima Mernissi : Islam et Féminisme" par ​L'Art de Comprendre</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/fatimamernissi-mini.webp</t>
+        </is>
+      </c>
+      <c r="J154" s="1" t="s">
+        <v>1250</v>
+      </c>
+      <c r="K154" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="L154" s="2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="M154" s="2" t="s">
+        <v>1463</v>
+      </c>
+      <c r="N154" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O154" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="P154" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="351.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A154" s="1" t="n">
+    <row r="155" customFormat="false" ht="351.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A155" s="1" t="n">
         <v>1941</v>
       </c>
-      <c r="B154" s="1" t="s">
+      <c r="B155" s="1" t="s">
         <v>1261</v>
       </c>
-      <c r="C154" s="2" t="s">
+      <c r="C155" s="2" t="s">
         <v>1262</v>
       </c>
-      <c r="D154" s="2" t="s">
+      <c r="D155" s="2" t="s">
         <v>1263</v>
       </c>
-      <c r="E154" s="2" t="s">
+      <c r="E155" s="2" t="s">
         <v>1264</v>
       </c>
-      <c r="F154" s="1" t="s">
+      <c r="F155" s="1" t="s">
         <v>1265</v>
       </c>
-      <c r="G154" s="2" t="s">
+      <c r="G155" s="2" t="s">
         <v>1266</v>
       </c>
-      <c r="H154" s="2" t="s">
+      <c r="H155" s="2" t="s">
         <v>1267</v>
       </c>
-      <c r="J154" s="1" t="s">
+      <c r="J155" s="1" t="s">
         <v>1268</v>
-      </c>
-      <c r="K154" s="2" t="s">
-        <v>1192</v>
-      </c>
-      <c r="L154" s="2" t="s">
-        <v>1061</v>
-      </c>
-      <c r="M154" s="2" t="s">
-        <v>1269</v>
-      </c>
-      <c r="O154" s="1" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="155" customFormat="false" ht="303" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A155" s="1" t="n">
-        <v>1942</v>
-      </c>
-      <c r="B155" s="1" t="s">
-        <v>1270</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>1271</v>
-      </c>
-      <c r="D155" s="2" t="s">
-        <v>1272</v>
-      </c>
-      <c r="E155" s="2" t="s">
-        <v>1273</v>
-      </c>
-      <c r="F155" s="1" t="s">
-        <v>1274</v>
-      </c>
-      <c r="G155" s="2" t="s">
-        <v>1275</v>
-      </c>
-      <c r="H155" s="2" t="s">
-        <v>1276</v>
-      </c>
-      <c r="J155" s="1" t="s">
-        <v>1277</v>
       </c>
       <c r="K155" s="2" t="s">
         <v>1192</v>
       </c>
       <c r="L155" s="2" t="s">
-        <v>1278</v>
+        <v>1061</v>
       </c>
       <c r="M155" s="2" t="s">
-        <v>1279</v>
+        <v>1269</v>
       </c>
       <c r="O155" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="P155" s="1" t="n">
+    </row>
+    <row r="156" customFormat="false" ht="303" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A156" s="1" t="n">
+        <v>1942</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>1273</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>1274</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>1275</v>
+      </c>
+      <c r="H156" s="2" t="s">
+        <v>1276</v>
+      </c>
+      <c r="J156" s="1" t="s">
+        <v>1277</v>
+      </c>
+      <c r="K156" s="2" t="s">
+        <v>1192</v>
+      </c>
+      <c r="L156" s="2" t="s">
+        <v>1278</v>
+      </c>
+      <c r="M156" s="2" t="s">
+        <v>1279</v>
+      </c>
+      <c r="O156" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="P156" s="1" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="265.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A156" s="1" t="n">
+    <row r="157" customFormat="false" ht="265.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A157" s="1" t="n">
         <v>1943</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="B157" s="1" t="s">
         <v>1243</v>
       </c>
-      <c r="C156" s="2" t="s">
+      <c r="C157" s="2" t="s">
         <v>1280</v>
       </c>
-      <c r="D156" s="2" t="s">
+      <c r="D157" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="E156" s="10" t="s">
+      <c r="E157" s="10" t="s">
         <v>1282</v>
       </c>
-      <c r="F156" s="1" t="s">
+      <c r="F157" s="1" t="s">
         <v>1283</v>
       </c>
-      <c r="G156" s="2" t="s">
+      <c r="G157" s="2" t="s">
         <v>1284</v>
       </c>
-      <c r="H156" s="2" t="s">
+      <c r="H157" s="2" t="s">
         <v>1285</v>
       </c>
-      <c r="J156" s="1" t="s">
+      <c r="J157" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K156" s="2" t="s">
+      <c r="K157" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L156" s="2" t="s">
+      <c r="L157" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="M156" s="2" t="s">
+      <c r="M157" s="2" t="s">
         <v>1286</v>
       </c>
-      <c r="O156" s="1" t="s">
+      <c r="O157" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="124.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C157" s="1"/>
-      <c r="D157" s="1"/>
-      <c r="E157" s="1"/>
-      <c r="G157" s="1"/>
-      <c r="H157" s="1"/>
-      <c r="I157" s="1"/>
-      <c r="K157" s="1"/>
-      <c r="L157" s="1"/>
-      <c r="M157" s="1"/>
-    </row>
-    <row r="158" customFormat="false" ht="280.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A158" s="1" t="n">
+    <row r="158" customFormat="false" ht="124.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C158" s="1"/>
+      <c r="D158" s="1"/>
+      <c r="E158" s="1"/>
+      <c r="G158" s="1"/>
+      <c r="H158" s="1"/>
+      <c r="I158" s="1"/>
+      <c r="K158" s="1"/>
+      <c r="L158" s="1"/>
+      <c r="M158" s="1"/>
+    </row>
+    <row r="159" customFormat="false" ht="280.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A159" s="1" t="n">
         <v>-1000</v>
       </c>
-      <c r="B158" s="1" t="n">
+      <c r="B159" s="1" t="n">
         <v>-900</v>
       </c>
-      <c r="C158" s="2" t="s">
+      <c r="C159" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="D158" s="2" t="s">
+      <c r="D159" s="2" t="s">
         <v>1288</v>
       </c>
-      <c r="E158" s="10" t="inlineStr">
+      <c r="E159" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://fr.wikipedia.org/wiki/Dialogue_du_pessimisme" title=" Wikipedia"&gt;Dialogue du PESSIMISME&lt;/a&gt; est un court texte akkadien composé en Mésopotamie qui met en scène un maître et son esclave.&lt;/p&gt; &lt;p&gt;Le maître &lt;a href="http://www.aroumah.net/seminar/Dialogue%20of%20Pessimism.pdf"&gt;annonce tour à tour &lt;/a&gt;qu'il va aller au palais, festoyer, aimer une femme, faire un sacrifice, prêter de l'argent ou servir son pays ; à chaque fois l'esclave l'approuve avec de bonnes raisons, puis, quand le maître change d'avis, l'approuve encore avec des raisons tout aussi bonnes. À la fin, le maître demande ce qui est bon : l'esclave répond qu'il vaut mieux mourir.&lt;/p&gt; &lt;p&gt;Chaque échange suit le même schéma : « Esclave, obéis-moi ! — Oui, mon maître, oui. » Le maître propose une action, l'esclave en vante les avantages ; le maître y renonce, l'esclave en montre aussitôt les dangers. Ainsi, faire l'amour à une femme fait oublier le chagrin, mais la femme est « un piège, un trou, un fossé » ; faire le bien de son pays est louable, mais personne ne distingue, parmi les crânes des morts, le bienfaiteur du malfaiteur.&lt;/p&gt; &lt;p&gt;Les spécialistes hésitent sur le sens du texte : satire comique du maître capricieux et de l'esclave flatteur, ou méditation sérieuse sur l'absence de valeur sûre ? Dans les deux cas, il met en évidence une idée troublante : pour chaque choix, on peut trouver des raisons aussi convaincantes que pour le choix contraire, de sorte que la raison seule ne permet pas de décider comment vivre.&lt;/p&gt; &lt;p&gt;Ironique ou désespéré, ce dialogue interroge la valeur de toute action humaine et annonce les grandes réflexions sceptiques et pessimistes, de Qohélet à Schopenhauer.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F159" t="inlineStr">
         <is>
           <t xml:space="preserve">0aawol43UdU</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr">
+      <c r="G159" t="inlineStr">
         <is>
           <t xml:space="preserve">"The Dialogue of Pessimism (Full Audiobook)" par abitof_ane_rd</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr">
+      <c r="H159" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/dialoguedupessimisme-mini.webp</t>
-        </is>
-      </c>
-      <c r="J158" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K158" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">metaphysique ; ethique</t>
-        </is>
-      </c>
-      <c r="L158" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="M158" s="2" t="s">
-        <v>1291</v>
-      </c>
-      <c r="O158" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="159" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A159" s="1" t="n">
-        <v>-700</v>
-      </c>
-      <c r="B159" s="1" t="n">
-        <v>-640</v>
-      </c>
-      <c r="C159" s="2" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D159" s="2" t="s">
-        <v>1293</v>
-      </c>
-      <c r="E159" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar" title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup&lt;a href="https://www.persee.fr/doc/ethio_0066-2127_1978_num_11_1_912" title="L'histoire d'Ahiqar en éthiopien par persée"&gt; concernent la parole &lt;/a&gt;: « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs le connaissaient : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une &lt;a href="https://www.youtube.com/watch?v=3HCHSrvEwuc" title="Sage Ahiqar Quotes Ancient Assyrian Wisdom par mir allround"&gt;diffusion aussi large &lt;/a&gt;à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AX9Hmh5qJ9U</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"The Story of Ahikar" par Study of Antiquity and the Middle Ages</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/ahiqar-mini.webp</t>
         </is>
       </c>
       <c r="J159" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K159" s="2" t="s">
-        <v>36</v>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique</t>
+        </is>
       </c>
       <c r="L159" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M159" s="2" t="s">
-        <v>1295</v>
+        <v>1291</v>
       </c>
       <c r="O159" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="n">
-        <v>-550</v>
+        <v>-700</v>
       </c>
       <c r="B160" s="1" t="n">
-        <v>-400</v>
+        <v>-640</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>1296</v>
+        <v>1292</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>1297</v>
-      </c>
-      <c r="E160" s="10" t="s">
-        <v>1298</v>
+        <v>1293</v>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar" title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup&lt;a href="https://www.persee.fr/doc/ethio_0066-2127_1978_num_11_1_912" title="L'histoire d'Ahiqar en éthiopien par persée"&gt; concernent la parole &lt;/a&gt;: « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs le connaissaient : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une &lt;a href="https://www.youtube.com/watch?v=3HCHSrvEwuc" title="Sage Ahiqar Quotes Ancient Assyrian Wisdom par mir allround"&gt;diffusion aussi large &lt;/a&gt;à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AX9Hmh5qJ9U</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The Story of Ahikar" par Study of Antiquity and the Middle Ages</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ahiqar-mini.webp</t>
+        </is>
       </c>
       <c r="J160" s="1" t="s">
-        <v>396</v>
+        <v>51</v>
       </c>
       <c r="K160" s="2" t="s">
-        <v>174</v>
+        <v>36</v>
       </c>
       <c r="L160" s="2" t="s">
-        <v>398</v>
+        <v>53</v>
       </c>
       <c r="M160" s="2" t="s">
-        <v>1299</v>
-      </c>
-      <c r="N160" s="1" t="s">
-        <v>400</v>
+        <v>1295</v>
       </c>
       <c r="O160" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="P160" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="n">
-        <v>-340</v>
+        <v>-550</v>
       </c>
       <c r="B161" s="1" t="n">
-        <v>-270</v>
+        <v>-400</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>1300</v>
+        <v>1296</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>1301</v>
+        <v>1297</v>
       </c>
       <c r="E161" s="10" t="s">
-        <v>1302</v>
+        <v>1298</v>
       </c>
       <c r="J161" s="1" t="s">
-        <v>51</v>
+        <v>396</v>
       </c>
       <c r="K161" s="2" t="s">
-        <v>1303</v>
+        <v>174</v>
       </c>
       <c r="L161" s="2" t="s">
-        <v>53</v>
+        <v>398</v>
       </c>
       <c r="M161" s="2" t="s">
-        <v>1304</v>
+        <v>1299</v>
+      </c>
+      <c r="N161" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O161" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="P161" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
-        <v>-250</v>
+        <v>-340</v>
       </c>
       <c r="B162" s="1" t="n">
-        <v>-220</v>
+        <v>-270</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>1305</v>
+        <v>1300</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>1306</v>
+        <v>1301</v>
       </c>
       <c r="E162" s="10" t="s">
-        <v>1307</v>
+        <v>1302</v>
       </c>
       <c r="J162" s="1" t="s">
-        <v>396</v>
+        <v>51</v>
       </c>
       <c r="K162" s="2" t="s">
-        <v>107</v>
+        <v>1303</v>
       </c>
       <c r="L162" s="2" t="s">
-        <v>398</v>
+        <v>53</v>
       </c>
       <c r="M162" s="2" t="s">
-        <v>1308</v>
-      </c>
-      <c r="N162" s="1" t="s">
-        <v>400</v>
+        <v>1304</v>
       </c>
       <c r="O162" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="P162" s="1" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13179,60 +13207,66 @@
         <v>-250</v>
       </c>
       <c r="B163" s="1" t="n">
-        <v>-100</v>
+        <v>-220</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>1309</v>
+        <v>1305</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>1310</v>
+        <v>1306</v>
       </c>
       <c r="E163" s="10" t="s">
-        <v>1311</v>
+        <v>1307</v>
       </c>
       <c r="J163" s="1" t="s">
-        <v>25</v>
+        <v>396</v>
       </c>
       <c r="K163" s="2" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="L163" s="2" t="s">
-        <v>27</v>
+        <v>398</v>
       </c>
       <c r="M163" s="2" t="s">
-        <v>1312</v>
+        <v>1308</v>
+      </c>
+      <c r="N163" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O163" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="P163" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="n">
-        <v>154</v>
+        <v>-250</v>
       </c>
       <c r="B164" s="1" t="n">
-        <v>222</v>
+        <v>-100</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>1313</v>
+        <v>1309</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>1314</v>
+        <v>1310</v>
       </c>
       <c r="E164" s="10" t="s">
-        <v>1315</v>
+        <v>1311</v>
       </c>
       <c r="J164" s="1" t="s">
-        <v>1316</v>
+        <v>25</v>
       </c>
       <c r="K164" s="2" t="s">
-        <v>107</v>
+        <v>36</v>
       </c>
       <c r="L164" s="2" t="s">
-        <v>1317</v>
+        <v>27</v>
       </c>
       <c r="M164" s="2" t="s">
-        <v>1318</v>
+        <v>1312</v>
       </c>
       <c r="O164" s="1" t="s">
         <v>29</v>
@@ -13240,139 +13274,139 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="n">
-        <v>45</v>
+        <v>154</v>
       </c>
       <c r="B165" s="1" t="n">
-        <v>117</v>
+        <v>222</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>1319</v>
+        <v>1313</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>1320</v>
+        <v>1314</v>
       </c>
       <c r="E165" s="10" t="s">
-        <v>1321</v>
+        <v>1315</v>
       </c>
       <c r="J165" s="1" t="s">
-        <v>267</v>
+        <v>1316</v>
       </c>
       <c r="K165" s="2" t="s">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="L165" s="2" t="s">
-        <v>296</v>
+        <v>1317</v>
       </c>
       <c r="M165" s="2" t="s">
-        <v>1322</v>
-      </c>
-      <c r="N165" s="1" t="s">
-        <v>72</v>
+        <v>1318</v>
       </c>
       <c r="O165" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="P165" s="1" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="n">
-        <v>1130</v>
+        <v>45</v>
       </c>
       <c r="B166" s="1" t="n">
-        <v>1160</v>
+        <v>117</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>1323</v>
+        <v>1319</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>1324</v>
+        <v>1320</v>
       </c>
       <c r="E166" s="10" t="s">
-        <v>1325</v>
+        <v>1321</v>
       </c>
       <c r="J166" s="1" t="s">
-        <v>96</v>
+        <v>267</v>
       </c>
       <c r="K166" s="2" t="s">
-        <v>427</v>
+        <v>62</v>
       </c>
       <c r="L166" s="2" t="s">
-        <v>641</v>
+        <v>296</v>
       </c>
       <c r="M166" s="2" t="s">
-        <v>1326</v>
+        <v>1322</v>
       </c>
       <c r="N166" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O166" s="1" t="s">
-        <v>100</v>
+        <v>271</v>
+      </c>
+      <c r="P166" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="n">
-        <v>832</v>
+        <v>1130</v>
       </c>
       <c r="B167" s="1" t="n">
-        <v>932</v>
+        <v>1160</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>1327</v>
+        <v>1323</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>1328</v>
+        <v>1324</v>
       </c>
       <c r="E167" s="10" t="s">
-        <v>1329</v>
+        <v>1325</v>
       </c>
       <c r="J167" s="1" t="s">
-        <v>396</v>
+        <v>96</v>
       </c>
       <c r="K167" s="2" t="s">
-        <v>346</v>
+        <v>427</v>
       </c>
       <c r="L167" s="2" t="s">
-        <v>1330</v>
+        <v>641</v>
       </c>
       <c r="M167" s="2" t="s">
-        <v>1331</v>
+        <v>1326</v>
       </c>
       <c r="N167" s="1" t="s">
-        <v>400</v>
+        <v>72</v>
       </c>
       <c r="O167" s="1" t="s">
-        <v>401</v>
+        <v>100</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="n">
-        <v>853</v>
+        <v>832</v>
       </c>
       <c r="B168" s="1" t="n">
-        <v>944</v>
+        <v>932</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>1332</v>
+        <v>1327</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>1333</v>
+        <v>1328</v>
       </c>
       <c r="E168" s="10" t="s">
-        <v>1334</v>
+        <v>1329</v>
       </c>
       <c r="J168" s="1" t="s">
-        <v>147</v>
+        <v>396</v>
       </c>
       <c r="K168" s="2" t="s">
-        <v>138</v>
+        <v>346</v>
       </c>
       <c r="L168" s="2" t="s">
-        <v>1335</v>
+        <v>1330</v>
       </c>
       <c r="M168" s="2" t="s">
-        <v>1336</v>
+        <v>1331</v>
+      </c>
+      <c r="N168" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O168" s="1" t="s">
         <v>401</v>
@@ -13380,69 +13414,63 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="1" t="n">
-        <v>874</v>
+        <v>853</v>
       </c>
       <c r="B169" s="1" t="n">
-        <v>936</v>
+        <v>944</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>1337</v>
+        <v>1332</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>1338</v>
+        <v>1333</v>
       </c>
       <c r="E169" s="10" t="s">
-        <v>1339</v>
+        <v>1334</v>
       </c>
       <c r="J169" s="1" t="s">
-        <v>545</v>
+        <v>147</v>
       </c>
       <c r="K169" s="2" t="s">
         <v>138</v>
       </c>
       <c r="L169" s="2" t="s">
-        <v>1340</v>
+        <v>1335</v>
       </c>
       <c r="M169" s="2" t="s">
-        <v>1341</v>
+        <v>1336</v>
       </c>
       <c r="O169" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P169" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="1" t="n">
-        <v>882</v>
+        <v>874</v>
       </c>
       <c r="B170" s="1" t="n">
-        <v>942</v>
+        <v>936</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>1342</v>
+        <v>1337</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>1343</v>
+        <v>1338</v>
       </c>
       <c r="E170" s="10" t="s">
-        <v>1344</v>
+        <v>1339</v>
       </c>
       <c r="J170" s="1" t="s">
-        <v>396</v>
+        <v>545</v>
       </c>
       <c r="K170" s="2" t="s">
-        <v>206</v>
+        <v>138</v>
       </c>
       <c r="L170" s="2" t="s">
-        <v>1345</v>
+        <v>1340</v>
       </c>
       <c r="M170" s="2" t="s">
-        <v>1346</v>
-      </c>
-      <c r="N170" s="1" t="s">
-        <v>400</v>
+        <v>1341</v>
       </c>
       <c r="O170" s="1" t="s">
         <v>401</v>
@@ -13453,168 +13481,168 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="1" t="n">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B171" s="1" t="n">
-        <v>931</v>
+        <v>942</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>1347</v>
+        <v>1342</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>1348</v>
+        <v>1343</v>
       </c>
       <c r="E171" s="10" t="s">
-        <v>1349</v>
+        <v>1344</v>
       </c>
       <c r="J171" s="1" t="s">
-        <v>545</v>
+        <v>396</v>
       </c>
       <c r="K171" s="2" t="s">
-        <v>138</v>
+        <v>206</v>
       </c>
       <c r="L171" s="2" t="s">
-        <v>1350</v>
+        <v>1345</v>
       </c>
       <c r="M171" s="2" t="s">
-        <v>1351</v>
+        <v>1346</v>
+      </c>
+      <c r="N171" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O171" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P171" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="1" t="n">
-        <v>994</v>
+        <v>883</v>
       </c>
       <c r="B172" s="1" t="n">
-        <v>1064</v>
+        <v>931</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>1352</v>
+        <v>1347</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>1353</v>
+        <v>1348</v>
       </c>
       <c r="E172" s="10" t="s">
-        <v>1354</v>
+        <v>1349</v>
       </c>
       <c r="J172" s="1" t="s">
         <v>545</v>
       </c>
       <c r="K172" s="2" t="s">
-        <v>1355</v>
+        <v>138</v>
       </c>
       <c r="L172" s="2" t="s">
-        <v>1335</v>
+        <v>1350</v>
       </c>
       <c r="M172" s="2" t="s">
-        <v>1356</v>
+        <v>1351</v>
       </c>
       <c r="O172" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P172" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="n">
-        <v>1004</v>
+        <v>994</v>
       </c>
       <c r="B173" s="1" t="n">
-        <v>1088</v>
+        <v>1064</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>1357</v>
+        <v>1352</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>1358</v>
+        <v>1353</v>
       </c>
       <c r="E173" s="10" t="s">
-        <v>1359</v>
+        <v>1354</v>
       </c>
       <c r="J173" s="1" t="s">
-        <v>147</v>
+        <v>545</v>
       </c>
       <c r="K173" s="2" t="s">
-        <v>206</v>
+        <v>1355</v>
       </c>
       <c r="L173" s="2" t="s">
-        <v>511</v>
+        <v>1335</v>
       </c>
       <c r="M173" s="2" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="O173" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P173" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="1" t="n">
-        <v>1021</v>
+        <v>1004</v>
       </c>
       <c r="B174" s="1" t="n">
-        <v>1058</v>
+        <v>1088</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="E174" s="10" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
       <c r="J174" s="1" t="s">
-        <v>396</v>
+        <v>147</v>
       </c>
       <c r="K174" s="2" t="s">
-        <v>1364</v>
+        <v>206</v>
       </c>
       <c r="L174" s="2" t="s">
-        <v>1330</v>
+        <v>511</v>
       </c>
       <c r="M174" s="2" t="s">
-        <v>1365</v>
-      </c>
-      <c r="N174" s="1" t="s">
-        <v>400</v>
+        <v>1360</v>
       </c>
       <c r="O174" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P174" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="1" t="n">
-        <v>1050</v>
+        <v>1021</v>
       </c>
       <c r="B175" s="1" t="n">
-        <v>1120</v>
+        <v>1058</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>1366</v>
+        <v>1361</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
       <c r="E175" s="10" t="s">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="J175" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K175" s="2" t="s">
-        <v>397</v>
+        <v>1364</v>
       </c>
       <c r="L175" s="2" t="s">
-        <v>1369</v>
+        <v>1330</v>
       </c>
       <c r="M175" s="2" t="s">
-        <v>1370</v>
+        <v>1365</v>
       </c>
       <c r="N175" s="1" t="s">
         <v>400</v>
@@ -13622,34 +13650,37 @@
       <c r="O175" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P175" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="1" t="n">
-        <v>1075</v>
+        <v>1050</v>
       </c>
       <c r="B176" s="1" t="n">
-        <v>1141</v>
+        <v>1120</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
       <c r="E176" s="10" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="J176" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K176" s="2" t="s">
-        <v>742</v>
+        <v>397</v>
       </c>
       <c r="L176" s="2" t="s">
-        <v>1374</v>
+        <v>1369</v>
       </c>
       <c r="M176" s="2" t="s">
-        <v>1375</v>
+        <v>1370</v>
       </c>
       <c r="N176" s="1" t="s">
         <v>400</v>
@@ -13657,37 +13688,34 @@
       <c r="O176" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P176" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="1" t="n">
-        <v>1092</v>
+        <v>1075</v>
       </c>
       <c r="B177" s="1" t="n">
-        <v>1167</v>
+        <v>1141</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>1376</v>
+        <v>1371</v>
       </c>
       <c r="D177" s="2" t="s">
-        <v>1377</v>
+        <v>1372</v>
       </c>
       <c r="E177" s="10" t="s">
-        <v>1378</v>
+        <v>1373</v>
       </c>
       <c r="J177" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K177" s="2" t="s">
-        <v>546</v>
+        <v>742</v>
       </c>
       <c r="L177" s="2" t="s">
-        <v>1330</v>
+        <v>1374</v>
       </c>
       <c r="M177" s="2" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
       <c r="N177" s="1" t="s">
         <v>400</v>
@@ -13695,34 +13723,37 @@
       <c r="O177" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P177" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="1" t="n">
-        <v>1110</v>
+        <v>1092</v>
       </c>
       <c r="B178" s="1" t="n">
-        <v>1180</v>
+        <v>1167</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
       <c r="E178" s="10" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="J178" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K178" s="2" t="s">
-        <v>206</v>
+        <v>546</v>
       </c>
       <c r="L178" s="2" t="s">
-        <v>1383</v>
+        <v>1330</v>
       </c>
       <c r="M178" s="2" t="s">
-        <v>1384</v>
+        <v>1379</v>
       </c>
       <c r="N178" s="1" t="s">
         <v>400</v>
@@ -13733,31 +13764,34 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="1" t="n">
-        <v>1150</v>
+        <v>1110</v>
       </c>
       <c r="B179" s="1" t="n">
-        <v>1210</v>
+        <v>1180</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>1385</v>
+        <v>1380</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>1386</v>
+        <v>1381</v>
       </c>
       <c r="E179" s="10" t="s">
-        <v>1387</v>
+        <v>1382</v>
       </c>
       <c r="J179" s="1" t="s">
-        <v>147</v>
+        <v>396</v>
       </c>
       <c r="K179" s="2" t="s">
-        <v>1388</v>
+        <v>206</v>
       </c>
       <c r="L179" s="2" t="s">
-        <v>1340</v>
+        <v>1383</v>
       </c>
       <c r="M179" s="2" t="s">
-        <v>1389</v>
+        <v>1384</v>
+      </c>
+      <c r="N179" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O179" s="1" t="s">
         <v>401</v>
@@ -13765,34 +13799,31 @@
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="1" t="n">
-        <v>1194</v>
+        <v>1150</v>
       </c>
       <c r="B180" s="1" t="n">
-        <v>1270</v>
+        <v>1210</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>1390</v>
+        <v>1385</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>1391</v>
+        <v>1386</v>
       </c>
       <c r="E180" s="10" t="s">
-        <v>1392</v>
+        <v>1387</v>
       </c>
       <c r="J180" s="1" t="s">
-        <v>396</v>
+        <v>147</v>
       </c>
       <c r="K180" s="2" t="s">
-        <v>791</v>
+        <v>1388</v>
       </c>
       <c r="L180" s="2" t="s">
-        <v>1369</v>
+        <v>1340</v>
       </c>
       <c r="M180" s="2" t="s">
-        <v>1393</v>
-      </c>
-      <c r="N180" s="1" t="s">
-        <v>1394</v>
+        <v>1389</v>
       </c>
       <c r="O180" s="1" t="s">
         <v>401</v>
@@ -13800,101 +13831,101 @@
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="1" t="n">
-        <v>1263</v>
+        <v>1194</v>
       </c>
       <c r="B181" s="1" t="n">
-        <v>1328</v>
+        <v>1270</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>1395</v>
+        <v>1390</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>1396</v>
+        <v>1391</v>
       </c>
       <c r="E181" s="10" t="s">
-        <v>1397</v>
+        <v>1392</v>
       </c>
       <c r="J181" s="1" t="s">
-        <v>545</v>
+        <v>396</v>
       </c>
       <c r="K181" s="2" t="s">
-        <v>1398</v>
+        <v>791</v>
       </c>
       <c r="L181" s="2" t="s">
-        <v>1399</v>
+        <v>1369</v>
       </c>
       <c r="M181" s="2" t="s">
-        <v>1400</v>
+        <v>1393</v>
+      </c>
+      <c r="N181" s="1" t="s">
+        <v>1394</v>
       </c>
       <c r="O181" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P181" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="1" t="n">
-        <v>1340</v>
+        <v>1263</v>
       </c>
       <c r="B182" s="1" t="n">
-        <v>1411</v>
+        <v>1328</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>1401</v>
+        <v>1395</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>1402</v>
+        <v>1396</v>
       </c>
       <c r="E182" s="10" t="s">
-        <v>1403</v>
+        <v>1397</v>
       </c>
       <c r="J182" s="1" t="s">
-        <v>396</v>
+        <v>545</v>
       </c>
       <c r="K182" s="2" t="s">
-        <v>231</v>
+        <v>1398</v>
       </c>
       <c r="L182" s="2" t="s">
-        <v>1374</v>
+        <v>1399</v>
       </c>
       <c r="M182" s="2" t="s">
-        <v>1404</v>
-      </c>
-      <c r="N182" s="1" t="s">
-        <v>1394</v>
+        <v>1400</v>
       </c>
       <c r="O182" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P182" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="1" t="n">
-        <v>1380</v>
+        <v>1340</v>
       </c>
       <c r="B183" s="1" t="n">
-        <v>1444</v>
+        <v>1411</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
       <c r="E183" s="10" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="J183" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K183" s="2" t="s">
-        <v>1408</v>
+        <v>231</v>
       </c>
       <c r="L183" s="2" t="s">
         <v>1374</v>
       </c>
       <c r="M183" s="2" t="s">
-        <v>1409</v>
+        <v>1404</v>
       </c>
       <c r="N183" s="1" t="s">
         <v>1394</v>
@@ -13905,31 +13936,31 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="1" t="n">
-        <v>1437</v>
+        <v>1380</v>
       </c>
       <c r="B184" s="1" t="n">
-        <v>1508</v>
+        <v>1444</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>1410</v>
+        <v>1405</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>1411</v>
+        <v>1406</v>
       </c>
       <c r="E184" s="10" t="s">
-        <v>1412</v>
+        <v>1407</v>
       </c>
       <c r="J184" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K184" s="2" t="s">
-        <v>1043</v>
+        <v>1408</v>
       </c>
       <c r="L184" s="2" t="s">
-        <v>1413</v>
+        <v>1374</v>
       </c>
       <c r="M184" s="2" t="s">
-        <v>1414</v>
+        <v>1409</v>
       </c>
       <c r="N184" s="1" t="s">
         <v>1394</v>
@@ -13940,31 +13971,34 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="1" t="n">
-        <v>1561</v>
+        <v>1437</v>
       </c>
       <c r="B185" s="1" t="n">
-        <v>1631</v>
+        <v>1508</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>1415</v>
+        <v>1410</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>1416</v>
+        <v>1411</v>
       </c>
       <c r="E185" s="10" t="s">
-        <v>1417</v>
+        <v>1412</v>
       </c>
       <c r="J185" s="1" t="s">
-        <v>147</v>
+        <v>396</v>
       </c>
       <c r="K185" s="2" t="s">
-        <v>206</v>
+        <v>1043</v>
       </c>
       <c r="L185" s="2" t="s">
-        <v>775</v>
+        <v>1413</v>
       </c>
       <c r="M185" s="2" t="s">
-        <v>1418</v>
+        <v>1414</v>
+      </c>
+      <c r="N185" s="1" t="s">
+        <v>1394</v>
       </c>
       <c r="O185" s="1" t="s">
         <v>401</v>
@@ -13972,136 +14006,133 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="1" t="n">
-        <v>1801</v>
+        <v>1561</v>
       </c>
       <c r="B186" s="1" t="n">
-        <v>1873</v>
+        <v>1631</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="E186" s="10" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
       <c r="J186" s="1" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="K186" s="2" t="s">
-        <v>304</v>
+        <v>206</v>
       </c>
       <c r="L186" s="2" t="s">
-        <v>1422</v>
+        <v>775</v>
       </c>
       <c r="M186" s="2" t="s">
-        <v>1423</v>
+        <v>1418</v>
       </c>
       <c r="O186" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P186" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="1" t="n">
-        <v>1849</v>
+        <v>1801</v>
       </c>
       <c r="B187" s="1" t="n">
-        <v>1905</v>
+        <v>1873</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>1424</v>
+        <v>1419</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>1425</v>
+        <v>1420</v>
       </c>
       <c r="E187" s="10" t="s">
-        <v>1426</v>
+        <v>1421</v>
       </c>
       <c r="J187" s="1" t="s">
         <v>25</v>
       </c>
       <c r="K187" s="2" t="s">
-        <v>1408</v>
+        <v>304</v>
       </c>
       <c r="L187" s="2" t="s">
-        <v>1427</v>
+        <v>1422</v>
       </c>
       <c r="M187" s="2" t="s">
-        <v>1428</v>
+        <v>1423</v>
       </c>
       <c r="O187" s="1" t="s">
         <v>401</v>
       </c>
       <c r="P187" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="1" t="n">
-        <v>1888</v>
+        <v>1849</v>
       </c>
       <c r="B188" s="1" t="n">
-        <v>1966</v>
+        <v>1905</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>1429</v>
+        <v>1424</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>1430</v>
+        <v>1425</v>
       </c>
       <c r="E188" s="10" t="s">
-        <v>1431</v>
+        <v>1426</v>
       </c>
       <c r="J188" s="1" t="s">
         <v>25</v>
       </c>
       <c r="K188" s="2" t="s">
-        <v>304</v>
+        <v>1408</v>
       </c>
       <c r="L188" s="2" t="s">
-        <v>1422</v>
+        <v>1427</v>
       </c>
       <c r="M188" s="2" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="O188" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P188" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="1" t="n">
-        <v>1905</v>
+        <v>1888</v>
       </c>
       <c r="B189" s="1" t="n">
-        <v>1973</v>
+        <v>1966</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="E189" s="10" t="s">
-        <v>1435</v>
+        <v>1431</v>
       </c>
       <c r="J189" s="1" t="s">
-        <v>1436</v>
+        <v>25</v>
       </c>
       <c r="K189" s="2" t="s">
         <v>304</v>
       </c>
       <c r="L189" s="2" t="s">
-        <v>1259</v>
+        <v>1422</v>
       </c>
       <c r="M189" s="2" t="s">
-        <v>1437</v>
-      </c>
-      <c r="N189" s="1" t="s">
-        <v>660</v>
+        <v>1432</v>
       </c>
       <c r="O189" s="1" t="s">
         <v>401</v>
@@ -14109,142 +14140,142 @@
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="1" t="n">
-        <v>1928</v>
+        <v>1905</v>
       </c>
       <c r="B190" s="1" t="n">
-        <v>2010</v>
+        <v>1973</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>1438</v>
+        <v>1433</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>1439</v>
+        <v>1434</v>
       </c>
       <c r="E190" s="10" t="s">
-        <v>1440</v>
+        <v>1435</v>
       </c>
       <c r="J190" s="1" t="s">
         <v>1436</v>
       </c>
       <c r="K190" s="2" t="s">
-        <v>26</v>
+        <v>304</v>
       </c>
       <c r="L190" s="2" t="s">
-        <v>1441</v>
+        <v>1259</v>
       </c>
       <c r="M190" s="2" t="s">
-        <v>1442</v>
+        <v>1437</v>
       </c>
       <c r="N190" s="1" t="s">
-        <v>513</v>
+        <v>660</v>
       </c>
       <c r="O190" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P190" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="1" t="n">
-        <v>1933</v>
+        <v>1928</v>
       </c>
       <c r="B191" s="1" t="n">
-        <v>1977</v>
+        <v>2010</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>1443</v>
+        <v>1438</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>1444</v>
+        <v>1439</v>
       </c>
       <c r="E191" s="10" t="s">
-        <v>1445</v>
+        <v>1440</v>
       </c>
       <c r="J191" s="1" t="s">
-        <v>147</v>
+        <v>1436</v>
       </c>
       <c r="K191" s="2" t="s">
-        <v>1043</v>
+        <v>26</v>
       </c>
       <c r="L191" s="2" t="s">
-        <v>1446</v>
+        <v>1441</v>
       </c>
       <c r="M191" s="2" t="s">
-        <v>1447</v>
+        <v>1442</v>
       </c>
       <c r="N191" s="1" t="s">
-        <v>660</v>
+        <v>513</v>
       </c>
       <c r="O191" s="1" t="s">
         <v>401</v>
       </c>
       <c r="P191" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="1" t="n">
-        <v>1935</v>
+        <v>1933</v>
       </c>
       <c r="B192" s="1" t="n">
-        <v>2021</v>
+        <v>1977</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>1448</v>
+        <v>1443</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>1449</v>
+        <v>1444</v>
       </c>
       <c r="E192" s="10" t="s">
-        <v>1450</v>
+        <v>1445</v>
       </c>
       <c r="J192" s="1" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="K192" s="2" t="s">
         <v>1043</v>
       </c>
       <c r="L192" s="2" t="s">
-        <v>1451</v>
+        <v>1446</v>
       </c>
       <c r="M192" s="2" t="s">
-        <v>1452</v>
+        <v>1447</v>
+      </c>
+      <c r="N192" s="1" t="s">
+        <v>660</v>
       </c>
       <c r="O192" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P192" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="1" t="n">
-        <v>1938</v>
+        <v>1935</v>
       </c>
       <c r="B193" s="1" t="n">
-        <v>2009</v>
+        <v>2021</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1453</v>
+        <v>1448</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>1454</v>
+        <v>1449</v>
       </c>
       <c r="E193" s="10" t="s">
-        <v>1455</v>
+        <v>1450</v>
       </c>
       <c r="J193" s="1" t="s">
-        <v>1250</v>
+        <v>25</v>
       </c>
       <c r="K193" s="2" t="s">
-        <v>1456</v>
+        <v>1043</v>
       </c>
       <c r="L193" s="2" t="s">
-        <v>1457</v>
+        <v>1451</v>
       </c>
       <c r="M193" s="2" t="s">
-        <v>1458</v>
-      </c>
-      <c r="N193" s="1" t="s">
-        <v>660</v>
+        <v>1452</v>
       </c>
       <c r="O193" s="1" t="s">
         <v>401</v>
@@ -16914,7 +16945,7 @@
     <hyperlink ref="E144" r:id="rId83" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cheikh_Anta_Diop&quot; title=&quot;Wikipedia&quot;&gt;Cheikh Anta DIOP&lt;/a&gt; était  un intellectuel sénégalais, historien, anthropologue, physicien et homme politique, considéré comme l’un des fondateurs de  &lt;a href=&quot;http://www.cheikhantadiop.net/&quot; title=&quot;cheikhantadiop &quot;&gt;l’historicité de l’Afrique &lt;/a&gt; et de la pensée afrocentrée. Né à Thieytou au Sénégal, il étudie la physique et la chimie en France, tout en approfondissant l’histoire et l’anthropologie, avant de devenir une figure majeure de la renaissance culturelle africaine dans la seconde moitié du XXᵉ siècle. Il milite aussi activement pour le panafricanisme et l’unification politique du continent, ce qui fait de lui à la fois un savant et un penseur politique engagé.  &lt;/p&gt; &lt;p&gt; Son apport le plus célèbre est la thèse selon laquelle l’Égypte ancienne est une   &lt;a href=&quot;https://www.persee.fr/doc/raipr_0033-9075_1969_num_9_1_1296&quot; title=&quot;civilisations Nègres par persée &quot;&gt;civilisation « nègre », &lt;/a&gt;  c’est‑à‑dire née d’une population d’origine subsaharienne et parente des peuples africains actuels. Dans Nations nègres et culture (1954) puis dans ses travaux ultérieurs, il mobilise des données linguistiques, anthropologiques et historiques pour montrer des parentés profondes entre les cosmo‑gonies égyptiennes et plusieurs traditions africaines (dogon, yoruba, ashanti, etc.), ce qui nourrit l’idée d’une « unité culturelle de l’Afrique noire ». Il entend ainsi retourner les discours racistes de l’époque en affirmant que l’Afrique n’est pas un continent sans histoire, mais que l’Égypte est un centre majeur de l’histoire africaine. &lt;/p&gt; &lt;p&gt; Sur le plan scientifique, il développe une approche pluridisciplinaire qui mêle linguistique, comparaison historique, anthropologie et études physique. Il critique fortement les biais culturels et eurocentrés de l’historiographie et de l’anthropologie coloniales, qui ont minimisé ou occulté l’apport des peuples africains aux civilisations humaines.  Pour lui, reconstituer &lt;a href=&quot;https://www.youtube.com/watch?v=KGlbVk3V9es&quot; title=&quot;conférence de Cheikh Anta Diop par pendanz &quot;&gt;une histoire africaine authentique &lt;/a&gt; permet non seulement de restaurer la dignité des peuples noirs, mais aussi de repenser l’histoire mondiale elle‑même. &lt;/p&gt; &lt;p&gt; Il est un penseur politique et un acteur de la scène panafricaniste : il défend un projet d’Afrique unifiée et fédéralisée, inspiré des idéaux de l’Unité africaine, et critique la division du continent héritée de la colonisation. Ses travaux influencent durablement les mouvements noirs, les études africaines et les réflexions sur la décolonisation des savoirs, tout en restant objet de débats parmi les égyptologues et les historiens. Aujourd’hui, il est souvent présenté comme l’un des grands précurseurs de la réhabilitation de l’Afrique dans l’histoire de l’humanité. &lt;/p&gt; &#10;&#10;"/>
     <hyperlink ref="E145" r:id="rId84" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Frantz_Fanon&quot; title=&quot;Wikipedia&quot;&gt;Frantz FANON&lt;/a&gt; était un penseur majeur de l’anticolonialisme, né en Martinique et devenu psychiatre, essayiste et militant engagé dans la guerre d’indépendance algérienne. Son œuvre cherche &lt;a href=&quot;https://www.youtube.com/watch?v=9hchLgKUSpU&quot; title=&quot;la Philosophie de Frantz FANON par parole de philosophe &quot;&gt;à comprendre comment &lt;/a&gt;  la colonisation détruit psychologiquement et socialement les peuples dominés, tout en fabriquant aussi une image déformée du colonisateur et du colonisé.&lt;/p&gt; &lt;p&gt; Dans Peau noire, masques blancs, il analyse la manière dont le racisme et la domination coloniale produisent un sentiment d’infériorité, des blessures psychiques et une aliénation de soi.  &lt;a href=&quot;https://fondation-frantzfanon.com/&quot; title=&quot;Fondation  Frantz FANON  &quot;&gt;Il montre que le colonisé &lt;/a&gt;  peut finir par intérioriser le regard du dominant, au point de porter un « masque » social pour tenter d’être reconnu dans un monde qui le rejette. &lt;/p&gt; &lt;p&gt; Sa pensée devient encore plus politique dans Les Damnés de la terre, où il défend l’idée que la décolonisation n’est pas seulement un changement administratif, mais une transformation radicale des rapports de pouvoir. Il insiste sur le fait que la colonisation repose elle-même sur la violence, et que la libération des colonisés passe par une rupture profonde avec cet ordre injuste. &lt;/p&gt; &lt;p&gt; Il est lu comme un précurseur des pensées décoloniales et postcoloniales, parce qu’il relie la politique, la psychologie, la culture et le corps vécu des dominés. Sa force est d’avoir montré que la lutte contre le colonialisme ne concerne pas seulement les territoires, mais aussi les esprits, les identités et les façons de penser le monde. &lt;/p&gt; &lt;audio controls title=&quot;Fanon, le phychiatre qui voulait libérer le monde par France Culture&quot;&gt;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/20905-24.05.2025-ITEMA_24146065-2025F23811S0145-NET_MFI_E4CF018B-14D9-469C-9942-543F6B9EFCA5-22.mp3&quot; type=&quot;audio/mpeg&quot;&gt; &lt;/audio&gt;"/>
     <hyperlink ref="H145" r:id="rId85" display="https://www.laphilo.fr/pho/fanon-mini.webp"/>
-    <hyperlink ref="H156" r:id="rId86" display="https://www.laphilo.fr/pho/zayd-mini.webp"/>
+    <hyperlink ref="H157" r:id="rId86" display="https://www.laphilo.fr/pho/zayd-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fiches — 3 fiches modifiées : David BENATAR, AMMONIOS d'Alexandrie, HAM SEOK-HEON ; 1 image
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-orientaux.xlsx
+++ b/data/frise-philosophes-orientaux.xlsx
@@ -13865,320 +13865,323 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A161" s="1">
+      <c r="A161" s="1" t="n">
+        <v>1901</v>
+      </c>
+      <c r="B161" s="1" t="n">
+        <v>1989</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>1617</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>1618</v>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ham_Seok-heon" title=" Wikipedia"&gt;HAM SEOK-HEON&lt;/a&gt; était un penseur, éducateur et militant quaker, &lt;a href="https://en.namu.wiki/w/%ED%95%A8%EC%84%9D%ED%97%8C" title="Ham Seok-heon par namu.wiki"&gt;figure majeure&lt;/a&gt; de la résistance non violente en Corée du Sud. Emprisonné sous l’occupation japonaise, il quitta le Nord communiste en 1947, puis s’opposa aux régimes autoritaires de Syngman Rhee, Park Chung-hee et Chun Doo-hwan.&lt;/p&gt; &lt;p&gt;Sa « philosophie ssial » fait du peuple ordinaire, la « graine » (&lt;em&gt;ssial&lt;/em&gt;), le véritable sujet de l’histoire : chaque personne porte en elle &lt;a href="https://www.youtube.com/watch?v=Bw8KgNNZa-Q" title="Ham Seok heon and The Voice of Ssial Extended Master Edition 1080p caption par James Ko"&gt;une vie spirituelle &lt;/a&gt;qui doit germer, et aucune autorité politique ou religieuse ne peut se substituer à elle. Dans &lt;em&gt;La Corée vue à travers le sens&lt;/em&gt;, il lit l’histoire coréenne, faite de souffrances répétées, comme une souffrance qui a une signification pour l’humanité entière. Inspiré par Gandhi, il défendit la non-violence et fut proposé pour le prix Nobel de la paix.&lt;/p&gt; &lt;p&gt;Étudiant à Tokyo dans les années 1920, il découvrit le mouvement « sans Église » d’Uchimura Kanzō, qui marqua durablement sa foi, avant de se rapprocher des quakers après la guerre. Son livre majeur parut d’abord sous le titre &lt;em&gt;L’histoire coréenne vue à la lumière de la Bible&lt;/em&gt;, avant d’être élargi pour s’adresser à tous, croyants ou non. En 1958, son article « Seul un peuple qui pense peut vivre », publié dans la revue &lt;em&gt;Sasanggye&lt;/em&gt;, lui valut d’être arrêté. En 1970, il fonda la revue &lt;em&gt;La Voix de la graine&lt;/em&gt; (&lt;em&gt;Ssial ui sori&lt;/em&gt;), interdite à plusieurs reprises par la censure. Sa pensée relie la non-violence de Gandhi, la mystique chrétienne et le taoïsme, et elle fut l’une des sources de la théologie du minjung.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bEWXBMPOzVU</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Ham Seok heon's Universal Christianity" par 숲대화 아카데미</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/hseokheon-mini.webp</t>
+        </is>
+      </c>
+      <c r="J161" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="K161" s="2" t="s">
+        <v>1408</v>
+      </c>
+      <c r="L161" s="2" t="s">
+        <v>1621</v>
+      </c>
+      <c r="M161" s="2" t="s">
+        <v>1622</v>
+      </c>
+      <c r="O161" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A162" s="1">
         <v>1903</v>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B162" t="inlineStr">
         <is>
           <t xml:space="preserve">1981</t>
         </is>
       </c>
-      <c r="C161" s="2" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1903 – 1981</t>
         </is>
       </c>
-      <c r="D161" s="2" t="inlineStr">
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Allameh TABATABAÏ</t>
         </is>
       </c>
-      <c r="E161" s="10" t="inlineStr">
+      <c r="E162" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Muhammad_Husayn_Tabataba%27i" title=" Wikipedia (en)"&gt;Allameh TABATABAÏ&lt;/a&gt; (de son nom Muhammad Husayn Tabatabaï ; « Allameh » signifie « le très savant ») est l’un des plus grands penseurs de l’islam chiite au XXe siècle. Né près de Tabriz, orphelin très jeune (il perd sa mère à cinq ans et son père à neuf ans), il étudie les sciences religieuses dans sa ville, puis au grand séminaire de Najaf, en Irak, où il lit Avicenne et Molla Sadra et s’initie à la mystique. Après des années difficiles comme paysan dans son village, il s’installe en 1946 à Qom, où il &lt;a href="http://www.teheran.ir/spip.php?article1302#gsc.tab=0" title="Portrait de Allâmeh Tabâtabâ’i par téhéran"&gt;enseigne la philosophie&lt;/a&gt;, discipline alors suspecte aux yeux de nombreux religieux.&lt;/p&gt; &lt;p&gt;Son œuvre la plus célèbre est &lt;em&gt;Al-Mizan&lt;/em&gt;, un commentaire du Coran en vingt-sept volumes, rédigé de 1954 à 1972, qui explique le Coran par le Coran lui-même. Philosophe, il fait revivre l’école de Molla Sadra et publie &lt;em&gt;Les Principes de la philosophie et la méthode réaliste&lt;/em&gt;, où il défend, avec son élève Morteza Motahhari, une philosophie réaliste contre le matérialisme marxiste, alors très influent chez les jeunes Iraniens.&lt;/p&gt; &lt;p&gt;De 1958 à 1977, il rencontre régulièrement le philosophe français &lt;a href="https://fr.wikipedia.org/wiki/Henry_Corbin" title=" Wikipedia"&gt;Henry Corbin&lt;/a&gt; pour de longs entretiens sur la philosophie, la mystique et les religions, l’un des grands dialogues spirituels entre l’Orient et l’Occident au XXe siècle. Avec &lt;a href="https://fr.wikipedia.org/wiki/Seyyed_Hossein_Nasr" title=" Wikipedia"&gt;Seyyed Hossein Nasr&lt;/a&gt;, il écrit aussi une présentation de l’islam chiite destinée aux lecteurs occidentaux. Il forme toute une génération de philosophes et de religieux iraniens. Il meurt à Qom en 1981 ; une grande université de Téhéran porte aujourd’hui son nom.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F162" t="inlineStr">
         <is>
           <t xml:space="preserve">ibacKDpQWvk</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr">
+      <c r="G162" t="inlineStr">
         <is>
           <t xml:space="preserve">"Part 1 - Allamah Tabataba'i Documentary - English Dubbed" par Kawthar Learning Circle</t>
         </is>
       </c>
-      <c r="H161" s="2" t="inlineStr">
+      <c r="H162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/tabatabai-mini.webp</t>
         </is>
       </c>
-      <c r="J161" s="1" t="inlineStr">
+      <c r="J162" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Perse</t>
         </is>
       </c>
-      <c r="K161" s="2" t="inlineStr">
+      <c r="K162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">metaphysique ; spiritualite</t>
         </is>
       </c>
-      <c r="L161" s="2" t="inlineStr">
+      <c r="L162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Falsafa ; Ishraqisme ; École d'Ispahan</t>
         </is>
       </c>
-      <c r="M161" s="2" t="inlineStr">
+      <c r="M162" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">philosophe et exégète chiite iranien, maître de la philosophie de Molla Sadra, interlocuteur d’Henry Corbin.</t>
         </is>
       </c>
-      <c r="O161" s="1" t="inlineStr">
+      <c r="O162" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">islam-juif</t>
         </is>
       </c>
-      <c r="P161" s="1">
+      <c r="P162" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A162" s="1" t="n">
+    <row r="163" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A163" s="1" t="n">
         <v>1906</v>
       </c>
-      <c r="B162" s="1" t="n">
+      <c r="B163" s="1" t="n">
         <v>2001</v>
       </c>
-      <c r="C162" s="2" t="s">
+      <c r="C163" s="2" t="s">
         <v>1152</v>
       </c>
-      <c r="D162" s="2" t="s">
+      <c r="D163" s="2" t="s">
         <v>1153</v>
       </c>
-      <c r="E162" s="20" t="s">
+      <c r="E163" s="20" t="s">
         <v>1154</v>
       </c>
-      <c r="F162" s="1" t="s">
+      <c r="F163" s="1" t="s">
         <v>1155</v>
       </c>
-      <c r="G162" s="2" t="s">
+      <c r="G163" s="2" t="s">
         <v>1156</v>
       </c>
-      <c r="H162" s="2" t="s">
+      <c r="H163" s="2" t="s">
         <v>1157</v>
       </c>
-      <c r="J162" s="1" t="s">
+      <c r="J163" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="K162" s="2" t="s">
+      <c r="K163" s="2" t="s">
         <v>1159</v>
       </c>
-      <c r="L162" s="2" t="inlineStr">
+      <c r="L163" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Négritude ; Socialisme africain</t>
         </is>
       </c>
-      <c r="M162" s="2" t="s">
+      <c r="M163" s="2" t="s">
         <v>1161</v>
       </c>
-      <c r="O162" s="1" t="s">
+      <c r="O163" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="P162" s="1" t="n">
+      <c r="P163" s="1" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A163" s="1">
+    <row r="164" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1">
         <v>1900</v>
       </c>
-      <c r="B163" s="1" t="inlineStr">
+      <c r="B164" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">1990</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1900 — 1990</t>
         </is>
       </c>
-      <c r="D163" s="2" t="s">
+      <c r="D164" s="2" t="s">
         <v>1163</v>
       </c>
-      <c r="E163" s="13" t="s">
+      <c r="E164" s="13" t="s">
         <v>1164</v>
       </c>
-      <c r="F163" s="1" t="s">
+      <c r="F164" s="1" t="s">
         <v>1165</v>
       </c>
-      <c r="G163" s="2" t="s">
+      <c r="G164" s="2" t="s">
         <v>1166</v>
       </c>
-      <c r="H163" s="2" t="s">
+      <c r="H164" s="2" t="s">
         <v>1167</v>
       </c>
-      <c r="J163" s="1" t="s">
+      <c r="J164" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="K163" s="2" t="s">
+      <c r="K164" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="L163" s="2" t="inlineStr">
+      <c r="L164" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bouddhisme Zen ; École de Kyōto</t>
         </is>
       </c>
-      <c r="M163" s="2" t="s">
+      <c r="M164" s="2" t="s">
         <v>1168</v>
       </c>
-      <c r="O163" s="1" t="s">
+      <c r="O164" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A164" s="1">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1">
         <v>1906</v>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B165" t="inlineStr">
         <is>
           <t xml:space="preserve">1993</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1906 – 1993</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">BUDDHADASA Bhikkhu</t>
         </is>
       </c>
-      <c r="E164" s="10" t="inlineStr">
+      <c r="E165" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Buddhadasa" title=" Wikipedia"&gt;BUDDHADASA Bhikkhu&lt;/a&gt; est un moine bouddhiste thaïlandais, l’un des grands réformateurs du bouddhisme &lt;a href="https://fr.wikipedia.org/wiki/Therav%C4%81da" title=" Wikipedia"&gt;Theravâda&lt;/a&gt; au XXe siècle. Son nom signifie « serviteur du Bouddha ». Fils d’un commerçant du sud de la Thaïlande, ordonné moine en 1926, il part étudier à Bangkok, mais il est déçu par des monastères qu’il juge plus soucieux de prestige que de libération. Il rentre&lt;a href="https://www.youtube.com/watch?v=8XrO_mjL9E4" title="Life and Work of Buddhadasa Bhikkhu par Buddhist Insights"&gt; dans sa région natale &lt;/a&gt;et fonde en 1932, dans une forêt, Suan Mokkh, le « jardin de la libération », qui deviendra un lieu de retraite pour des pratiquants du monde entier.&lt;/p&gt; &lt;p&gt;Revenant aux textes anciens en pâli, il veut dégager le cœur de l’enseignement du Bouddha des rituels, des superstitions et du commerce des mérites. Il distingue la « langue des gens », qui prend les mots à la lettre, et la « langue du dhamma », qui en saisit le sens profond. Ainsi, la renaissance ne désigne pas d’abord le passage d’une vie à une autre, mais la naissance du sentiment de « moi » et de « mien », qui se produit à chaque instant et que la pratique doit apprendre à défaire. Son idéal est un esprit « libre et vide » de cet attachement.&lt;/p&gt; &lt;p&gt;Persuadé qu’au fond toutes les religions disent la même chose, il dialogue avec des chrétiens et des musulmans. Il propose aussi un «&lt;a href="https://www.persee.fr/doc/rhr_0035-1423_1988_num_205_2_1932" title="Bhikkhu Buddhadasa. Bouddhisme et socialismes par Persée"&gt; socialisme du dhamma &lt;/a&gt;», qui fonde l’organisation de la société sur la modération et le partage plutôt que sur l’accumulation. Pendant les années démocratiques de 1973 à 1976, ses idées sont largement diffusées, et il débat à la télévision avec l’homme politique Kukrit Pramoj.&amp;nbsp;&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F165" t="inlineStr">
         <is>
           <t xml:space="preserve">B7qLDffCy_s</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr">
+      <c r="G165" t="inlineStr">
         <is>
           <t xml:space="preserve">"8612 - [3 of 6] TheThings Called 'The Five Khandhas' | Buddhadāsa Bhikkhu" par Buddhadasa Bhikkhu</t>
         </is>
       </c>
-      <c r="H164" s="2" t="inlineStr">
+      <c r="H165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/buddhadasa-mini.webp</t>
         </is>
       </c>
-      <c r="J164" s="1" t="inlineStr">
+      <c r="J165" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Thaïlandaise</t>
         </is>
       </c>
-      <c r="K164" s="2" t="inlineStr">
+      <c r="K165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">spiritualite ; ethique</t>
         </is>
       </c>
-      <c r="L164" s="2" t="inlineStr">
+      <c r="L165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bouddhisme Theravada</t>
         </is>
       </c>
-      <c r="M164" s="2" t="inlineStr">
+      <c r="M165" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">moine bouddhiste thaïlandais, réformateur du Theravâda, penseur du « socialisme du dhamma ».</t>
         </is>
       </c>
-      <c r="O164" s="1" t="inlineStr">
+      <c r="O165" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">inde</t>
         </is>
       </c>
-      <c r="P164" s="1">
+      <c r="P165" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A165" s="1" t="n">
+    <row r="166" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A166" s="1" t="n">
         <v>1909</v>
       </c>
-      <c r="B165" s="1" t="n">
+      <c r="B166" s="1" t="n">
         <v>1972</v>
       </c>
-      <c r="C165" s="2" t="s">
+      <c r="C166" s="2" t="s">
         <v>1169</v>
       </c>
-      <c r="D165" s="2" t="s">
+      <c r="D166" s="2" t="s">
         <v>1170</v>
       </c>
-      <c r="E165" s="2" t="inlineStr">
+      <c r="E166" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Kwame_Nkrumah" title=" Wikipedia"&gt;Kwame Nkrumah&lt;/a&gt; (1909-1972) est un homme d’État et philosophe ghanéen, premier dirigeant du Ghana indépendant et l’un des pères du &lt;a href="https://fr.wikipedia.org/wiki/Panafricanisme" title=" Wikipedia"&gt;panafricanisme&lt;/a&gt;. Né en Côte-de-l’Or, colonie britannique, il étudie aux États-Unis, où il lit Hegel, Marx et Marcus Garvey, puis à Londres. En 1945, il organise avec George Padmore et &lt;a href="https://fr.wikipedia.org/wiki/W._E._B._Du_Bois" title=" Wikipedia"&gt;W. E. B. Du Bois&lt;/a&gt; le congrès panafricain de Manchester.&lt;/p&gt; &lt;p&gt;Revenu au pays, il fonde en 1949 le Convention People’s Party et mène une campagne d’« action positive », non violente, qui le conduit en prison puis au pouvoir. Le 6 mars 1957, le Ghana devient le premier pays d’Afrique subsaharienne à obtenir son indépendance ; Nkrumah en est Premier ministre, puis président en 1960. Il milite pour l’unité du continent dans &lt;em&gt;L’Afrique doit s’unir&lt;/em&gt; (1963) et participe la même année à la fondation de l’&lt;a href="https://fr.wikipedia.org/wiki/Organisation_de_l%27unit%C3%A9_africaine" title=" Wikipedia"&gt;Organisation de l’unité africaine&lt;/a&gt;. Dans &lt;em&gt;Le Consciencisme&lt;/em&gt; (1964), il propose une philosophie pour l’Afrique décolonisée : unir l’héritage africain traditionnel, communautaire et égalitaire, l’apport de l’islam et celui de l’Europe chrétienne en une synthèse socialiste. Dans &lt;em&gt;Le Néo-colonialisme&lt;/em&gt; (1965), il montre que l’indépendance politique ne suffit pas si l’économie reste sous contrôle étranger.&lt;/p&gt; &lt;p&gt;Devenu autoritaire, il est renversé en 1966 par un coup d’État et meurt en exil, à Bucarest, en 1972. Il reste une figure majeure de la pensée politique africaine, célébrée au Ghana, où le jour de sa naissance, le 21 septembre, est un jour férié en son honneur.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F165" s="1" t="s">
+      <c r="F166" s="1" t="s">
         <v>1172</v>
       </c>
-      <c r="G165" s="2" t="s">
+      <c r="G166" s="2" t="s">
         <v>1173</v>
       </c>
-      <c r="H165" s="2" t="s">
+      <c r="H166" s="2" t="s">
         <v>1174</v>
       </c>
-      <c r="J165" s="1" t="s">
+      <c r="J166" s="1" t="s">
         <v>1000</v>
       </c>
-      <c r="K165" s="2" t="s">
+      <c r="K166" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L165" s="1" t="inlineStr">
+      <c r="L166" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Consciencisme ; Socialisme africain</t>
         </is>
       </c>
-      <c r="M165" s="2" t="s">
+      <c r="M166" s="2" t="s">
         <v>1176</v>
-      </c>
-      <c r="O165" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="P165" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="166" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A166" s="1" t="n">
-        <v>1913</v>
-      </c>
-      <c r="B166" s="1" t="n">
-        <v>2008</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>1177</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>1178</v>
-      </c>
-      <c r="E166" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F166" s="1" t="s">
-        <v>1180</v>
-      </c>
-      <c r="G166" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aimé Cesaire : la négritude par Ina Culture</t>
-        </is>
-      </c>
-      <c r="H166" s="2" t="s">
-        <v>1182</v>
-      </c>
-      <c r="J166" s="1" t="s">
-        <v>1183</v>
-      </c>
-      <c r="K166" s="2" t="s">
-        <v>1159</v>
-      </c>
-      <c r="L166" s="2" t="s">
-        <v>1160</v>
-      </c>
-      <c r="M166" s="2" t="s">
-        <v>1184</v>
       </c>
       <c r="O166" s="1" t="s">
         <v>660</v>
@@ -14187,130 +14190,132 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="54.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="236.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="n">
+        <v>1913</v>
+      </c>
+      <c r="B167" s="1" t="n">
+        <v>2008</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E167" s="22" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F167" s="1" t="s">
+        <v>1180</v>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aimé Cesaire : la négritude par Ina Culture</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="J167" s="1" t="s">
+        <v>1183</v>
+      </c>
+      <c r="K167" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="L167" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="M167" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="O167" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="P167" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="54.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A168" s="1" t="n">
         <v>1917</v>
       </c>
-      <c r="B167" s="1" t="s">
+      <c r="B168" s="1" t="s">
         <v>1185</v>
       </c>
-      <c r="C167" s="2" t="s">
+      <c r="C168" s="2" t="s">
         <v>1186</v>
       </c>
-      <c r="D167" s="2" t="s">
+      <c r="D168" s="2" t="s">
         <v>1187</v>
       </c>
-      <c r="E167" s="2" t="s">
+      <c r="E168" s="2" t="s">
         <v>1188</v>
       </c>
-      <c r="F167" s="1" t="s">
+      <c r="F168" s="1" t="s">
         <v>1189</v>
       </c>
-      <c r="G167" s="2" t="s">
+      <c r="G168" s="2" t="s">
         <v>1190</v>
       </c>
-      <c r="H167" s="2" t="s">
+      <c r="H168" s="2" t="s">
         <v>1191</v>
       </c>
-      <c r="J167" s="1" t="s">
+      <c r="J168" s="1" t="s">
         <v>874</v>
       </c>
-      <c r="K167" s="2" t="s">
+      <c r="K168" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="L167" s="2" t="s">
+      <c r="L168" s="2" t="s">
         <v>1193</v>
       </c>
-      <c r="M167" s="2" t="s">
+      <c r="M168" s="2" t="s">
         <v>1194</v>
       </c>
-      <c r="N167" s="1" t="s">
+      <c r="N168" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="O167" s="1" t="s">
+      <c r="O168" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A168" s="1" t="n">
+    <row r="169" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A169" s="1" t="n">
         <v>1923</v>
       </c>
-      <c r="B168" s="1" t="n">
+      <c r="B169" s="1" t="n">
         <v>1986</v>
       </c>
-      <c r="C168" s="2" t="s">
+      <c r="C169" s="2" t="s">
         <v>1195</v>
       </c>
-      <c r="D168" s="2" t="s">
+      <c r="D169" s="2" t="s">
         <v>1196</v>
       </c>
-      <c r="E168" s="22" t="s">
+      <c r="E169" s="22" t="s">
         <v>1197</v>
       </c>
-      <c r="F168" s="1" t="s">
+      <c r="F169" s="1" t="s">
         <v>1198</v>
       </c>
-      <c r="G168" s="2" t="s">
+      <c r="G169" s="2" t="s">
         <v>1199</v>
       </c>
-      <c r="H168" s="2" t="s">
+      <c r="H169" s="2" t="s">
         <v>1200</v>
       </c>
-      <c r="J168" s="1" t="s">
+      <c r="J169" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="K168" s="2" t="s">
+      <c r="K169" s="2" t="s">
         <v>848</v>
       </c>
-      <c r="L168" s="2" t="s">
+      <c r="L169" s="2" t="s">
         <v>1061</v>
       </c>
-      <c r="M168" s="2" t="s">
+      <c r="M169" s="2" t="s">
         <v>1201</v>
-      </c>
-      <c r="O168" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="P168" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="169" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A169" s="1" t="n">
-        <v>1925</v>
-      </c>
-      <c r="B169" s="1" t="n">
-        <v>1961</v>
-      </c>
-      <c r="C169" s="2" t="s">
-        <v>1202</v>
-      </c>
-      <c r="D169" s="2" t="s">
-        <v>1203</v>
-      </c>
-      <c r="E169" s="22" t="s">
-        <v>1204</v>
-      </c>
-      <c r="F169" s="1" t="s">
-        <v>1205</v>
-      </c>
-      <c r="G169" s="2" t="s">
-        <v>1206</v>
-      </c>
-      <c r="H169" s="2" t="s">
-        <v>1207</v>
-      </c>
-      <c r="J169" s="1" t="s">
-        <v>1183</v>
-      </c>
-      <c r="K169" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L169" s="2" t="s">
-        <v>1208</v>
-      </c>
-      <c r="M169" s="2" t="s">
-        <v>1209</v>
       </c>
       <c r="O169" s="1" t="s">
         <v>660</v>
@@ -14319,853 +14324,865 @@
         <v>3</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="1" t="n">
+        <v>1925</v>
+      </c>
+      <c r="B170" s="1" t="n">
+        <v>1961</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E170" s="22" t="s">
+        <v>1204</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>1205</v>
+      </c>
+      <c r="G170" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="H170" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="J170" s="1" t="s">
+        <v>1183</v>
+      </c>
+      <c r="K170" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="L170" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="M170" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="O170" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="P170" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A171" s="1" t="n">
         <v>1930</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B171" s="1" t="s">
         <v>1731</v>
       </c>
-      <c r="C170" s="2" t="s">
+      <c r="C171" s="2" t="s">
         <v>1732</v>
       </c>
-      <c r="D170" s="2" t="s">
+      <c r="D171" s="2" t="s">
         <v>1733</v>
       </c>
-      <c r="E170" s="10" t="inlineStr">
+      <c r="E171" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Li_Zehou" title=" Wikipedia"&gt;LI Zehou&lt;/a&gt; est l’un des philosophes chinois les plus influents de la seconde moitié du XXe siècle. Originaire du Hunan, diplômé de philosophie de l’université de Pékin en 1954, il se fit connaître dès les années 1950 dans les grands débats sur l’esthétique, puis devint, dans les années 1980, le maître à penser de toute une génération d’étudiants chinois.&lt;/p&gt; &lt;p&gt;Lecteur de Kant et de Marx, il soutient que les formes de la sensibilité et de la raison ne sont pas données d’avance, mais se sont formées au cours de l’histoire humaine, par la fabrication et l’usage des outils : c’est ce qu’il appelle la « sédimentation ». Le beau est ainsi « la forme de la liberté »,&lt;a href="https://www.youtube.com/watch?v=JEfuhVCN-fU" title="Hidden Truths About Confucius and Li Zehou's Philosophical par Vis Philo"&gt; l’humanisation de la nature&lt;/a&gt; par le travail collectif. Son livre &lt;em&gt;Le Chemin de la beauté&lt;/em&gt; (1981), qui parcourt l’histoire de l’art chinois, fut un immense succès. Il propose aussi de comprendre la culture chinoise comme une « culture de la joie » et du sentiment, plutôt que de la faute et du salut.&lt;/p&gt; &lt;p&gt;Après les événements de Tiananmen en 1989, ses ouvrages furent critiqués et il s’installa en 1992 aux États-Unis, où il enseigna dans plusieurs universités ; il mourut en 2021 à Boulder, dans le Colorado.&lt;a href="https://www.loyolaparis.fr/wp-content/uploads/2022/03/103-coin-des-penseurs-mars-2022.pdf" title="En mémoire à Li Zehou par loyolaparis"&gt; Dans ses derniers livres&lt;/a&gt;, il développe une « ontologie du sentiment » qui fait des émotions, cultivées par les rites et la musique, le fondement de la vie morale. Il est l’un des rares philosophes chinois contemporains à figurer dans la grande anthologie Norton de théorie et de critique littéraires.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr">
+      <c r="F171" t="inlineStr">
         <is>
           <t xml:space="preserve">p4w9h3oS5Hc</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr">
+      <c r="G171" t="inlineStr">
         <is>
           <t xml:space="preserve">"What Confucius and Li Zehou Can Teach Us About the True Meaning of Life?" par VIS PHILO</t>
         </is>
       </c>
-      <c r="H170" s="2" t="s">
+      <c r="H171" s="2" t="s">
         <v>1735</v>
       </c>
-      <c r="J170" s="1" t="s">
+      <c r="J171" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="K170" s="2" t="s">
+      <c r="K171" s="2" t="s">
         <v>1736</v>
       </c>
-      <c r="L170" s="2" t="s">
+      <c r="L171" s="2" t="s">
         <v>1193</v>
       </c>
-      <c r="M170" s="2" t="s">
+      <c r="M171" s="2" t="s">
         <v>1737</v>
       </c>
-      <c r="O170" s="1" t="s">
+      <c r="O171" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P170" s="1" t="n">
+      <c r="P171" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A171" s="1" t="n">
-        <v>1931</v>
-      </c>
-      <c r="B171" s="1" t="s">
-        <v>1210</v>
-      </c>
-      <c r="C171" s="2" t="s">
-        <v>1211</v>
-      </c>
-      <c r="D171" s="2" t="s">
-        <v>1212</v>
-      </c>
-      <c r="E171" s="2" t="s">
-        <v>1213</v>
-      </c>
-      <c r="F171" s="1" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G171" s="2" t="s">
-        <v>1215</v>
-      </c>
-      <c r="H171" s="2" t="s">
-        <v>1216</v>
-      </c>
-      <c r="J171" s="1" t="s">
-        <v>1217</v>
-      </c>
-      <c r="K171" s="2" t="s">
-        <v>848</v>
-      </c>
-      <c r="L171" s="2" t="s">
-        <v>1061</v>
-      </c>
-      <c r="M171" s="2" t="s">
-        <v>1218</v>
-      </c>
-      <c r="O171" s="1" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="172" customFormat="false" ht="307.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="1" t="n">
         <v>1931</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>1219</v>
+        <v>1210</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>1220</v>
+        <v>1211</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>1221</v>
-      </c>
-      <c r="E172" s="10" t="s">
-        <v>1222</v>
+        <v>1212</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>1213</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>1223</v>
+        <v>1214</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>1224</v>
+        <v>1215</v>
       </c>
       <c r="H172" s="2" t="s">
-        <v>1225</v>
+        <v>1216</v>
       </c>
       <c r="J172" s="1" t="s">
-        <v>1000</v>
+        <v>1217</v>
       </c>
       <c r="K172" s="2" t="s">
-        <v>1001</v>
+        <v>848</v>
       </c>
       <c r="L172" s="2" t="s">
-        <v>952</v>
+        <v>1061</v>
       </c>
       <c r="M172" s="2" t="s">
-        <v>1226</v>
+        <v>1218</v>
       </c>
       <c r="O172" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="P172" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="173" customFormat="false" ht="307.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="n">
-        <v>1928</v>
-      </c>
-      <c r="B173" s="1" t="n">
-        <v>2010</v>
+        <v>1931</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>1219</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>1438</v>
+        <v>1220</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>1439</v>
+        <v>1221</v>
       </c>
       <c r="E173" s="10" t="s">
-        <v>1440</v>
+        <v>1222</v>
+      </c>
+      <c r="F173" s="1" t="s">
+        <v>1223</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H173" s="2" t="s">
+        <v>1225</v>
       </c>
       <c r="J173" s="1" t="s">
-        <v>1436</v>
+        <v>1000</v>
       </c>
       <c r="K173" s="2" t="s">
-        <v>26</v>
+        <v>1001</v>
       </c>
       <c r="L173" s="2" t="s">
-        <v>1441</v>
+        <v>952</v>
       </c>
       <c r="M173" s="2" t="s">
-        <v>1442</v>
-      </c>
-      <c r="N173" s="1" t="s">
-        <v>513</v>
+        <v>1226</v>
       </c>
       <c r="O173" s="1" t="s">
-        <v>401</v>
+        <v>660</v>
       </c>
       <c r="P173" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A174" s="1">
+      <c r="A174" s="1" t="n">
+        <v>1928</v>
+      </c>
+      <c r="B174" s="1" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>1438</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>1439</v>
+      </c>
+      <c r="E174" s="10" t="s">
+        <v>1440</v>
+      </c>
+      <c r="J174" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="K174" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L174" s="2" t="s">
+        <v>1441</v>
+      </c>
+      <c r="M174" s="2" t="s">
+        <v>1442</v>
+      </c>
+      <c r="N174" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="O174" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="P174" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A175" s="1">
         <v>1931</v>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B175" t="inlineStr">
         <is>
           <t xml:space="preserve">2019</t>
         </is>
       </c>
-      <c r="C174" s="2" t="inlineStr">
+      <c r="C175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1931 – 2019</t>
         </is>
       </c>
-      <c r="D174" s="2" t="inlineStr">
+      <c r="D175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">John MBITI</t>
         </is>
       </c>
-      <c r="E174" s="10" t="inlineStr">
+      <c r="E175" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/John_Mbiti" title=" Wikipedia (en)"&gt;John MBITI&lt;/a&gt; est un philosophe et théologien kényan, pionnier de l’étude des religions africaines. Né à Kitui, dans l’est du Kenya, il étudie à l’université de Makerere, en Ouganda, puis aux États-Unis et à Cambridge, où il soutient un doctorat de théologie. Prêtre anglican, il enseigne à Makerere de 1964 à 1974, puis dirige l’Institut œcuménique du Conseil œcuménique des Églises, en Suisse, où il est ensuite pasteur à Burgdorf et professeur à l’université de Berne.&lt;/p&gt; &lt;p&gt;Son livre&lt;a href="https://www.youtube.com/watch?v=DElzy-ho9SA" title="Was Mbiti right? Why Africa struggles to build the future par In My Own Personal Opinion"&gt; &lt;em&gt;Religions et philosophie africaines&lt;/em&gt;&lt;/a&gt; (1969), fondé sur de longues enquêtes, conteste l’idée répandue chez les missionnaires que les religions traditionnelles africaines seraient « démoniaques » : elles méritent selon lui le même respect que le christianisme, l’islam ou le bouddhisme. Il y propose une thèse célèbre sur le temps : dans les langues qu’il étudie, le temps se compose surtout du présent vécu (&lt;em&gt;sasa&lt;/em&gt;) et d’un passé profond (&lt;em&gt;zamani&lt;/em&gt;), le futur lointain restant presque absent. Les défunts dont on garde le souvenir, les « morts-vivants », appartiennent encore au présent de la communauté.&lt;/p&gt; &lt;p&gt;Il résume la conception africaine de la personne par une formule souvent citée : « Je suis parce que nous sommes, et puisque nous sommes, donc je suis », qui fait écho à la notion d’&lt;a href="https://fr.wikipedia.org/wiki/Ubuntu_%28philosophie%29" title=" Wikipedia"&gt;ubuntu&lt;/a&gt;. Ses thèses ont été discutées, notamment par ceux qui lui reprochent de généraliser à toute l’Afrique des observations particulières, mais elles ont ouvert un champ immense à la &lt;a href="https://fr.wikipedia.org/wiki/Philosophie_africaine" title=" Wikipedia"&gt;philosophie africaine&lt;/a&gt;. Il meurt à Burgdorf en 2019.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr">
+      <c r="F175" t="inlineStr">
         <is>
           <t xml:space="preserve">mIaNQw1ECeI</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
+      <c r="G175" t="inlineStr">
         <is>
           <t xml:space="preserve">"Prof Mbiti Interview Full" par Missio Africanus</t>
         </is>
       </c>
-      <c r="H174" s="2" t="inlineStr">
+      <c r="H175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/jmbiti-mini.webp</t>
         </is>
       </c>
-      <c r="J174" s="1" t="inlineStr">
+      <c r="J175" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kényane</t>
         </is>
       </c>
-      <c r="K174" s="2" t="inlineStr">
+      <c r="K175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">spiritualite ; metaphysique</t>
         </is>
       </c>
-      <c r="L174" s="2" t="inlineStr">
+      <c r="L175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Philosophie africaine ; Ethnophilosophie</t>
         </is>
       </c>
-      <c r="M174" s="2" t="inlineStr">
+      <c r="M175" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">théologien et philosophe kényan, auteur de Religions et philosophie africaines, penseur du temps africain.</t>
         </is>
       </c>
-      <c r="O174" s="1" t="inlineStr">
+      <c r="O175" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">sud</t>
         </is>
       </c>
-      <c r="P174" s="1">
+      <c r="P175" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A175" s="1" t="n">
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A176" s="1" t="n">
         <v>1933</v>
       </c>
-      <c r="B175" s="1" t="n">
+      <c r="B176" s="1" t="n">
         <v>1977</v>
       </c>
-      <c r="C175" s="2" t="s">
+      <c r="C176" s="2" t="s">
         <v>1443</v>
       </c>
-      <c r="D175" s="2" t="s">
+      <c r="D176" s="2" t="s">
         <v>1444</v>
       </c>
-      <c r="E175" s="10" t="inlineStr">
+      <c r="E176" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%27Al%C3%AE_Shar%C3%AE%27at%C3%AE" title=" Wikipedia"&gt;Ali SHARIATI&lt;/a&gt; est un sociologue et penseur iranien né dans un village du Khorassan et mort à Southampton, en Angleterre, en 1977. Fils d'un prédicateur réformateur, il part en 1959 étudier à Paris, où il soutient un doctorat à la Sorbonne. Il y suit les cours de l'orientaliste Louis Massignon, s'engage aux côtés des Algériens en lutte pour leur indépendance et découvre Sartre et Frantz Fanon, qu'il contribue à faire connaître en Iran.&lt;/p&gt; &lt;p&gt;De retour en 1964, il est arrêté, puis enseigne à Mashhad. À partir de 1969, ses conférences dans un centre religieux de Téhéran attirent des milliers d'étudiants, et&lt;a href="https://www.youtube.com/watch?v=B0A3DJotbp4" title="Construire l'identité révolutionnaire par le Dr. Ali Shariati par Incroyable Maisvrai"&gt; leurs enregistrements &lt;/a&gt;circulent dans tout le pays. Le régime du shah ferme le centre en 1972 et l'emprisonne dix-huit mois. Il meurt peu après avoir quitté l'Iran, dans des circonstances que ses partisans jugent suspectes.&lt;/p&gt; &lt;p&gt;Il oppose deux chiismes. Le « chiisme rouge », celui d'Ali et de son fils Hussein, mort en martyr, est une religion de justice et de révolte contre l'oppression. Le « chiisme noir », devenu religion d'État sous les Safavides, est une religion de deuil, de résignation et de soumission au clergé.&lt;/p&gt; &lt;p&gt;Il appelle les peuples du tiers-monde au « retour à soi » : retrouver dans leur propre culture la force de se libérer, sans imiter ni le capitalisme occidental ni le marxisme, dont il reprend pourtant le vocabulaire. Mort deux ans avant la révolution de 1979, il en est souvent considéré comme l'inspirateur. Dans &lt;em&gt;Fatima est Fatima&lt;/em&gt;, il propose aux Iraniennes la fille du Prophète comme modèle d'une femme engagée, ni recluse ni occidentalisée.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F176" t="inlineStr">
         <is>
           <t xml:space="preserve">11mj2VwIgpA</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
+      <c r="G176" t="inlineStr">
         <is>
           <t xml:space="preserve">"Connaître l'Islam par la méthode par le Dr. Ali Shariati (Conférence 2) en Français" par Incroyable Maisvrai</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr">
+      <c r="H176" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/alishariati-mini.webp</t>
         </is>
       </c>
-      <c r="J175" s="1" t="s">
+      <c r="J176" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="K175" s="2" t="s">
+      <c r="K176" s="2" t="s">
         <v>1043</v>
       </c>
-      <c r="L175" s="2" t="s">
+      <c r="L176" s="2" t="s">
         <v>1446</v>
       </c>
-      <c r="M175" s="2" t="s">
+      <c r="M176" s="2" t="s">
         <v>1447</v>
       </c>
-      <c r="N175" s="1" t="s">
+      <c r="N176" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="O175" s="1" t="s">
+      <c r="O176" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P175" s="1" t="n">
+      <c r="P176" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="248.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A176" s="1" t="n">
+    <row r="177" customFormat="false" ht="248.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A177" s="1" t="n">
         <v>1934</v>
-      </c>
-      <c r="B176" s="1" t="s">
-        <v>1227</v>
-      </c>
-      <c r="C176" s="2" t="s">
-        <v>1228</v>
-      </c>
-      <c r="D176" s="2" t="s">
-        <v>1229</v>
-      </c>
-      <c r="E176" s="2" t="s">
-        <v>1230</v>
-      </c>
-      <c r="F176" s="1" t="s">
-        <v>1231</v>
-      </c>
-      <c r="G176" s="2" t="s">
-        <v>1232</v>
-      </c>
-      <c r="H176" s="2" t="s">
-        <v>1233</v>
-      </c>
-      <c r="J176" s="1" t="s">
-        <v>1217</v>
-      </c>
-      <c r="K176" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L176" s="2" t="s">
-        <v>1061</v>
-      </c>
-      <c r="M176" s="2" t="s">
-        <v>1234</v>
-      </c>
-      <c r="O176" s="1" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="177" customFormat="false" ht="328.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A177" s="1" t="n">
-        <v>1935</v>
       </c>
       <c r="B177" s="1" t="s">
         <v>1227</v>
       </c>
       <c r="C177" s="2" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>1229</v>
+      </c>
+      <c r="E177" s="2" t="s">
+        <v>1230</v>
+      </c>
+      <c r="F177" s="1" t="s">
+        <v>1231</v>
+      </c>
+      <c r="G177" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="H177" s="2" t="s">
+        <v>1233</v>
+      </c>
+      <c r="J177" s="1" t="s">
+        <v>1217</v>
+      </c>
+      <c r="K177" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="L177" s="2" t="s">
+        <v>1061</v>
+      </c>
+      <c r="M177" s="2" t="s">
+        <v>1234</v>
+      </c>
+      <c r="O177" s="1" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="328.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A178" s="1" t="n">
+        <v>1935</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C178" s="2" t="s">
         <v>1235</v>
       </c>
-      <c r="D177" s="2" t="s">
+      <c r="D178" s="2" t="s">
         <v>1236</v>
       </c>
-      <c r="E177" s="20" t="inlineStr">
+      <c r="E178" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sophie_Oluwole"  title=" Wikipedia"&gt;Sophie OLUWOLE&lt;/a&gt;  était une philosophe nigériane, considérée comme la première femme nigériane à obtenir un doctorat en philosophie dans une université de son pays. Elle a consacré sa vie à montrer que l’Afrique produit une &lt;a href="https://theconversation.com/sophie-oluwole-la-pionniere-nigeriane-qui-a-redefini-la-philosophie-278158" title="Sophie oluwole : la pionnière nigérienne qui a redefini la philosophie par conversation"&gt;pensée philosophique &lt;/a&gt; rigoureuse, ancrée dans ses traditions orales et notamment dans la culture iorubá. Professeure à l’Université d’Ibadan, elle s’est imposée comme une figure majeure de la philosophie africaine contemporaine et une pionnière pour les femmes dans ce domaine. &lt;/p&gt; &lt;p&gt; Elle  se définit comme une « traditionnaliste critique » : elle valorise les sages‑i oraux africains, mais les analyse avec les outils de la raison philosophique moderne. Elle accorde une grande importance à Ifá, le système de sagesse iorubá autour du sage Orunmila, qu’elle considère comme un véritable système philosophique structuré, et non seulement comme une religion ou une superstition. Pour elle, la philosophie n’est pas réservée à ceux qui savent lire et écrire ; la tradition orale africaine abrite une rationalité et une logique comparables à celles des traditions grecques classiques, &lt;/p&gt; &lt;p&gt; Un de ses travaux les plus célèbres est la comparaison entre Socrate et Orunmila, qu’elle présente comme deux « saints‑patrons » de la philosophie, l’un occidental et l’autre africain. Elle montre que tant Socrate que le sage iorubá pratiquent un questionnement critique, une recherche de la vérité et un souci de l’éthique personnelle, ce qui détruit l’idée eurocentrée selon laquelle la philosophie est une invention exclusive de la Grèce antique. Cette démarche vise à décoloniser la &lt;a href="https://www.youtube.com/watch?v=5b-54lmHCOo" title="Sophie Oluwole par Sahara Tv"&gt;discipline philosophique &lt;/a&gt; et à reconnaître la pluralité des sources de la pensée rationnelle humaine. &lt;/p&gt; &lt;p&gt; Dans ses réflexions sur le genre et la culture, Oluwole critique également les représentations négatives des femmes dans les mythes et les traditions orales, tout en défendant leur rôle intellectuel et spirituel. Elle insiste sur la nécessité de rebâtir des politiques de développement africain à partir de la langue et des savoirs autochtones, plutôt que de copier aveuglément les modèles occidentaux. Ainsi, sa philosophie articule critique de la domination culturelle, reconnaissance de la sagesse traditionnelle et engagement concret pour la dignité, l’égalité et l’autonomie des peuples africains.&lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F177" s="1" t="s">
+      <c r="F178" s="1" t="s">
         <v>1238</v>
       </c>
-      <c r="G177" s="2" t="s">
+      <c r="G178" s="2" t="s">
         <v>1239</v>
       </c>
-      <c r="H177" s="2" t="s">
+      <c r="H178" s="2" t="s">
         <v>1240</v>
       </c>
-      <c r="J177" s="1" t="s">
+      <c r="J178" s="1" t="s">
         <v>1241</v>
       </c>
-      <c r="K177" s="2" t="s">
+      <c r="K178" s="2" t="s">
         <v>1001</v>
       </c>
-      <c r="L177" s="2" t="s">
+      <c r="L178" s="2" t="s">
         <v>952</v>
       </c>
-      <c r="M177" s="2" t="s">
+      <c r="M178" s="2" t="s">
         <v>1242</v>
       </c>
-      <c r="N177" s="1" t="s">
+      <c r="N178" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="O177" s="1" t="s">
+      <c r="O178" s="1" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="323.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A178" s="1" t="n">
+    <row r="179" customFormat="false" ht="323.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A179" s="1" t="n">
         <v>1935</v>
       </c>
-      <c r="B178" s="1" t="s">
+      <c r="B179" s="1" t="s">
         <v>1243</v>
       </c>
-      <c r="C178" s="2" t="s">
+      <c r="C179" s="2" t="s">
         <v>1244</v>
       </c>
-      <c r="D178" s="2" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mohammed Abed AL-JABRI</t>
         </is>
       </c>
-      <c r="E178" s="10" t="s">
+      <c r="E179" s="10" t="s">
         <v>1246</v>
       </c>
-      <c r="F178" s="1" t="s">
+      <c r="F179" s="1" t="s">
         <v>1247</v>
       </c>
-      <c r="G178" s="2" t="s">
+      <c r="G179" s="2" t="s">
         <v>1248</v>
       </c>
-      <c r="H178" s="2" t="s">
+      <c r="H179" s="2" t="s">
         <v>1249</v>
       </c>
-      <c r="J178" s="1" t="s">
+      <c r="J179" s="1" t="s">
         <v>1250</v>
       </c>
-      <c r="K178" s="2" t="s">
+      <c r="K179" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="L178" s="2" t="s">
+      <c r="L179" s="2" t="s">
         <v>1128</v>
       </c>
-      <c r="M178" s="2" t="s">
+      <c r="M179" s="2" t="s">
         <v>1251</v>
       </c>
-      <c r="O178" s="1" t="s">
+      <c r="O179" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="347.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A179" s="1">
+    <row r="180" customFormat="false" ht="347.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A180" s="1">
         <v>1933</v>
       </c>
-      <c r="B179" s="1">
+      <c r="B180" s="1">
         <v>2005</v>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1933 — 2005</t>
         </is>
       </c>
-      <c r="D179" s="2" t="s">
+      <c r="D180" s="2" t="s">
         <v>1253</v>
       </c>
-      <c r="E179" s="10" t="inlineStr">
+      <c r="E180" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Vine_Deloria,_Jr."  title="Wikipedia"&gt;Vine DELORIA Jr.&lt;/a&gt; était  un intellectuel sioux (tribu Yankton Dakota), théologien, historien et activiste pour les droits des peuples autochtones d’Amérique du Nord. Il est surtout connu pour son livre Custer Died for Your Sins: An Indian Manifesto (1969), qui a profondément marqué le mouvement des droits indigènes aux États‑Unis et a contribué à lancer les études amérindiennes. Il se présente comme un penseur « révolutionnaire » qui critique la décadence de la culture américaine et milite pour que les jeunes Amérindiens se reconnectent d’abord  &lt;a href="https://www.youtube.com/watch?v=QOL0Gm22Jy0" title="The world we used to live in par UW Video"&gt;à leurs propres savoirs &lt;/a&gt;  avant de s’approprier la pensée occidentale.&lt;/p&gt; &lt;p&gt; Sa philosophie repose sur une critique radicale de la pensée occidentale linéaire, centrée sur l’écrit et sur une histoire vue comme progressiste, contrairement à une compréhension « spatiale » et holistique du monde propre aux peuples autochtones. Il insiste sur la centralité de la terre, du territoire sacré et des relations entre les êtres vivants (humains, non‑humains, esprits) comme fondement de l’éthique et de la spiritualité indigènes. Pour lui, la religion amérindienne n’est pas constituée de « croyances » abstraites, mais de pratiques concrètes et d’expériences vécues dans la relation au paysage, aux ancêtres et aux communautés. &lt;/p&gt; &lt;p&gt; Dans  &lt;a href="https://www.persee.fr/doc/jsa_0037-9174_1971_num_60_1_3015_t1_0335_0000_2" title="peau rouge, Vine Deloria par persée"&gt;God is Red (1973), &lt;/a&gt; il confronte la vision chrétienne du monde à la vision amérindienne, montrant que les traditions autochtones sont plus en phase avec les problèmes contemporains, notamment environnementaux et spirituels. Il critique l’anthropologie et autres sciences occidentales qui ont longtemps traité les peuples indigènes comme des objets d’étude, souvent racistes et coloniaux, et plaide pour une connaissance « indigène » qui se fonde sur la parole, la mémoire et la pratique plutôt que sur la seule abstraction. Il dénonce aussi le marxisme lorsqu’il réduit les cultures non‑européennes à des « cas » sociologiques, tout en reconnaissant que sa critique du capitalisme peut servir les luttes autochtones. &lt;/p&gt; &lt;p&gt; Il est souvent considéré comme un penseur clé de la décolonisation : il requalifie la souveraineté indigène non comme un simple statut politique, mais comme une forme de pouvoir constituant ancré dans la relation sacrée à la terre. Il défend des sociétés autochtones comme possédant des formes de pensée rationnelles, religieuses et politiques propres, capables de proposer des alternatives à la modernité capitaliste et extractiviste. Sa pensée continue d’inspirer les mouvements indigènes ainsi que les théoriciens de la justice environnementale et de la décolonisation des savoirs. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F179" s="1" t="s">
+      <c r="F180" s="1" t="s">
         <v>1255</v>
       </c>
-      <c r="G179" s="2" t="s">
+      <c r="G180" s="2" t="s">
         <v>1256</v>
       </c>
-      <c r="H179" s="2" t="s">
+      <c r="H180" s="2" t="s">
         <v>1257</v>
       </c>
-      <c r="J179" s="1" t="s">
+      <c r="J180" s="1" t="s">
         <v>1258</v>
       </c>
-      <c r="K179" s="2" t="s">
+      <c r="K180" s="2" t="s">
         <v>1043</v>
       </c>
-      <c r="L179" s="2" t="s">
+      <c r="L180" s="2" t="s">
         <v>1259</v>
       </c>
-      <c r="M179" s="2" t="s">
+      <c r="M180" s="2" t="s">
         <v>1260</v>
       </c>
-      <c r="O179" s="1" t="s">
+      <c r="O180" s="1" t="s">
         <v>660</v>
-      </c>
-    </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A180" s="1" t="n">
-        <v>1938</v>
-      </c>
-      <c r="B180" s="1" t="n">
-        <v>2009</v>
-      </c>
-      <c r="C180" s="2" t="s">
-        <v>1453</v>
-      </c>
-      <c r="D180" s="2" t="s">
-        <v>1454</v>
-      </c>
-      <c r="E180" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abdelk%C3%A9bir_Khatibi" title=" Wikipedia"&gt;Abdelkébir KHATIBI&lt;/a&gt; est un écrivain, sociologue et penseur marocain né à El Jadida. Il étudie la sociologie à la Sorbonne, où il soutient la première thèse consacrée au roman maghrébin, puis dirige à Rabat l'Institut de sociologie, et ensuite l'Institut universitaire de la recherche scientifique. Il a &lt;a href="https://www.contretemps.eu/abdelkebir-khatibi-principe-revolution/" title="Abdelkebir Khatibi, le principe révolution par contretemps"&gt;également animé &lt;/a&gt;pendant de longues années la principale revue marocaine de sciences sociales.&lt;/p&gt; &lt;p&gt;Son œuvre, écrite en français, mêle le roman, la poésie et l'essai. &lt;em&gt;La Mémoire tatouée&lt;/em&gt; (1971), sous-titrée « autobiographie d'un décolonisé », raconte son enfance entre deux langues et deux cultures. Il étudie aussi les signes de la culture populaire et savante du Maghreb : le tatouage, la calligraphie, le conte, le tapis. Roland Barthes lui rendit hommage dans un texte intitulé « Ce que je dois à Khatibi ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Maghreb pluriel&lt;/em&gt; (1983), il formule son idée centrale, la « double critique ». Pour décoloniser la pensée, il ne suffit pas de critiquer l'Occident et sa prétention à l'universel ; il faut critiquer en même temps son propre héritage, la théologie et le pouvoir patriarcal, sans quoi l'on ne fait que retourner le discours du maître. Il appelle &lt;a href="https://www.persee.fr/doc/horma_0984-2616_2009_num_60_1_2725" title="hommage à Abdelkébir Khatibi par persée"&gt;« pensée-autre » &lt;/a&gt;cette pensée qui ne se réfugie ni dans l'identité ni dans l'imitation.&lt;/p&gt; &lt;p&gt;Avec &lt;em&gt;Amour bilingue&lt;/em&gt;, il médite sur la « bi-langue » : écrire dans la langue de l'autre, habitée en secret par la langue maternelle, n'est pas une perte mais une chance. Jacques Derrida dialogue avec lui dans &lt;em&gt;Le Monolinguisme de l'autre&lt;/em&gt;. Il a aussi forgé le mot « aimance » pour désigner une relation d'affinité et d'hospitalité entre les êtres, les langues et les cultures.&lt;/p&gt;  &lt;audio controls title="Les arabes immigrés, traditions et racines par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/27050-16.09.2026-ITEMA_24673584-2023C3372E0379-NET_MFC_351639A3-9329-4471-B711-76D39FE2EEF5-25-c35cc310ff8a2a782c2f9f8d9928d6e9.m4a" type="audio/mp4" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">f8Kms-rwdIc</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Marc Gontard - Abdelkébir Khatibi de Selegan au déconstructivisme" par سلسلة لقاء مع الموجه</t>
-        </is>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/abdelkebirkhatibi-mini.webp</t>
-        </is>
-      </c>
-      <c r="J180" s="1" t="s">
-        <v>1250</v>
-      </c>
-      <c r="K180" s="2" t="s">
-        <v>1456</v>
-      </c>
-      <c r="L180" s="2" t="s">
-        <v>1457</v>
-      </c>
-      <c r="M180" s="2" t="s">
-        <v>1458</v>
-      </c>
-      <c r="N180" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="O180" s="1" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="1" t="n">
-        <v>1940</v>
+        <v>1938</v>
       </c>
       <c r="B181" s="1" t="n">
-        <v>2015</v>
+        <v>2009</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>1459</v>
+        <v>1453</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="E181" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fatima_Mernissi" title=" Wikipedia"&gt;Fatima MERNISSI&lt;/a&gt; est une sociologue et écrivaine marocaine qui grandit dans une grande maison familiale où les femmes vivent à l'écart, enfance qu'elle racontera dans &lt;em&gt;Rêves de femmes&lt;/em&gt; (1994). Appartenant à la première génération de Marocaines scolarisées, elle étudie à Rabat, à Paris, puis aux États-Unis, où elle obtient un doctorat, avant d'enseigner la sociologie à l'université Mohammed V de Rabat.&lt;/p&gt; &lt;p&gt;Son premier livre, &lt;em&gt;Sexe, idéologie, islam&lt;/em&gt; (1975), étudie la&lt;a href="https://scienceetbiencommun.pressbooks.pub/citoyennes/chapter/__unknown__/" title="Fatima Mernissi, sociologue, écrivaine et féministe marocaine par esbc"&gt; place faite aux femmes&lt;/a&gt; dans la société marocaine. Mais c'est &lt;em&gt;Le Harem politique&lt;/em&gt; (1987) qui la rend célèbre, et qui fut interdit dans son pays. Traduite dans de nombreuses langues, son œuvre a ouvert la voie à ce que l'on a appelé le féminisme islamique.&lt;/p&gt; &lt;p&gt;Elle y mène une &lt;a href="https://www.youtube.com/watch?v=Qb6iaPFs-ZI" title="Une vie : Fatima Mernissi par Brut"&gt;enquête d'historienne&lt;/a&gt; sur les paroles attribuées au Prophète qui servent à écarter les femmes de la vie publique. En utilisant les règles mêmes de la science religieuse traditionnelle, elle examine qui les a rapportées, à quel moment et dans quel intérêt, et montre leur fragilité. Pour elle, le message du Prophète était favorable à l'égalité ; ce sont les hommes de pouvoir qui, après lui, ont imposé une lecture hostile aux femmes.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Sultanes oubliées&lt;/em&gt;, elle rappelle les femmes qui ont gouverné en terre d'islam. Elle a aussi retourné le regard vers l'Europe : &lt;em&gt;Le Harem et l'Occident&lt;/em&gt; montre que les femmes occidentales sont enfermées, elles, par la tyrannie de l'image et de la minceur. Elle a animé au Maroc de nombreux ateliers d'écriture et reçu en 2003 le prix Prince des Asturies. L'année suivante, le prix Érasme lui fut décerné en même temps qu'au philosophe iranien Abdolkarim Soroush.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Abdelk%C3%A9bir_Khatibi" title=" Wikipedia"&gt;Abdelkébir KHATIBI&lt;/a&gt; est un écrivain, sociologue et penseur marocain né à El Jadida. Il étudie la sociologie à la Sorbonne, où il soutient la première thèse consacrée au roman maghrébin, puis dirige à Rabat l'Institut de sociologie, et ensuite l'Institut universitaire de la recherche scientifique. Il a &lt;a href="https://www.contretemps.eu/abdelkebir-khatibi-principe-revolution/" title="Abdelkebir Khatibi, le principe révolution par contretemps"&gt;également animé &lt;/a&gt;pendant de longues années la principale revue marocaine de sciences sociales.&lt;/p&gt; &lt;p&gt;Son œuvre, écrite en français, mêle le roman, la poésie et l'essai. &lt;em&gt;La Mémoire tatouée&lt;/em&gt; (1971), sous-titrée « autobiographie d'un décolonisé », raconte son enfance entre deux langues et deux cultures. Il étudie aussi les signes de la culture populaire et savante du Maghreb : le tatouage, la calligraphie, le conte, le tapis. Roland Barthes lui rendit hommage dans un texte intitulé « Ce que je dois à Khatibi ».&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Maghreb pluriel&lt;/em&gt; (1983), il formule son idée centrale, la « double critique ». Pour décoloniser la pensée, il ne suffit pas de critiquer l'Occident et sa prétention à l'universel ; il faut critiquer en même temps son propre héritage, la théologie et le pouvoir patriarcal, sans quoi l'on ne fait que retourner le discours du maître. Il appelle &lt;a href="https://www.persee.fr/doc/horma_0984-2616_2009_num_60_1_2725" title="hommage à Abdelkébir Khatibi par persée"&gt;« pensée-autre » &lt;/a&gt;cette pensée qui ne se réfugie ni dans l'identité ni dans l'imitation.&lt;/p&gt; &lt;p&gt;Avec &lt;em&gt;Amour bilingue&lt;/em&gt;, il médite sur la « bi-langue » : écrire dans la langue de l'autre, habitée en secret par la langue maternelle, n'est pas une perte mais une chance. Jacques Derrida dialogue avec lui dans &lt;em&gt;Le Monolinguisme de l'autre&lt;/em&gt;. Il a aussi forgé le mot « aimance » pour désigner une relation d'affinité et d'hospitalité entre les êtres, les langues et les cultures.&lt;/p&gt;  &lt;audio controls title="Les arabes immigrés, traditions et racines par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/27050-16.09.2026-ITEMA_24673584-2023C3372E0379-NET_MFC_351639A3-9329-4471-B711-76D39FE2EEF5-25-c35cc310ff8a2a782c2f9f8d9928d6e9.m4a" type="audio/mp4" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t xml:space="preserve">UQab1UXbrM4</t>
+          <t xml:space="preserve">f8Kms-rwdIc</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Fatima Mernissi : Islam et Féminisme" par ​L'Art de Comprendre</t>
+          <t xml:space="preserve">"Marc Gontard - Abdelkébir Khatibi de Selegan au déconstructivisme" par سلسلة لقاء مع الموجه</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/fatimamernissi-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/abdelkebirkhatibi-mini.webp</t>
         </is>
       </c>
       <c r="J181" s="1" t="s">
         <v>1250</v>
       </c>
       <c r="K181" s="2" t="s">
-        <v>1043</v>
+        <v>1456</v>
       </c>
       <c r="L181" s="2" t="s">
-        <v>1462</v>
+        <v>1457</v>
       </c>
       <c r="M181" s="2" t="s">
-        <v>1463</v>
+        <v>1458</v>
       </c>
       <c r="N181" s="1" t="s">
-        <v>72</v>
+        <v>660</v>
       </c>
       <c r="O181" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P181" s="1" t="n">
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A182" s="1" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B182" s="1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="E182" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fatima_Mernissi" title=" Wikipedia"&gt;Fatima MERNISSI&lt;/a&gt; est une sociologue et écrivaine marocaine qui grandit dans une grande maison familiale où les femmes vivent à l'écart, enfance qu'elle racontera dans &lt;em&gt;Rêves de femmes&lt;/em&gt; (1994). Appartenant à la première génération de Marocaines scolarisées, elle étudie à Rabat, à Paris, puis aux États-Unis, où elle obtient un doctorat, avant d'enseigner la sociologie à l'université Mohammed V de Rabat.&lt;/p&gt; &lt;p&gt;Son premier livre, &lt;em&gt;Sexe, idéologie, islam&lt;/em&gt; (1975), étudie la&lt;a href="https://scienceetbiencommun.pressbooks.pub/citoyennes/chapter/__unknown__/" title="Fatima Mernissi, sociologue, écrivaine et féministe marocaine par esbc"&gt; place faite aux femmes&lt;/a&gt; dans la société marocaine. Mais c'est &lt;em&gt;Le Harem politique&lt;/em&gt; (1987) qui la rend célèbre, et qui fut interdit dans son pays. Traduite dans de nombreuses langues, son œuvre a ouvert la voie à ce que l'on a appelé le féminisme islamique.&lt;/p&gt; &lt;p&gt;Elle y mène une &lt;a href="https://www.youtube.com/watch?v=Qb6iaPFs-ZI" title="Une vie : Fatima Mernissi par Brut"&gt;enquête d'historienne&lt;/a&gt; sur les paroles attribuées au Prophète qui servent à écarter les femmes de la vie publique. En utilisant les règles mêmes de la science religieuse traditionnelle, elle examine qui les a rapportées, à quel moment et dans quel intérêt, et montre leur fragilité. Pour elle, le message du Prophète était favorable à l'égalité ; ce sont les hommes de pouvoir qui, après lui, ont imposé une lecture hostile aux femmes.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Sultanes oubliées&lt;/em&gt;, elle rappelle les femmes qui ont gouverné en terre d'islam. Elle a aussi retourné le regard vers l'Europe : &lt;em&gt;Le Harem et l'Occident&lt;/em&gt; montre que les femmes occidentales sont enfermées, elles, par la tyrannie de l'image et de la minceur. Elle a animé au Maroc de nombreux ateliers d'écriture et reçu en 2003 le prix Prince des Asturies. L'année suivante, le prix Érasme lui fut décerné en même temps qu'au philosophe iranien Abdolkarim Soroush.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UQab1UXbrM4</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Fatima Mernissi : Islam et Féminisme" par ​L'Art de Comprendre</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/fatimamernissi-mini.webp</t>
+        </is>
+      </c>
+      <c r="J182" s="1" t="s">
+        <v>1250</v>
+      </c>
+      <c r="K182" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="L182" s="2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="M182" s="2" t="s">
+        <v>1463</v>
+      </c>
+      <c r="N182" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O182" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="P182" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="351.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A182" s="1" t="n">
+    <row r="183" customFormat="false" ht="351.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A183" s="1" t="n">
         <v>1941</v>
       </c>
-      <c r="B182" s="1" t="s">
+      <c r="B183" s="1" t="s">
         <v>1261</v>
       </c>
-      <c r="C182" s="2" t="s">
+      <c r="C183" s="2" t="s">
         <v>1262</v>
       </c>
-      <c r="D182" s="2" t="s">
+      <c r="D183" s="2" t="s">
         <v>1263</v>
       </c>
-      <c r="E182" s="2" t="s">
+      <c r="E183" s="2" t="s">
         <v>1264</v>
       </c>
-      <c r="F182" s="1" t="s">
+      <c r="F183" s="1" t="s">
         <v>1265</v>
       </c>
-      <c r="G182" s="2" t="s">
+      <c r="G183" s="2" t="s">
         <v>1266</v>
       </c>
-      <c r="H182" s="2" t="s">
+      <c r="H183" s="2" t="s">
         <v>1267</v>
       </c>
-      <c r="J182" s="1" t="s">
+      <c r="J183" s="1" t="s">
         <v>1268</v>
       </c>
-      <c r="K182" s="2" t="s">
+      <c r="K183" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="L182" s="2" t="s">
+      <c r="L183" s="2" t="s">
         <v>1061</v>
       </c>
-      <c r="M182" s="2" t="s">
+      <c r="M183" s="2" t="s">
         <v>1269</v>
       </c>
-      <c r="O182" s="1" t="s">
+      <c r="O183" s="1" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="303" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A183" s="1" t="n">
+    <row r="184" customFormat="false" ht="303" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A184" s="1" t="n">
         <v>1942</v>
       </c>
-      <c r="B183" s="1" t="s">
+      <c r="B184" s="1" t="s">
         <v>1270</v>
       </c>
-      <c r="C183" s="2" t="s">
+      <c r="C184" s="2" t="s">
         <v>1271</v>
       </c>
-      <c r="D183" s="2" t="s">
+      <c r="D184" s="2" t="s">
         <v>1272</v>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">
 &lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Paulin_Hountondji"  title=" Wikipedia"&gt;Paulin HOUTONDJI&lt;/a&gt;  était un philosophe et intellectuel béninois. Il est reconnu pour ses contributions importantes à la philosophie africaine contemporaine, en particulier pour son engagement critique envers les approches essentialistes et ethnophilosophiques qui ont souvent caractérisé la &lt;a href="https://www.youtube.com/watch?v=F3zPoQrzxp8"  title="pauli Hountondji par ithephilosopher"&gt; pensée philosophique africaine&lt;/a&gt;.&lt;/p&gt; &lt;p&gt; Il a étudié la philosophie en France, à la Sorbonne, où il a obtenu son doctorat en philosophie en 1970. Son travail a été influencé par des penseurs occidentaux tels que Karl Marx et Ludwig Wittgenstein, ainsi que par des philosophes africains comme Frantz Fanon. &lt;/p&gt; &lt;p&gt; L'une de ses œuvres les plus célèbres est le livre intitulé "Sur la philosophie africaine : critique de l'ethnophilosophie" (1976), dans lequel il remet en question l'approche essentialiste qui considère la philosophie africaine comme étant &lt;a href="https://theconversation.com/paulin-hountondji-le-penseur-qui-a-defriche-la-reflexion-sur-la-philosophie-africaine-222722"  title="pauli Hountondji parthe conversation"&gt; fondamentalement différente &lt;/a&gt;  de la philosophie occidentale en raison de ses prétendues racines culturelles profondes. Il soutient plutôt que la philosophie doit être étudiée de manière critique et indépendante de toute influence culturelle préconçue.&lt;/p&gt; &lt;p&gt; En plus de son travail philosophique, Paulin J. Il a été impliqué dans la vie politique de son pays. Il a occupé divers postes, notamment celui de ministre de l'Éducation nationale au Bénin. Son engagement envers la promotion de la pensée critique et son influence dans le domaine de la philosophie africaine lui ont valu une reconnaissance internationale. &lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F183" s="1" t="s">
+      <c r="F184" s="1" t="s">
         <v>1274</v>
       </c>
-      <c r="G183" s="2" t="s">
+      <c r="G184" s="2" t="s">
         <v>1275</v>
       </c>
-      <c r="H183" s="2" t="s">
+      <c r="H184" s="2" t="s">
         <v>1276</v>
       </c>
-      <c r="J183" s="1" t="s">
+      <c r="J184" s="1" t="s">
         <v>1277</v>
       </c>
-      <c r="K183" s="2" t="s">
+      <c r="K184" s="2" t="s">
         <v>1192</v>
       </c>
-      <c r="L183" s="2" t="s">
+      <c r="L184" s="2" t="s">
         <v>1278</v>
       </c>
-      <c r="M183" s="2" t="s">
+      <c r="M184" s="2" t="s">
         <v>1279</v>
       </c>
-      <c r="O183" s="1" t="s">
+      <c r="O184" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="P183" s="1" t="n">
+      <c r="P184" s="1" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="265.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A184" s="1" t="n">
+    <row r="185" customFormat="false" ht="265.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A185" s="1" t="n">
         <v>1943</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="B185" s="1" t="s">
         <v>1243</v>
       </c>
-      <c r="C184" s="2" t="s">
+      <c r="C185" s="2" t="s">
         <v>1280</v>
       </c>
-      <c r="D184" s="2" t="s">
+      <c r="D185" s="2" t="s">
         <v>1281</v>
       </c>
-      <c r="E184" s="10" t="s">
+      <c r="E185" s="10" t="s">
         <v>1282</v>
       </c>
-      <c r="F184" s="1" t="s">
+      <c r="F185" s="1" t="s">
         <v>1283</v>
       </c>
-      <c r="G184" s="2" t="s">
+      <c r="G185" s="2" t="s">
         <v>1284</v>
       </c>
-      <c r="H184" s="2" t="s">
+      <c r="H185" s="2" t="s">
         <v>1285</v>
       </c>
-      <c r="J184" s="1" t="s">
+      <c r="J185" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K184" s="2" t="s">
+      <c r="K185" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L184" s="2" t="s">
+      <c r="L185" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="M184" s="2" t="s">
+      <c r="M185" s="2" t="s">
         <v>1286</v>
       </c>
-      <c r="O184" s="1" t="s">
+      <c r="O185" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="124.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C185" s="1"/>
-      <c r="D185" s="1"/>
-      <c r="E185" s="1"/>
-      <c r="G185" s="1"/>
-      <c r="H185" s="1"/>
-      <c r="I185" s="1"/>
-      <c r="K185" s="1"/>
-      <c r="L185" s="1"/>
-      <c r="M185" s="1"/>
-    </row>
-    <row r="186" customFormat="false" ht="280.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A186" s="1" t="n">
+    <row r="186" customFormat="false" ht="124.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C186" s="1"/>
+      <c r="D186" s="1"/>
+      <c r="E186" s="1"/>
+      <c r="G186" s="1"/>
+      <c r="H186" s="1"/>
+      <c r="I186" s="1"/>
+      <c r="K186" s="1"/>
+      <c r="L186" s="1"/>
+      <c r="M186" s="1"/>
+    </row>
+    <row r="187" customFormat="false" ht="280.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A187" s="1" t="n">
         <v>-1000</v>
       </c>
-      <c r="B186" s="1" t="n">
+      <c r="B187" s="1" t="n">
         <v>-900</v>
       </c>
-      <c r="C186" s="2" t="s">
+      <c r="C187" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="D186" s="2" t="s">
+      <c r="D187" s="2" t="s">
         <v>1288</v>
       </c>
-      <c r="E186" s="10" t="inlineStr">
+      <c r="E187" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;Le &lt;a href="https://fr.wikipedia.org/wiki/Dialogue_du_pessimisme" title=" Wikipedia"&gt;Dialogue du PESSIMISME&lt;/a&gt; est un court texte akkadien composé en Mésopotamie qui met en scène un maître et son esclave.&lt;/p&gt; &lt;p&gt;Le maître &lt;a href="http://www.aroumah.net/seminar/Dialogue%20of%20Pessimism.pdf"&gt;annonce tour à tour &lt;/a&gt;qu'il va aller au palais, festoyer, aimer une femme, faire un sacrifice, prêter de l'argent ou servir son pays ; à chaque fois l'esclave l'approuve avec de bonnes raisons, puis, quand le maître change d'avis, l'approuve encore avec des raisons tout aussi bonnes. À la fin, le maître demande ce qui est bon : l'esclave répond qu'il vaut mieux mourir.&lt;/p&gt; &lt;p&gt;Chaque échange suit le même schéma : « Esclave, obéis-moi ! — Oui, mon maître, oui. » Le maître propose une action, l'esclave en vante les avantages ; le maître y renonce, l'esclave en montre aussitôt les dangers. Ainsi, faire l'amour à une femme fait oublier le chagrin, mais la femme est « un piège, un trou, un fossé » ; faire le bien de son pays est louable, mais personne ne distingue, parmi les crânes des morts, le bienfaiteur du malfaiteur.&lt;/p&gt; &lt;p&gt;Les spécialistes hésitent sur le sens du texte : satire comique du maître capricieux et de l'esclave flatteur, ou méditation sérieuse sur l'absence de valeur sûre ? Dans les deux cas, il met en évidence une idée troublante : pour chaque choix, on peut trouver des raisons aussi convaincantes que pour le choix contraire, de sorte que la raison seule ne permet pas de décider comment vivre.&lt;/p&gt; &lt;p&gt;Ironique ou désespéré, ce dialogue interroge la valeur de toute action humaine et annonce les grandes réflexions sceptiques et pessimistes, de Qohélet à Schopenhauer.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F187" t="inlineStr">
         <is>
           <t xml:space="preserve">0aawol43UdU</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr">
+      <c r="G187" t="inlineStr">
         <is>
           <t xml:space="preserve">"The Dialogue of Pessimism (Full Audiobook)" par abitof_ane_rd</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr">
+      <c r="H187" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.laphilo.fr/pho/dialoguedupessimisme-mini.webp</t>
-        </is>
-      </c>
-      <c r="J186" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K186" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">metaphysique ; ethique</t>
-        </is>
-      </c>
-      <c r="L186" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="M186" s="2" t="s">
-        <v>1291</v>
-      </c>
-      <c r="O186" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="187" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A187" s="1" t="n">
-        <v>-700</v>
-      </c>
-      <c r="B187" s="1" t="n">
-        <v>-640</v>
-      </c>
-      <c r="C187" s="2" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D187" s="2" t="s">
-        <v>1293</v>
-      </c>
-      <c r="E187" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar" title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup&lt;a href="https://www.persee.fr/doc/ethio_0066-2127_1978_num_11_1_912" title="L'histoire d'Ahiqar en éthiopien par persée"&gt; concernent la parole &lt;/a&gt;: « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs le connaissaient : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une &lt;a href="https://www.youtube.com/watch?v=3HCHSrvEwuc" title="Sage Ahiqar Quotes Ancient Assyrian Wisdom par mir allround"&gt;diffusion aussi large &lt;/a&gt;à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AX9Hmh5qJ9U</t>
-        </is>
-      </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"The Story of Ahikar" par Study of Antiquity and the Middle Ages</t>
-        </is>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/ahiqar-mini.webp</t>
         </is>
       </c>
       <c r="J187" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K187" s="2" t="s">
-        <v>36</v>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metaphysique ; ethique</t>
+        </is>
       </c>
       <c r="L187" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M187" s="2" t="s">
-        <v>1295</v>
+        <v>1291</v>
       </c>
       <c r="O187" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="292.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="1" t="n">
-        <v>154</v>
+        <v>-700</v>
       </c>
       <c r="B188" s="1" t="n">
-        <v>222</v>
+        <v>-640</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>1313</v>
+        <v>1292</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>1314</v>
-      </c>
-      <c r="E188" s="10" t="s">
-        <v>1315</v>
+        <v>1293</v>
+      </c>
+      <c r="E188" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ahiqar" title=" Wikipedia"&gt;AHIQAR&lt;/a&gt; est un sage présenté comme le chancelier des rois assyriens Sennachérib et Assarhaddon (680-669 avant J.-C.). Son histoire et ses maximes nous sont parvenues par des papyrus araméens retrouvés à Éléphantine, en Égypte, datant de la fin du Ve siècle avant J.-C.&lt;/p&gt; &lt;p&gt;Le récit raconte comment Ahiqar, trahi par son neveu adoptif Nadin qu'il avait élevé, est condamné à mort, sauvé par un ami, puis rétabli dans son honneur. Il est suivi d'un recueil de proverbes sur la prudence dans les paroles, l'éducation des enfants, la loyauté et l'ingratitude.&lt;/p&gt; &lt;p&gt;Parmi ses maximes, beaucoup&lt;a href="https://www.persee.fr/doc/ethio_0066-2127_1978_num_11_1_912" title="L'histoire d'Ahiqar en éthiopien par persée"&gt; concernent la parole &lt;/a&gt;: « Garde ta bouche plus que toute autre chose », « Un mot est un oiseau : une fois lâché, personne ne peut le rattraper ». D'autres prônent la sévérité dans l'éducation des enfants, la fidélité au roi, la méfiance envers les méchants et la reconnaissance envers ceux qui nous ont fait du bien. Dans certaines versions, Ahiqar reproche longuement à Nadin son ingratitude à travers une série de comparaisons tirées de la nature.&lt;/p&gt; &lt;p&gt;Les Grecs le connaissaient : le philosophe Démocrite aurait, selon une tradition, emprunté ses préceptes, et la légendaire &lt;em&gt;Vie d'Ésope&lt;/em&gt; reprend presque entièrement son histoire. Le personnage apparaît aussi dans le Coran sous les traits de Luqman le Sage selon certains commentateurs. Peu de textes antiques ont connu une &lt;a href="https://www.youtube.com/watch?v=3HCHSrvEwuc" title="Sage Ahiqar Quotes Ancient Assyrian Wisdom par mir allround"&gt;diffusion aussi large &lt;/a&gt;à travers les langues et les religions.&lt;/p&gt; &lt;p&gt;L'histoire d'Ahiqar a connu un succès immense : on la retrouve dans la Bible (livre de Tobie), chez les Grecs, dans les traditions syriaque, arabe et arménienne. Elle montre la circulation d'une même sagesse populaire dans tout le Proche-Orient.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AX9Hmh5qJ9U</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The Story of Ahikar" par Study of Antiquity and the Middle Ages</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/ahiqar-mini.webp</t>
+        </is>
       </c>
       <c r="J188" s="1" t="s">
-        <v>1316</v>
+        <v>51</v>
       </c>
       <c r="K188" s="2" t="s">
-        <v>107</v>
+        <v>36</v>
       </c>
       <c r="L188" s="2" t="s">
-        <v>1317</v>
+        <v>53</v>
       </c>
       <c r="M188" s="2" t="s">
-        <v>1318</v>
+        <v>1295</v>
       </c>
       <c r="O188" s="1" t="s">
         <v>29</v>
@@ -15173,104 +15190,98 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="1" t="n">
-        <v>832</v>
+        <v>154</v>
       </c>
       <c r="B189" s="1" t="n">
-        <v>932</v>
+        <v>222</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>1327</v>
+        <v>1313</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>1328</v>
+        <v>1314</v>
       </c>
       <c r="E189" s="10" t="s">
-        <v>1329</v>
+        <v>1315</v>
       </c>
       <c r="J189" s="1" t="s">
-        <v>396</v>
+        <v>1316</v>
       </c>
       <c r="K189" s="2" t="s">
-        <v>346</v>
+        <v>107</v>
       </c>
       <c r="L189" s="2" t="s">
-        <v>1330</v>
+        <v>1317</v>
       </c>
       <c r="M189" s="2" t="s">
-        <v>1331</v>
-      </c>
-      <c r="N189" s="1" t="s">
-        <v>400</v>
+        <v>1318</v>
       </c>
       <c r="O189" s="1" t="s">
-        <v>401</v>
+        <v>29</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="1" t="n">
-        <v>874</v>
+        <v>832</v>
       </c>
       <c r="B190" s="1" t="n">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>1337</v>
+        <v>1327</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>1338</v>
+        <v>1328</v>
       </c>
       <c r="E190" s="10" t="s">
-        <v>1339</v>
+        <v>1329</v>
       </c>
       <c r="J190" s="1" t="s">
-        <v>545</v>
+        <v>396</v>
       </c>
       <c r="K190" s="2" t="s">
-        <v>138</v>
+        <v>346</v>
       </c>
       <c r="L190" s="2" t="s">
-        <v>1340</v>
+        <v>1330</v>
       </c>
       <c r="M190" s="2" t="s">
-        <v>1341</v>
+        <v>1331</v>
+      </c>
+      <c r="N190" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O190" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P190" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="1" t="n">
-        <v>882</v>
+        <v>874</v>
       </c>
       <c r="B191" s="1" t="n">
-        <v>942</v>
+        <v>936</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>1342</v>
+        <v>1337</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>1343</v>
+        <v>1338</v>
       </c>
       <c r="E191" s="10" t="s">
-        <v>1344</v>
+        <v>1339</v>
       </c>
       <c r="J191" s="1" t="s">
-        <v>396</v>
+        <v>545</v>
       </c>
       <c r="K191" s="2" t="s">
-        <v>206</v>
+        <v>138</v>
       </c>
       <c r="L191" s="2" t="s">
-        <v>1345</v>
+        <v>1340</v>
       </c>
       <c r="M191" s="2" t="s">
-        <v>1346</v>
-      </c>
-      <c r="N191" s="1" t="s">
-        <v>400</v>
+        <v>1341</v>
       </c>
       <c r="O191" s="1" t="s">
         <v>401</v>
@@ -15281,170 +15292,170 @@
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="1" t="n">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B192" s="1" t="n">
-        <v>931</v>
+        <v>942</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>1347</v>
+        <v>1342</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>1348</v>
+        <v>1343</v>
       </c>
       <c r="E192" s="10" t="s">
-        <v>1349</v>
+        <v>1344</v>
       </c>
       <c r="J192" s="1" t="s">
-        <v>545</v>
+        <v>396</v>
       </c>
       <c r="K192" s="2" t="s">
-        <v>138</v>
+        <v>206</v>
       </c>
       <c r="L192" s="2" t="s">
-        <v>1350</v>
+        <v>1345</v>
       </c>
       <c r="M192" s="2" t="s">
-        <v>1351</v>
+        <v>1346</v>
+      </c>
+      <c r="N192" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O192" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P192" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="1" t="n">
-        <v>994</v>
+        <v>883</v>
       </c>
       <c r="B193" s="1" t="n">
-        <v>1064</v>
+        <v>931</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1352</v>
+        <v>1347</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>1353</v>
+        <v>1348</v>
       </c>
       <c r="E193" s="10" t="s">
-        <v>1354</v>
+        <v>1349</v>
       </c>
       <c r="J193" s="1" t="s">
         <v>545</v>
       </c>
       <c r="K193" s="2" t="s">
-        <v>1355</v>
+        <v>138</v>
       </c>
       <c r="L193" s="2" t="s">
-        <v>1335</v>
+        <v>1350</v>
       </c>
       <c r="M193" s="2" t="s">
-        <v>1356</v>
+        <v>1351</v>
       </c>
       <c r="O193" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P193" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="1" t="n">
-        <v>1004</v>
+        <v>994</v>
       </c>
       <c r="B194" s="1" t="n">
-        <v>1088</v>
+        <v>1064</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>1357</v>
+        <v>1352</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>1358</v>
+        <v>1353</v>
       </c>
       <c r="E194" s="10" t="s">
-        <v>1359</v>
+        <v>1354</v>
       </c>
       <c r="J194" s="1" t="s">
-        <v>147</v>
+        <v>545</v>
       </c>
       <c r="K194" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="L194" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Néoplatonisme ; Ismaélisme</t>
-        </is>
+        <v>1355</v>
+      </c>
+      <c r="L194" s="2" t="s">
+        <v>1335</v>
       </c>
       <c r="M194" s="2" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="O194" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P194" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="1" t="n">
-        <v>1021</v>
+        <v>1004</v>
       </c>
       <c r="B195" s="1" t="n">
-        <v>1058</v>
+        <v>1088</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="E195" s="10" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
       <c r="J195" s="1" t="s">
-        <v>396</v>
+        <v>147</v>
       </c>
       <c r="K195" s="2" t="s">
-        <v>1364</v>
-      </c>
-      <c r="L195" s="2" t="s">
-        <v>1330</v>
+        <v>206</v>
+      </c>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Néoplatonisme ; Ismaélisme</t>
+        </is>
       </c>
       <c r="M195" s="2" t="s">
-        <v>1365</v>
-      </c>
-      <c r="N195" s="1" t="s">
-        <v>400</v>
+        <v>1360</v>
       </c>
       <c r="O195" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P195" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="1" t="n">
-        <v>1050</v>
+        <v>1021</v>
       </c>
       <c r="B196" s="1" t="n">
-        <v>1120</v>
+        <v>1058</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>1366</v>
+        <v>1361</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
       <c r="E196" s="10" t="s">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="J196" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K196" s="2" t="s">
-        <v>397</v>
+        <v>1364</v>
       </c>
       <c r="L196" s="2" t="s">
-        <v>1369</v>
+        <v>1330</v>
       </c>
       <c r="M196" s="2" t="s">
-        <v>1370</v>
+        <v>1365</v>
       </c>
       <c r="N196" s="1" t="s">
         <v>400</v>
@@ -15452,34 +15463,37 @@
       <c r="O196" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P196" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="1" t="n">
-        <v>1075</v>
+        <v>1050</v>
       </c>
       <c r="B197" s="1" t="n">
-        <v>1141</v>
+        <v>1120</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
       <c r="E197" s="10" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="J197" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K197" s="2" t="s">
-        <v>742</v>
+        <v>397</v>
       </c>
       <c r="L197" s="2" t="s">
-        <v>1374</v>
+        <v>1369</v>
       </c>
       <c r="M197" s="2" t="s">
-        <v>1375</v>
+        <v>1370</v>
       </c>
       <c r="N197" s="1" t="s">
         <v>400</v>
@@ -15487,37 +15501,34 @@
       <c r="O197" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P197" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="1" t="n">
-        <v>1092</v>
+        <v>1075</v>
       </c>
       <c r="B198" s="1" t="n">
-        <v>1167</v>
+        <v>1141</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>1376</v>
+        <v>1371</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>1377</v>
+        <v>1372</v>
       </c>
       <c r="E198" s="10" t="s">
-        <v>1378</v>
+        <v>1373</v>
       </c>
       <c r="J198" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K198" s="2" t="s">
-        <v>546</v>
+        <v>742</v>
       </c>
       <c r="L198" s="2" t="s">
-        <v>1330</v>
+        <v>1374</v>
       </c>
       <c r="M198" s="2" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
       <c r="N198" s="1" t="s">
         <v>400</v>
@@ -15525,34 +15536,37 @@
       <c r="O198" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P198" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="1" t="n">
-        <v>1110</v>
+        <v>1092</v>
       </c>
       <c r="B199" s="1" t="n">
-        <v>1180</v>
+        <v>1167</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
       <c r="E199" s="10" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="J199" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K199" s="2" t="s">
-        <v>206</v>
+        <v>546</v>
       </c>
       <c r="L199" s="2" t="s">
-        <v>1383</v>
+        <v>1330</v>
       </c>
       <c r="M199" s="2" t="s">
-        <v>1384</v>
+        <v>1379</v>
       </c>
       <c r="N199" s="1" t="s">
         <v>400</v>
@@ -15563,31 +15577,34 @@
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="1" t="n">
-        <v>1150</v>
+        <v>1110</v>
       </c>
       <c r="B200" s="1" t="n">
-        <v>1210</v>
+        <v>1180</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>1385</v>
+        <v>1380</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>1386</v>
+        <v>1381</v>
       </c>
       <c r="E200" s="10" t="s">
-        <v>1387</v>
+        <v>1382</v>
       </c>
       <c r="J200" s="1" t="s">
-        <v>147</v>
+        <v>396</v>
       </c>
       <c r="K200" s="2" t="s">
-        <v>1388</v>
+        <v>206</v>
       </c>
       <c r="L200" s="2" t="s">
-        <v>1340</v>
+        <v>1383</v>
       </c>
       <c r="M200" s="2" t="s">
-        <v>1389</v>
+        <v>1384</v>
+      </c>
+      <c r="N200" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="O200" s="1" t="s">
         <v>401</v>
@@ -15595,36 +15612,31 @@
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="1" t="n">
-        <v>1194</v>
+        <v>1150</v>
       </c>
       <c r="B201" s="1" t="n">
-        <v>1270</v>
+        <v>1210</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>1390</v>
+        <v>1385</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>1391</v>
+        <v>1386</v>
       </c>
       <c r="E201" s="10" t="s">
-        <v>1392</v>
+        <v>1387</v>
       </c>
       <c r="J201" s="1" t="s">
-        <v>396</v>
+        <v>147</v>
       </c>
       <c r="K201" s="2" t="s">
-        <v>791</v>
-      </c>
-      <c r="L201" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Philosophie juive médiévale ; Mysticisme ; Kabbale</t>
-        </is>
+        <v>1388</v>
+      </c>
+      <c r="L201" s="2" t="s">
+        <v>1340</v>
       </c>
       <c r="M201" s="2" t="s">
-        <v>1393</v>
-      </c>
-      <c r="N201" s="1" t="s">
-        <v>1394</v>
+        <v>1389</v>
       </c>
       <c r="O201" s="1" t="s">
         <v>401</v>
@@ -15632,101 +15644,103 @@
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="1" t="n">
-        <v>1263</v>
+        <v>1194</v>
       </c>
       <c r="B202" s="1" t="n">
-        <v>1328</v>
+        <v>1270</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>1395</v>
+        <v>1390</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>1396</v>
+        <v>1391</v>
       </c>
       <c r="E202" s="10" t="s">
-        <v>1397</v>
+        <v>1392</v>
       </c>
       <c r="J202" s="1" t="s">
-        <v>545</v>
+        <v>396</v>
       </c>
       <c r="K202" s="2" t="s">
-        <v>1398</v>
-      </c>
-      <c r="L202" s="2" t="s">
-        <v>1399</v>
+        <v>791</v>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie juive médiévale ; Mysticisme ; Kabbale</t>
+        </is>
       </c>
       <c r="M202" s="2" t="s">
-        <v>1400</v>
+        <v>1393</v>
+      </c>
+      <c r="N202" s="1" t="s">
+        <v>1394</v>
       </c>
       <c r="O202" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P202" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="1" t="n">
-        <v>1380</v>
+        <v>1263</v>
       </c>
       <c r="B203" s="1" t="n">
-        <v>1444</v>
+        <v>1328</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>1405</v>
+        <v>1395</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>1406</v>
+        <v>1396</v>
       </c>
       <c r="E203" s="10" t="s">
-        <v>1407</v>
+        <v>1397</v>
       </c>
       <c r="J203" s="1" t="s">
-        <v>396</v>
+        <v>545</v>
       </c>
       <c r="K203" s="2" t="s">
-        <v>1408</v>
+        <v>1398</v>
       </c>
       <c r="L203" s="2" t="s">
-        <v>1374</v>
+        <v>1399</v>
       </c>
       <c r="M203" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="N203" s="1" t="s">
-        <v>1394</v>
+        <v>1400</v>
       </c>
       <c r="O203" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P203" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="1" t="n">
-        <v>1437</v>
+        <v>1380</v>
       </c>
       <c r="B204" s="1" t="n">
-        <v>1508</v>
+        <v>1444</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>1410</v>
+        <v>1405</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>1411</v>
+        <v>1406</v>
       </c>
       <c r="E204" s="10" t="s">
-        <v>1412</v>
+        <v>1407</v>
       </c>
       <c r="J204" s="1" t="s">
         <v>396</v>
       </c>
       <c r="K204" s="2" t="s">
-        <v>1043</v>
+        <v>1408</v>
       </c>
       <c r="L204" s="2" t="s">
-        <v>1413</v>
+        <v>1374</v>
       </c>
       <c r="M204" s="2" t="s">
-        <v>1414</v>
+        <v>1409</v>
       </c>
       <c r="N204" s="1" t="s">
         <v>1394</v>
@@ -15737,33 +15751,34 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="1" t="n">
-        <v>1561</v>
+        <v>1437</v>
       </c>
       <c r="B205" s="1" t="n">
-        <v>1631</v>
+        <v>1508</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>1415</v>
+        <v>1410</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>1416</v>
+        <v>1411</v>
       </c>
       <c r="E205" s="10" t="s">
-        <v>1417</v>
+        <v>1412</v>
       </c>
       <c r="J205" s="1" t="s">
-        <v>147</v>
+        <v>396</v>
       </c>
       <c r="K205" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="L205" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ishraqisme ; École d'Ispahan</t>
-        </is>
+        <v>1043</v>
+      </c>
+      <c r="L205" s="2" t="s">
+        <v>1413</v>
       </c>
       <c r="M205" s="2" t="s">
-        <v>1418</v>
+        <v>1414</v>
+      </c>
+      <c r="N205" s="1" t="s">
+        <v>1394</v>
       </c>
       <c r="O205" s="1" t="s">
         <v>401</v>
@@ -15771,136 +15786,135 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="1" t="n">
-        <v>1801</v>
+        <v>1561</v>
       </c>
       <c r="B206" s="1" t="n">
-        <v>1873</v>
+        <v>1631</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="E206" s="10" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
       <c r="J206" s="1" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="K206" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="L206" s="2" t="s">
-        <v>1422</v>
+        <v>206</v>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ishraqisme ; École d'Ispahan</t>
+        </is>
       </c>
       <c r="M206" s="2" t="s">
-        <v>1423</v>
+        <v>1418</v>
       </c>
       <c r="O206" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="P206" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="1" t="n">
-        <v>1849</v>
+        <v>1801</v>
       </c>
       <c r="B207" s="1" t="n">
-        <v>1905</v>
+        <v>1873</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>1424</v>
+        <v>1419</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>1425</v>
+        <v>1420</v>
       </c>
       <c r="E207" s="10" t="s">
-        <v>1426</v>
+        <v>1421</v>
       </c>
       <c r="J207" s="1" t="s">
         <v>25</v>
       </c>
       <c r="K207" s="2" t="s">
-        <v>1408</v>
+        <v>304</v>
       </c>
       <c r="L207" s="2" t="s">
-        <v>1427</v>
+        <v>1422</v>
       </c>
       <c r="M207" s="2" t="s">
-        <v>1428</v>
+        <v>1423</v>
       </c>
       <c r="O207" s="1" t="s">
         <v>401</v>
       </c>
       <c r="P207" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="1" t="n">
-        <v>1888</v>
+        <v>1849</v>
       </c>
       <c r="B208" s="1" t="n">
-        <v>1966</v>
+        <v>1905</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>1429</v>
+        <v>1424</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>1430</v>
+        <v>1425</v>
       </c>
       <c r="E208" s="10" t="s">
-        <v>1431</v>
+        <v>1426</v>
       </c>
       <c r="J208" s="1" t="s">
         <v>25</v>
       </c>
       <c r="K208" s="2" t="s">
-        <v>304</v>
+        <v>1408</v>
       </c>
       <c r="L208" s="2" t="s">
-        <v>1422</v>
+        <v>1427</v>
       </c>
       <c r="M208" s="2" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="O208" s="1" t="s">
         <v>401</v>
       </c>
+      <c r="P208" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="1" t="n">
-        <v>1905</v>
+        <v>1888</v>
       </c>
       <c r="B209" s="1" t="n">
-        <v>1973</v>
+        <v>1966</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="E209" s="10" t="s">
-        <v>1435</v>
+        <v>1431</v>
       </c>
       <c r="J209" s="1" t="s">
-        <v>1436</v>
+        <v>25</v>
       </c>
       <c r="K209" s="2" t="s">
         <v>304</v>
       </c>
       <c r="L209" s="2" t="s">
-        <v>1259</v>
+        <v>1422</v>
       </c>
       <c r="M209" s="2" t="s">
-        <v>1437</v>
-      </c>
-      <c r="N209" s="1" t="s">
-        <v>660</v>
+        <v>1432</v>
       </c>
       <c r="O209" s="1" t="s">
         <v>401</v>
@@ -15908,31 +15922,34 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="1" t="n">
-        <v>1935</v>
+        <v>1905</v>
       </c>
       <c r="B210" s="1" t="n">
-        <v>2021</v>
+        <v>1973</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>1448</v>
+        <v>1433</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>1449</v>
+        <v>1434</v>
       </c>
       <c r="E210" s="10" t="s">
-        <v>1450</v>
+        <v>1435</v>
       </c>
       <c r="J210" s="1" t="s">
-        <v>25</v>
+        <v>1436</v>
       </c>
       <c r="K210" s="2" t="s">
-        <v>1043</v>
+        <v>304</v>
       </c>
       <c r="L210" s="2" t="s">
-        <v>1451</v>
+        <v>1259</v>
       </c>
       <c r="M210" s="2" t="s">
-        <v>1452</v>
+        <v>1437</v>
+      </c>
+      <c r="N210" s="1" t="s">
+        <v>660</v>
       </c>
       <c r="O210" s="1" t="s">
         <v>401</v>
@@ -15940,95 +15957,89 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="1" t="n">
-        <v>613</v>
+        <v>1935</v>
       </c>
       <c r="B211" s="1" t="n">
-        <v>696</v>
+        <v>2021</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>1464</v>
+        <v>1448</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>1465</v>
+        <v>1449</v>
       </c>
       <c r="E211" s="10" t="s">
-        <v>1466</v>
-      </c>
-      <c r="H211" s="2" t="s">
-        <v>1467</v>
+        <v>1450</v>
       </c>
       <c r="J211" s="1" t="s">
-        <v>916</v>
+        <v>25</v>
       </c>
       <c r="K211" s="2" t="s">
-        <v>231</v>
+        <v>1043</v>
       </c>
       <c r="L211" s="2" t="s">
-        <v>444</v>
+        <v>1451</v>
       </c>
       <c r="M211" s="2" t="s">
-        <v>1468</v>
+        <v>1452</v>
       </c>
       <c r="O211" s="1" t="s">
-        <v>271</v>
+        <v>401</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="1" t="n">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="B212" s="1" t="n">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>1469</v>
+        <v>1464</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>1470</v>
+        <v>1465</v>
       </c>
       <c r="E212" s="10" t="s">
-        <v>1471</v>
+        <v>1466</v>
       </c>
       <c r="H212" s="2" t="s">
-        <v>1472</v>
+        <v>1467</v>
       </c>
       <c r="J212" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K212" s="2" t="s">
-        <v>206</v>
+        <v>231</v>
       </c>
       <c r="L212" s="2" t="s">
         <v>444</v>
       </c>
       <c r="M212" s="2" t="s">
-        <v>1473</v>
+        <v>1468</v>
       </c>
       <c r="O212" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P212" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="1" t="n">
-        <v>625</v>
+        <v>617</v>
       </c>
       <c r="B213" s="1" t="n">
-        <v>702</v>
+        <v>686</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>1474</v>
+        <v>1469</v>
       </c>
       <c r="D213" s="2" t="s">
-        <v>1475</v>
+        <v>1470</v>
       </c>
       <c r="E213" s="10" t="s">
-        <v>1476</v>
+        <v>1471</v>
       </c>
       <c r="H213" s="2" t="s">
-        <v>1477</v>
+        <v>1472</v>
       </c>
       <c r="J213" s="1" t="s">
         <v>916</v>
@@ -16036,48 +16047,51 @@
       <c r="K213" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="L213" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhisme Mahayana ; Huayan</t>
-        </is>
+      <c r="L213" s="2" t="s">
+        <v>444</v>
       </c>
       <c r="M213" s="2" t="s">
-        <v>1478</v>
+        <v>1473</v>
       </c>
       <c r="O213" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P213" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="1" t="n">
-        <v>857</v>
+        <v>625</v>
       </c>
       <c r="B214" s="1" t="n">
-        <v>910</v>
+        <v>702</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>1479</v>
+        <v>1474</v>
       </c>
       <c r="D214" s="2" t="s">
-        <v>1480</v>
+        <v>1475</v>
       </c>
       <c r="E214" s="10" t="s">
-        <v>1481</v>
+        <v>1476</v>
       </c>
       <c r="H214" s="2" t="s">
-        <v>1482</v>
+        <v>1477</v>
       </c>
       <c r="J214" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K214" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="L214" s="2" t="s">
-        <v>917</v>
+        <v>206</v>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme Mahayana ; Huayan</t>
+        </is>
       </c>
       <c r="M214" s="2" t="s">
-        <v>1483</v>
+        <v>1478</v>
       </c>
       <c r="O214" s="1" t="s">
         <v>271</v>
@@ -16085,34 +16099,34 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="1" t="n">
-        <v>1055</v>
+        <v>857</v>
       </c>
       <c r="B215" s="1" t="n">
-        <v>1101</v>
+        <v>910</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>1484</v>
+        <v>1479</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>1485</v>
+        <v>1480</v>
       </c>
       <c r="E215" s="10" t="s">
-        <v>1486</v>
+        <v>1481</v>
       </c>
       <c r="H215" s="2" t="s">
-        <v>1487</v>
+        <v>1482</v>
       </c>
       <c r="J215" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K215" s="2" t="s">
-        <v>546</v>
+        <v>397</v>
       </c>
       <c r="L215" s="2" t="s">
-        <v>444</v>
+        <v>917</v>
       </c>
       <c r="M215" s="2" t="s">
-        <v>1488</v>
+        <v>1483</v>
       </c>
       <c r="O215" s="1" t="s">
         <v>271</v>
@@ -16120,22 +16134,22 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="1" t="n">
-        <v>1158</v>
+        <v>1055</v>
       </c>
       <c r="B216" s="1" t="n">
-        <v>1210</v>
+        <v>1101</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>1489</v>
+        <v>1484</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>1490</v>
+        <v>1485</v>
       </c>
       <c r="E216" s="10" t="s">
-        <v>1491</v>
+        <v>1486</v>
       </c>
       <c r="H216" s="2" t="s">
-        <v>1492</v>
+        <v>1487</v>
       </c>
       <c r="J216" s="1" t="s">
         <v>916</v>
@@ -16144,10 +16158,10 @@
         <v>546</v>
       </c>
       <c r="L216" s="2" t="s">
-        <v>799</v>
+        <v>444</v>
       </c>
       <c r="M216" s="2" t="s">
-        <v>1493</v>
+        <v>1488</v>
       </c>
       <c r="O216" s="1" t="s">
         <v>271</v>
@@ -16155,72 +16169,69 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="1" t="n">
-        <v>1337</v>
+        <v>1158</v>
       </c>
       <c r="B217" s="1" t="n">
-        <v>1392</v>
+        <v>1210</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>1494</v>
+        <v>1489</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>1495</v>
+        <v>1490</v>
       </c>
       <c r="E217" s="10" t="s">
-        <v>1496</v>
+        <v>1491</v>
       </c>
       <c r="H217" s="2" t="s">
-        <v>1497</v>
+        <v>1492</v>
       </c>
       <c r="J217" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K217" s="2" t="s">
-        <v>62</v>
+        <v>546</v>
       </c>
       <c r="L217" s="2" t="s">
-        <v>917</v>
+        <v>799</v>
       </c>
       <c r="M217" s="2" t="s">
-        <v>1498</v>
+        <v>1493</v>
       </c>
       <c r="O217" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P217" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="1" t="n">
-        <v>1342</v>
+        <v>1337</v>
       </c>
       <c r="B218" s="1" t="n">
-        <v>1398</v>
+        <v>1392</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>1499</v>
+        <v>1494</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>1500</v>
+        <v>1495</v>
       </c>
       <c r="E218" s="10" t="s">
-        <v>1501</v>
+        <v>1496</v>
       </c>
       <c r="H218" s="2" t="s">
-        <v>1502</v>
+        <v>1497</v>
       </c>
       <c r="J218" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K218" s="2" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="L218" s="2" t="s">
         <v>917</v>
       </c>
       <c r="M218" s="2" t="s">
-        <v>1503</v>
+        <v>1498</v>
       </c>
       <c r="O218" s="1" t="s">
         <v>271</v>
@@ -16231,69 +16242,72 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="1" t="n">
-        <v>1376</v>
+        <v>1342</v>
       </c>
       <c r="B219" s="1" t="n">
-        <v>1433</v>
+        <v>1398</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>1504</v>
+        <v>1499</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>1505</v>
+        <v>1500</v>
       </c>
       <c r="E219" s="10" t="s">
-        <v>1506</v>
+        <v>1501</v>
       </c>
       <c r="H219" s="2" t="s">
-        <v>1507</v>
+        <v>1502</v>
       </c>
       <c r="J219" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K219" s="2" t="s">
-        <v>427</v>
+        <v>80</v>
       </c>
       <c r="L219" s="2" t="s">
-        <v>799</v>
+        <v>917</v>
       </c>
       <c r="M219" s="2" t="s">
-        <v>1508</v>
+        <v>1503</v>
       </c>
       <c r="O219" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P219" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="1" t="n">
-        <v>1489</v>
+        <v>1376</v>
       </c>
       <c r="B220" s="1" t="n">
-        <v>1546</v>
+        <v>1433</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>1514</v>
+        <v>1504</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>1515</v>
+        <v>1505</v>
       </c>
       <c r="E220" s="10" t="s">
-        <v>1516</v>
+        <v>1506</v>
       </c>
       <c r="H220" s="2" t="s">
-        <v>1517</v>
+        <v>1507</v>
       </c>
       <c r="J220" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K220" s="2" t="s">
-        <v>231</v>
+        <v>427</v>
       </c>
       <c r="L220" s="2" t="s">
-        <v>917</v>
+        <v>799</v>
       </c>
       <c r="M220" s="2" t="s">
-        <v>1518</v>
+        <v>1508</v>
       </c>
       <c r="O220" s="1" t="s">
         <v>271</v>
@@ -16301,34 +16315,34 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="1" t="n">
-        <v>1501</v>
+        <v>1489</v>
       </c>
       <c r="B221" s="1" t="n">
-        <v>1572</v>
+        <v>1546</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>1519</v>
+        <v>1514</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>1520</v>
+        <v>1515</v>
       </c>
       <c r="E221" s="10" t="s">
-        <v>1521</v>
+        <v>1516</v>
       </c>
       <c r="H221" s="2" t="s">
-        <v>1522</v>
+        <v>1517</v>
       </c>
       <c r="J221" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K221" s="2" t="s">
-        <v>62</v>
+        <v>231</v>
       </c>
       <c r="L221" s="2" t="s">
         <v>917</v>
       </c>
       <c r="M221" s="2" t="s">
-        <v>1523</v>
+        <v>1518</v>
       </c>
       <c r="O221" s="1" t="s">
         <v>271</v>
@@ -16336,34 +16350,34 @@
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="1" t="n">
+        <v>1501</v>
+      </c>
+      <c r="B222" s="1" t="n">
+        <v>1572</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>1519</v>
+      </c>
+      <c r="D222" s="2" t="s">
         <v>1520</v>
       </c>
-      <c r="B222" s="1" t="n">
-        <v>1604</v>
-      </c>
-      <c r="C222" s="2" t="s">
-        <v>1524</v>
-      </c>
-      <c r="D222" s="2" t="s">
-        <v>1525</v>
-      </c>
       <c r="E222" s="10" t="s">
-        <v>1526</v>
+        <v>1521</v>
       </c>
       <c r="H222" s="2" t="s">
-        <v>1527</v>
+        <v>1522</v>
       </c>
       <c r="J222" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K222" s="2" t="s">
-        <v>427</v>
+        <v>62</v>
       </c>
       <c r="L222" s="2" t="s">
-        <v>799</v>
+        <v>917</v>
       </c>
       <c r="M222" s="2" t="s">
-        <v>1528</v>
+        <v>1523</v>
       </c>
       <c r="O222" s="1" t="s">
         <v>271</v>
@@ -16371,34 +16385,34 @@
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="1" t="n">
+        <v>1520</v>
+      </c>
+      <c r="B223" s="1" t="n">
+        <v>1604</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>1524</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>1525</v>
+      </c>
+      <c r="E223" s="10" t="s">
+        <v>1526</v>
+      </c>
+      <c r="H223" s="2" t="s">
         <v>1527</v>
-      </c>
-      <c r="B223" s="1" t="n">
-        <v>1572</v>
-      </c>
-      <c r="C223" s="2" t="s">
-        <v>1529</v>
-      </c>
-      <c r="D223" s="2" t="s">
-        <v>1530</v>
-      </c>
-      <c r="E223" s="10" t="s">
-        <v>1531</v>
-      </c>
-      <c r="H223" s="2" t="s">
-        <v>1532</v>
       </c>
       <c r="J223" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K223" s="2" t="s">
-        <v>257</v>
+        <v>427</v>
       </c>
       <c r="L223" s="2" t="s">
-        <v>917</v>
+        <v>799</v>
       </c>
       <c r="M223" s="2" t="s">
-        <v>1533</v>
+        <v>1528</v>
       </c>
       <c r="O223" s="1" t="s">
         <v>271</v>
@@ -16406,24 +16420,22 @@
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="1" t="n">
-        <v>1535</v>
+        <v>1527</v>
       </c>
       <c r="B224" s="1" t="n">
-        <v>1598</v>
+        <v>1572</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>1534</v>
+        <v>1529</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>1535</v>
-      </c>
-      <c r="E224" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/S%C5%8Fng_Hon"  title=" Wikipedia (en)"&gt;SEONG HON&lt;/a&gt;, dit Ugye, était un lettré néoconfucéen, ami de Yi I, qui passa l’essentiel de sa vie à enseigner à l’écart de la cour, dans la région de Paju. Il refusa presque toutes les charges que la cour lui offrait.&lt;/p&gt; &lt;p&gt;À partir de 1572, il relança avec Yi I le débat des Quatre et des Sept, en prenant cette fois le parti de Yi Hwang : il défendait que les sentiments moraux et les émotions ordinaires ont des sources distinctes, et que l’« esprit humain » ne se confond pas avec l’« esprit de la Voie ». Ces échanges obligèrent Yi I à préciser sa propre théorie. Pour Yi I, au contraire, seule l’énergie matérielle (&lt;em&gt;gi&lt;/em&gt;) se met en mouvement, et le principe (&lt;em&gt;i&lt;/em&gt;) la guide sans agir lui-même. Ses disciples contribuèrent ensuite à la formation de la faction de l’Ouest (Seoin), dont il est considéré comme l’un des maîtres.&lt;/p&gt; &lt;p&gt;Fils de Seong Su-chim, un disciple de Jo Gwang-jo qui s’était retiré après la purge de 1519, il hérita de son père le refus des honneurs et la priorité donnée à la culture de soi. Ses lettres avec Yi I forment, après celles de Yi Hwang et de Gi Dae-seung, la seconde grande correspondance du débat des Quatre et des Sept. Pendant la guerre de 1592, il rejoignit le prince héritier, mais on lui reprocha de ne pas être venu saluer le roi lors de sa fuite vers le nord, et la faction du Nord fit plus tard retirer ses titres posthumes. Réhabilité, il entra en 1681, en même temps que Yi I, dans le sanctuaire de Confucius, signe de l’influence durable de son école sur la vie intellectuelle de Joseon.&lt;/p&gt;</t>
-        </is>
+        <v>1530</v>
+      </c>
+      <c r="E224" s="10" t="s">
+        <v>1531</v>
       </c>
       <c r="H224" s="2" t="s">
-        <v>1537</v>
+        <v>1532</v>
       </c>
       <c r="J224" s="1" t="s">
         <v>916</v>
@@ -16435,7 +16447,7 @@
         <v>917</v>
       </c>
       <c r="M224" s="2" t="s">
-        <v>1538</v>
+        <v>1533</v>
       </c>
       <c r="O224" s="1" t="s">
         <v>271</v>
@@ -16443,98 +16455,97 @@
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="1" t="n">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="B225" s="1" t="n">
-        <v>1584</v>
+        <v>1598</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>1539</v>
+        <v>1534</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>1540</v>
-      </c>
-      <c r="E225" s="10" t="s">
-        <v>1541</v>
+        <v>1535</v>
+      </c>
+      <c r="E225" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/S%C5%8Fng_Hon"  title=" Wikipedia (en)"&gt;SEONG HON&lt;/a&gt;, dit Ugye, était un lettré néoconfucéen, ami de Yi I, qui passa l’essentiel de sa vie à enseigner à l’écart de la cour, dans la région de Paju. Il refusa presque toutes les charges que la cour lui offrait.&lt;/p&gt; &lt;p&gt;À partir de 1572, il relança avec Yi I le débat des Quatre et des Sept, en prenant cette fois le parti de Yi Hwang : il défendait que les sentiments moraux et les émotions ordinaires ont des sources distinctes, et que l’« esprit humain » ne se confond pas avec l’« esprit de la Voie ». Ces échanges obligèrent Yi I à préciser sa propre théorie. Pour Yi I, au contraire, seule l’énergie matérielle (&lt;em&gt;gi&lt;/em&gt;) se met en mouvement, et le principe (&lt;em&gt;i&lt;/em&gt;) la guide sans agir lui-même. Ses disciples contribuèrent ensuite à la formation de la faction de l’Ouest (Seoin), dont il est considéré comme l’un des maîtres.&lt;/p&gt; &lt;p&gt;Fils de Seong Su-chim, un disciple de Jo Gwang-jo qui s’était retiré après la purge de 1519, il hérita de son père le refus des honneurs et la priorité donnée à la culture de soi. Ses lettres avec Yi I forment, après celles de Yi Hwang et de Gi Dae-seung, la seconde grande correspondance du débat des Quatre et des Sept. Pendant la guerre de 1592, il rejoignit le prince héritier, mais on lui reprocha de ne pas être venu saluer le roi lors de sa fuite vers le nord, et la faction du Nord fit plus tard retirer ses titres posthumes. Réhabilité, il entra en 1681, en même temps que Yi I, dans le sanctuaire de Confucius, signe de l’influence durable de son école sur la vie intellectuelle de Joseon.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="H225" s="2" t="s">
-        <v>1542</v>
+        <v>1537</v>
       </c>
       <c r="J225" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K225" s="2" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="L225" s="2" t="s">
         <v>917</v>
       </c>
       <c r="M225" s="2" t="s">
-        <v>1543</v>
+        <v>1538</v>
       </c>
       <c r="O225" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P225" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="1" t="n">
-        <v>1607</v>
+        <v>1536</v>
       </c>
       <c r="B226" s="1" t="n">
-        <v>1689</v>
+        <v>1584</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>1544</v>
+        <v>1539</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>1545</v>
+        <v>1540</v>
       </c>
       <c r="E226" s="10" t="s">
-        <v>1546</v>
+        <v>1541</v>
       </c>
       <c r="H226" s="2" t="s">
-        <v>1547</v>
+        <v>1542</v>
       </c>
       <c r="J226" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K226" s="2" t="s">
-        <v>80</v>
+        <v>268</v>
       </c>
       <c r="L226" s="2" t="s">
         <v>917</v>
       </c>
       <c r="M226" s="2" t="s">
-        <v>1548</v>
+        <v>1543</v>
       </c>
       <c r="O226" s="1" t="s">
         <v>271</v>
       </c>
       <c r="P226" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="1" t="n">
-        <v>1622</v>
+        <v>1607</v>
       </c>
       <c r="B227" s="1" t="n">
-        <v>1673</v>
+        <v>1689</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>1549</v>
+        <v>1544</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>1550</v>
+        <v>1545</v>
       </c>
       <c r="E227" s="10" t="s">
-        <v>1551</v>
+        <v>1546</v>
       </c>
       <c r="H227" s="2" t="s">
-        <v>1552</v>
+        <v>1547</v>
       </c>
       <c r="J227" s="1" t="s">
         <v>916</v>
@@ -16543,118 +16554,121 @@
         <v>80</v>
       </c>
       <c r="L227" s="2" t="s">
-        <v>992</v>
+        <v>917</v>
       </c>
       <c r="M227" s="2" t="s">
-        <v>1553</v>
+        <v>1548</v>
       </c>
       <c r="O227" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P227" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="1" t="n">
-        <v>1649</v>
+        <v>1622</v>
       </c>
       <c r="B228" s="1" t="n">
-        <v>1736</v>
+        <v>1673</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>1554</v>
+        <v>1549</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>1555</v>
+        <v>1550</v>
       </c>
       <c r="E228" s="10" t="s">
-        <v>1556</v>
+        <v>1551</v>
       </c>
       <c r="H228" s="2" t="s">
-        <v>1557</v>
+        <v>1552</v>
       </c>
       <c r="J228" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K228" s="2" t="s">
-        <v>951</v>
+        <v>80</v>
       </c>
       <c r="L228" s="2" t="s">
-        <v>691</v>
+        <v>992</v>
       </c>
       <c r="M228" s="2" t="s">
-        <v>1558</v>
+        <v>1553</v>
       </c>
       <c r="O228" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P228" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="1" t="n">
-        <v>1682</v>
+        <v>1649</v>
       </c>
       <c r="B229" s="1" t="n">
-        <v>1751</v>
+        <v>1736</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>1559</v>
+        <v>1554</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>1560</v>
+        <v>1555</v>
       </c>
       <c r="E229" s="10" t="s">
-        <v>1561</v>
+        <v>1556</v>
       </c>
       <c r="H229" s="2" t="s">
-        <v>1562</v>
+        <v>1557</v>
       </c>
       <c r="J229" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K229" s="2" t="s">
-        <v>247</v>
+        <v>951</v>
       </c>
       <c r="L229" s="2" t="s">
-        <v>917</v>
+        <v>691</v>
       </c>
       <c r="M229" s="2" t="s">
-        <v>1563</v>
+        <v>1558</v>
       </c>
       <c r="O229" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P229" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="1" t="n">
-        <v>1731</v>
+        <v>1682</v>
       </c>
       <c r="B230" s="1" t="n">
-        <v>1783</v>
+        <v>1751</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>1564</v>
+        <v>1559</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>1565</v>
+        <v>1560</v>
       </c>
       <c r="E230" s="10" t="s">
-        <v>1566</v>
+        <v>1561</v>
       </c>
       <c r="H230" s="2" t="s">
-        <v>1567</v>
+        <v>1562</v>
       </c>
       <c r="J230" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K230" s="2" t="s">
-        <v>409</v>
+        <v>247</v>
       </c>
       <c r="L230" s="2" t="s">
-        <v>992</v>
+        <v>917</v>
       </c>
       <c r="M230" s="2" t="s">
-        <v>1568</v>
+        <v>1563</v>
       </c>
       <c r="O230" s="1" t="s">
         <v>271</v>
@@ -16662,34 +16676,34 @@
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="1" t="n">
-        <v>1737</v>
+        <v>1731</v>
       </c>
       <c r="B231" s="1" t="n">
-        <v>1805</v>
+        <v>1783</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>1569</v>
+        <v>1564</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>1570</v>
+        <v>1565</v>
       </c>
       <c r="E231" s="10" t="s">
-        <v>1571</v>
+        <v>1566</v>
       </c>
       <c r="H231" s="2" t="s">
-        <v>1572</v>
+        <v>1567</v>
       </c>
       <c r="J231" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K231" s="2" t="s">
-        <v>1159</v>
+        <v>409</v>
       </c>
       <c r="L231" s="2" t="s">
         <v>992</v>
       </c>
       <c r="M231" s="2" t="s">
-        <v>1573</v>
+        <v>1568</v>
       </c>
       <c r="O231" s="1" t="s">
         <v>271</v>
@@ -16697,107 +16711,107 @@
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="1" t="n">
-        <v>1762</v>
+        <v>1737</v>
       </c>
       <c r="B232" s="1" t="n">
-        <v>1836</v>
+        <v>1805</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>1574</v>
+        <v>1569</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>1575</v>
+        <v>1570</v>
       </c>
       <c r="E232" s="10" t="s">
-        <v>1576</v>
+        <v>1571</v>
       </c>
       <c r="H232" s="2" t="s">
-        <v>1577</v>
+        <v>1572</v>
       </c>
       <c r="J232" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K232" s="2" t="s">
-        <v>80</v>
+        <v>1159</v>
       </c>
       <c r="L232" s="2" t="s">
         <v>992</v>
       </c>
       <c r="M232" s="2" t="s">
-        <v>1578</v>
+        <v>1573</v>
       </c>
       <c r="O232" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P232" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="1" t="n">
-        <v>1792</v>
+        <v>1762</v>
       </c>
       <c r="B233" s="1" t="n">
-        <v>1868</v>
+        <v>1836</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>1579</v>
+        <v>1574</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>1580</v>
+        <v>1575</v>
       </c>
       <c r="E233" s="10" t="s">
-        <v>1581</v>
+        <v>1576</v>
       </c>
       <c r="H233" s="2" t="s">
-        <v>1582</v>
+        <v>1577</v>
       </c>
       <c r="J233" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K233" s="2" t="s">
-        <v>387</v>
+        <v>80</v>
       </c>
       <c r="L233" s="2" t="s">
-        <v>917</v>
+        <v>992</v>
       </c>
       <c r="M233" s="2" t="s">
-        <v>1583</v>
+        <v>1578</v>
       </c>
       <c r="O233" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P233" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="1" t="n">
-        <v>1803</v>
+        <v>1792</v>
       </c>
       <c r="B234" s="1" t="n">
-        <v>1877</v>
+        <v>1868</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>1584</v>
+        <v>1579</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>1585</v>
+        <v>1580</v>
       </c>
       <c r="E234" s="10" t="s">
-        <v>1586</v>
+        <v>1581</v>
       </c>
       <c r="H234" s="2" t="s">
-        <v>1587</v>
+        <v>1582</v>
       </c>
       <c r="J234" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K234" s="2" t="s">
-        <v>409</v>
+        <v>387</v>
       </c>
       <c r="L234" s="2" t="s">
-        <v>992</v>
+        <v>917</v>
       </c>
       <c r="M234" s="2" t="s">
-        <v>1588</v>
+        <v>1583</v>
       </c>
       <c r="O234" s="1" t="s">
         <v>271</v>
@@ -16805,34 +16819,34 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="1" t="n">
-        <v>1824</v>
+        <v>1803</v>
       </c>
       <c r="B235" s="1" t="n">
-        <v>1864</v>
+        <v>1877</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>1589</v>
+        <v>1584</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>1590</v>
+        <v>1585</v>
       </c>
       <c r="E235" s="10" t="s">
-        <v>1591</v>
+        <v>1586</v>
       </c>
       <c r="H235" s="2" t="s">
-        <v>1592</v>
+        <v>1587</v>
       </c>
       <c r="J235" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K235" s="2" t="s">
-        <v>1408</v>
+        <v>409</v>
       </c>
       <c r="L235" s="2" t="s">
-        <v>1593</v>
+        <v>992</v>
       </c>
       <c r="M235" s="2" t="s">
-        <v>1594</v>
+        <v>1588</v>
       </c>
       <c r="O235" s="1" t="s">
         <v>271</v>
@@ -16840,34 +16854,34 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="1" t="n">
-        <v>1859</v>
+        <v>1824</v>
       </c>
       <c r="B236" s="1" t="n">
-        <v>1925</v>
+        <v>1864</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>1595</v>
+        <v>1589</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>1596</v>
+        <v>1590</v>
       </c>
       <c r="E236" s="10" t="s">
-        <v>1597</v>
+        <v>1591</v>
       </c>
       <c r="H236" s="2" t="s">
-        <v>1598</v>
+        <v>1592</v>
       </c>
       <c r="J236" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K236" s="2" t="s">
-        <v>80</v>
+        <v>1408</v>
       </c>
       <c r="L236" s="2" t="s">
-        <v>917</v>
+        <v>1593</v>
       </c>
       <c r="M236" s="2" t="s">
-        <v>1599</v>
+        <v>1594</v>
       </c>
       <c r="O236" s="1" t="s">
         <v>271</v>
@@ -16875,107 +16889,107 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="1" t="n">
-        <v>1879</v>
+        <v>1859</v>
       </c>
       <c r="B237" s="1" t="n">
-        <v>1944</v>
+        <v>1925</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>1600</v>
+        <v>1595</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>1601</v>
+        <v>1596</v>
       </c>
       <c r="E237" s="10" t="s">
-        <v>1602</v>
+        <v>1597</v>
       </c>
       <c r="H237" s="2" t="s">
-        <v>1603</v>
+        <v>1598</v>
       </c>
       <c r="J237" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K237" s="2" t="s">
-        <v>1408</v>
+        <v>80</v>
       </c>
       <c r="L237" s="2" t="s">
-        <v>799</v>
+        <v>917</v>
       </c>
       <c r="M237" s="2" t="s">
-        <v>1604</v>
+        <v>1599</v>
       </c>
       <c r="O237" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="P237" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="1" t="n">
-        <v>1880</v>
+        <v>1879</v>
       </c>
       <c r="B238" s="1" t="n">
-        <v>1936</v>
+        <v>1944</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>1605</v>
+        <v>1600</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>1606</v>
+        <v>1601</v>
       </c>
       <c r="E238" s="10" t="s">
-        <v>1607</v>
+        <v>1602</v>
       </c>
       <c r="H238" s="2" t="s">
-        <v>1608</v>
+        <v>1603</v>
       </c>
       <c r="J238" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K238" s="2" t="s">
-        <v>848</v>
+        <v>1408</v>
       </c>
       <c r="L238" s="2" t="s">
-        <v>1609</v>
+        <v>799</v>
       </c>
       <c r="M238" s="2" t="s">
-        <v>1610</v>
+        <v>1604</v>
       </c>
       <c r="O238" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="P238" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="1" t="n">
-        <v>1890</v>
+        <v>1880</v>
       </c>
       <c r="B239" s="1" t="n">
-        <v>1981</v>
+        <v>1936</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>1611</v>
+        <v>1605</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>1612</v>
+        <v>1606</v>
       </c>
       <c r="E239" s="10" t="s">
-        <v>1613</v>
+        <v>1607</v>
       </c>
       <c r="H239" s="2" t="s">
-        <v>1614</v>
+        <v>1608</v>
       </c>
       <c r="J239" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K239" s="2" t="s">
-        <v>138</v>
+        <v>848</v>
       </c>
       <c r="L239" s="2" t="s">
-        <v>1615</v>
+        <v>1609</v>
       </c>
       <c r="M239" s="2" t="s">
-        <v>1616</v>
+        <v>1610</v>
       </c>
       <c r="O239" s="1" t="s">
         <v>271</v>
@@ -16983,34 +16997,34 @@
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="1" t="n">
-        <v>1901</v>
+        <v>1890</v>
       </c>
       <c r="B240" s="1" t="n">
-        <v>1989</v>
+        <v>1981</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>1617</v>
+        <v>1611</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>1618</v>
+        <v>1612</v>
       </c>
       <c r="E240" s="10" t="s">
-        <v>1619</v>
+        <v>1613</v>
       </c>
       <c r="H240" s="2" t="s">
-        <v>1620</v>
+        <v>1614</v>
       </c>
       <c r="J240" s="1" t="s">
         <v>916</v>
       </c>
       <c r="K240" s="2" t="s">
-        <v>1408</v>
+        <v>138</v>
       </c>
       <c r="L240" s="2" t="s">
-        <v>1621</v>
+        <v>1615</v>
       </c>
       <c r="M240" s="2" t="s">
-        <v>1622</v>
+        <v>1616</v>
       </c>
       <c r="O240" s="1" t="s">
         <v>271</v>
@@ -21958,14 +21972,14 @@
     <hyperlink ref="E152" r:id="rId76" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Mohamed_Iqbal&quot; title=&quot;Wikipedia&quot;&gt;Muhammad IQBAL&lt;/a&gt; était un philosophe‑poète pakistanais, poète se plaçant à la croisée de l’islam, de la modernité et de la pensée occidentale. Considéré comme l’un des  &lt;a href=&quot;https://www.saphirnews.com/Mohammed-Iqbal-un-revolutionnaire-en-islam_a24652.html&quot; title=&quot;Mohamed Iqbal, un révolutionnaire en Islam par saphirnews&quot;&gt;grands penseurs musulmans &lt;/a&gt; de son époque, il cherche à réformer l’Islam en l’ouvrant à la rationalité et à l’action, tout en restant profondément enraciné dans la tradition soufie et coranique. &lt;/p&gt; &lt;p&gt; Sa philosophie tourne autour du « Khudi » (le Soi), c’est‑à‑dire une  &lt;a href=&quot;https://www.youtube.com/watch?v=ekC6_wffi10&quot; title=&quot;Mohamed Iqbal par Perennial Wisdom&quot;&gt;individualité spirituelle forte, &lt;/a&gt; capable de se libérer de toute passivité mystique et de toute soumission fataliste. Pour lui, l’homme n’est pas appelé à s’effacer dans un tout indifférencié, mais à affirmer son moi comme centre de liberté, de volonté et de responsabilité devant Dieu, en prolongeant ainsi la dynamique de la création. &lt;/p&gt; &lt;p&gt; Il  valorise aussi une lecture active et historique de l’Islam, où la loi et la pensée religieuse ne sont pas figées, mais appelées à se réinterpréter à la lumière de l’expérience humaine et du progrès. Il milite pour une société ouverte, où la foi se traduit par l’engagement, la justice, l’éducation et la dignité du travail, plutôt que par un rigorisme puritain ou un repli identitaire. &lt;/p&gt; &lt;p&gt; Il est souvent vu comme un penseur à la fois panislamiste et humaniste : il rêve d’une communauté musulmane unifiée, mais fondée sur la liberté intérieure, la créativité individuelle et le respect de la diversité humaine. Son œuvre, surtout poétique, mêle mystique et volonté de transformer le monde, ce qui fait de lui un des premiers philosophes à articuler Islam, modernité et affirmation de soi. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Iqbal : soufisme indo-pakistanais par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/11200-02.10.2011-ITEMA_20312518-2011C14958E0033-ITE_00045911_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
     <hyperlink ref="H156" r:id="rId77" display="https://www.laphilo.fr/pho/brambedkar-mini.webp"/>
     <hyperlink ref="E157" r:id="rId78" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jiddu_Krishnamurti&quot;  title=&quot;Wikipedia&quot;&gt;Jiddu KRISHNAMURTI&lt;/a&gt;  était  un penseur indien qui a profondément marqué la réflexion sur la liberté intérieure, la conscience et l’éducation.  &lt;a href=&quot;https://citations.ouest-france.fr/citations-jiddu-krishnamurti-1049.html&quot; title=&quot;Citations Krishnamurti par citations ouest france&quot;&gt;Sa parole &lt;/a&gt; est souvent résumée par l’idée que « la vérité est un pays sans chemins » : on ne peut pas atteindre le réel par l’autorité, le dogme, le rituel ou un système de pensée tout fait.  .&lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve la critique du conditionnement psychologique. Il explique que l’être humain vit prisonnier de ses peurs, de ses habitudes, de ses croyances et des images qu’il se fabrique sur lui-même et sur les autres ; pour lui, cette prison mentale empêche de voir clairement. &lt;/p&gt; &lt;p&gt; Il ne propose pas une  &lt;a href=&quot;https://www.youtube.com/watch?v=Uk3Kdoouw-E&quot; title=&quot;Perceptions Empties consciousness : Krishnamurti &quot;&gt;méthode au sens classique, &lt;/a&gt; ni un chemin spirituel à suivre mécaniquement. À la place, il invite à une observation directe de l’esprit, sans jugement et sans choix, qu’il associe à une forme de méditation véritable ; cette attention nue permettrait de comprendre la pensée en train de se faire et de se défaire. &lt;/p&gt; &lt;p&gt; Il relie toujours la transformation individuelle au changement du monde. Il pense qu’une société plus juste ne peut naître que d’une conscience intérieure libérée de l’autorité, de la violence psychologique et de la dépendance aux systèmes ; sa philosophie est donc moins une doctrine qu’un appel à voir par soi-même, ici et maintenant. &lt;/p&gt; &#10;&lt;audio controls title=&quot;Krishnamurti, une vie par France Culture&quot;&gt;&#10;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/14090-10.10.2014-ITEMA_20678757-2014C23018S0283-21.mp3&quot; type=&quot;audio/mpeg&quot;&gt;&#10;&lt;/audio&gt;"/>
-    <hyperlink ref="E162" r:id="rId79" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/L%C3%A9opold_S%C3%A9dar_Senghor&quot; title=&quot;Wikipedia&quot;&gt;Léopold Sédar SENGHOR&lt;/a&gt; était à la fois un grand poète-philosophe francophone et un homme d’État sénégalais, premier président de la République du Sénégal (1960–1980) et premier Africain membre de l’Académie française. Formé dans le système scolaire français, il incarne une figure hybride, à la croisée de l’Afrique et de la France, de la négritude et de la francophonie. &lt;/p&gt; &lt;p&gt; Au cœur de sa pensée se trouve le concept de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/N%C3%A9gritude&quot;  title=&quot;Négridude par Wikipedia&quot;&gt;« négritude », &lt;/a&gt; qu’il définit comme la reconnaissance du fait d’être noir et l’acceptation de cette identité, de son histoire, de sa culture et de sa destinée. Il en fait une valeur poétique et politique : la négritude vise à restaurer la dignité du peuple noir après la colonisation, en affirmant la beauté de la culture afro‑africaine, de ses langues, de ses rythmes et de son rapport à la vie et à la nature. &lt;/p&gt; &lt;p&gt; Dans sa poésie, il met en avant une sensibilité particulière, une « sensorialité » et une intuition qu’il oppose à la rationalité occidentale jugée plus froide, ce qui fait de ses vers une ode à la terre africaine, aux corps noirs, aux masques, aux danses et aux ancêtres. Des textes comme Femme noire ou Chants d’ombre célèbrent à la fois la femme‑enfant, la femme‑mère, la terre‑Afrique et la mémoire collective, dans une langue riche en images et en musique. &lt;/p&gt; &lt;p&gt; Par‑delà la négritude, il rêve d’une   &lt;a href=&quot;https://www.youtube.com/watch?v=sINJIeY4UKo&quot;  title=&quot;Senghor par RTS&quot;&gt;« Civilisation de l’Universel »,&lt;/a&gt;  c’est‑à‑dire d’un monde où différentes traditions (africaines, européennes, etc.) pourraient se mêler dans un métissage créateur plutôt que s’affronter. Philosophe politique, poète et humaniste, il reste l’une des figures majeures de la littérature francophone, à la fois comme chantre de la fierté noire et comme théoricien d’un dialogue entre cultures. &lt;/p&gt; &lt;audio controls title=&quot;Senghor ‘Tu te languis’ par France Culture&quot;&gt;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/21713-25.11.2025-ITEMA_24321734-2025C53416E0132-ITE_00154728_RSCE-21-996409c1a2c68ce243e4f4ef83e00211.mp3&quot; type=&quot;audio/mpeg&quot;&gt; &lt;/audio&gt;"/>
-    <hyperlink ref="E163" r:id="rId80" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Keiji_Nishitani&quot;  title=&quot;Wikipedia&quot;&gt;Keiji NISHITANI &lt;/a&gt; un philosophe japonais membre de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/%C3%89cole_de_Kyoto&quot;  title=&quot;école de Kyoto par Wikipedia&quot;&gt;l’École de Kyoto, &lt;/a&gt;  au côté de Nishida Kitarō et Tanabe Hajime, et l’un des penseurs modernes les plus originaux sur la religion, le bouddhisme et l’expérience du néant. Il cherche à penser ensemble la crise métaphysique de la modernité occidentale et la voie spirituelle du bouddhisme, notamment le zen et le bouddhisme du Vide (śūnyatā). &lt;/p&gt; &lt;p&gt; Sa réflexion prend comme point de départ le nihilisme moderne, c’est‑à‑dire le sentiment profond que tout est vidé de sens, de valeur et d’origine absolue, auquel il confronte l’expérience bouddhique de la vacuité radicale. Selon lui, la modernité enferme l’homme dans un soi narcissique et isolé, coupé de tout fondement ultime, et ce qui surgit alors n’est pas seulement le doute, mais une « grande incertitude » qui mène au vide de soi‑même. &lt;/p&gt; &lt;p&gt; Il propose alors une  &lt;a href=&quot;https://www.persee.fr/doc/ebisu_1340-3656_2005_num_34_1_1419&quot;  title=&quot;l’un e le tout en question par Persée&quot;&gt;« conversion » spirituelle &lt;/a&gt; : le même néant qui menaçait d’anéantir l’individu peut devenir, lorsque l’on cesse de le fuir, le point de départ d’une nouvelle compréhension du religieux, où le soi s’efface au profit d’une ouverture à l’être tout entier. Pour lui, la religion ne se réduit ni à dogme, ni à institution, ni à simple psychologie, mais à une expérience où le sujet, au cœur de sa plus grande déréliction, découvre que le monde peut être habité de sacrement, de manière « immanemment sainte ». &lt;/p&gt; &lt;p&gt; Il s’inscrit dans une entreprise de « philosophie entre Orient et Occident », où la pensée occidentale rencontre la tradition bouddhique pour repenser ensemble l’être, le mal, la liberté et la responsabilité. À travers des ouvrages comme Religion et néant (Religion and Nothingness), il devient l’une des figures clés du dialogue philosophique et religieux entre Asie et Europe, articulant la crise de la modernité et la possibilité d’une   &lt;a href=&quot;https://www.youtube.com/watch?v=Ak12Fplzo0U&quot;  title=&quot;The void is not the end Nishitani Keiji par NullSOPHY&quot;&gt;renaissance spirituelle &lt;/a&gt; fondée sur la vacuité éclairée. &lt;/p&gt;&#10;&#10;"/>
-    <hyperlink ref="H165" r:id="rId81" display="https://www.laphilo.fr/pho/knkrumah-mini.webp"/>
-    <hyperlink ref="E167" r:id="rId82" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Tran_Duc_Thao&quot; title=&quot; Wikipedia&quot;&gt;Tran Duc THAO&lt;/a&gt; était un philosophe vietnamien  connu pour sa tentative originale d’articuler phénoménologie et marxisme, ainsi que pour son engagement anticolonial et révolutionnaire.  Après la victoire vietnamienne de 1954, il retourne au Vietnam, enseigne à l’université de Hanoï et devient doyen de faculté, avant de connaître des mises à l’écart politiques et une relative marginalisation. &lt;/p&gt; &lt;p&gt; Son  &lt;a href=&quot;https://www.historicalmaterialism.org/figure/tran-duc-thao/&quot;  title=&quot;Tran Duc Thao par Historical materialism &quot;&gt;projet central  &lt;/a&gt; est de produire une synthèse entre phénoménologie et matérialisme dialectique, en partant de l’idée que la phénoménologie permet de saisir &quot;l’expérience vécue&quot; de la domination et du travail. &#10;Il cherche à &quot;réviser&quot; le marxisme pour le rendre attentif à la conscience, au vécu, à la subjectivité, tout en refusant un marxisme mécaniste qui réduirait tout au seul niveau économique. Cette synthèse est mise au service d’un projet politique anticolonial : il s’agit de penser l’émancipation à partir de la vie concrète des colonisés, en montrant le colonialisme comme une forme particulièrement &quot;perfectionnée&quot; du capitalisme. &lt;/p&gt; &lt;p&gt; Il publi en 1951 : &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie_et_mat%C3%A9rialisme_dialectique&quot;  title=&quot;Phénoménologie et matérialisme dialectique par Wikipedia &quot;&gt;&quot;Phénoménologie et matérialisme dialectique&quot; &lt;/a&gt;: Il y soutient que les limites de la phénoménologie ne peuvent être dépassées qu’en intégrant la théorie marxiste du travail et de la société, et que le marxisme a besoin d’une réélaboration phénoménologique pour retrouver &quot;l’inspiration originelle&quot; de Marx. &lt;/p&gt; &lt;p&gt; À partir des années 1960, il développe une théorie matérialiste de la conscience et du langage, en critiquant le structuralisme qui tend à enfermer le langage dans sa seule structure formelle. Il introduit notamment l’idée de &quot;langage de la vie réelle&quot; : un ensemble de significations objectives constituées dans l’activité matérielle des êtres humains, indépendamment de toute conscience individuelle. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie comme indissociable de la pratique politique : pour lui, la séparation entre théorie et pratique vient d’une compréhension insuffisante de la théorie et  affirme que la libération économique ne suffit pas si elle ne s’accompagne pas de &lt;a href=&quot;https://www.youtube.com/watch?v=NoHrpeGJpr8&quot; title=&quot; GAZA : POURQUOI DISCUTER NE SERT PLUS À RIEN par Padu &quot;&gt;libertés individuelles &lt;/a&gt; effectives (liberté d’expression, de réunion, etc.), distinguant ainsi contenu et forme de la liberté. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="E168" r:id="rId83" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cheikh_Anta_Diop&quot; title=&quot;Wikipedia&quot;&gt;Cheikh Anta DIOP&lt;/a&gt; était  un intellectuel sénégalais, historien, anthropologue, physicien et homme politique, considéré comme l’un des fondateurs de  &lt;a href=&quot;http://www.cheikhantadiop.net/&quot; title=&quot;cheikhantadiop &quot;&gt;l’historicité de l’Afrique &lt;/a&gt; et de la pensée afrocentrée. Né à Thieytou au Sénégal, il étudie la physique et la chimie en France, tout en approfondissant l’histoire et l’anthropologie, avant de devenir une figure majeure de la renaissance culturelle africaine dans la seconde moitié du XXᵉ siècle. Il milite aussi activement pour le panafricanisme et l’unification politique du continent, ce qui fait de lui à la fois un savant et un penseur politique engagé.  &lt;/p&gt; &lt;p&gt; Son apport le plus célèbre est la thèse selon laquelle l’Égypte ancienne est une   &lt;a href=&quot;https://www.persee.fr/doc/raipr_0033-9075_1969_num_9_1_1296&quot; title=&quot;civilisations Nègres par persée &quot;&gt;civilisation « nègre », &lt;/a&gt;  c’est‑à‑dire née d’une population d’origine subsaharienne et parente des peuples africains actuels. Dans Nations nègres et culture (1954) puis dans ses travaux ultérieurs, il mobilise des données linguistiques, anthropologiques et historiques pour montrer des parentés profondes entre les cosmo‑gonies égyptiennes et plusieurs traditions africaines (dogon, yoruba, ashanti, etc.), ce qui nourrit l’idée d’une « unité culturelle de l’Afrique noire ». Il entend ainsi retourner les discours racistes de l’époque en affirmant que l’Afrique n’est pas un continent sans histoire, mais que l’Égypte est un centre majeur de l’histoire africaine. &lt;/p&gt; &lt;p&gt; Sur le plan scientifique, il développe une approche pluridisciplinaire qui mêle linguistique, comparaison historique, anthropologie et études physique. Il critique fortement les biais culturels et eurocentrés de l’historiographie et de l’anthropologie coloniales, qui ont minimisé ou occulté l’apport des peuples africains aux civilisations humaines.  Pour lui, reconstituer &lt;a href=&quot;https://www.youtube.com/watch?v=KGlbVk3V9es&quot; title=&quot;conférence de Cheikh Anta Diop par pendanz &quot;&gt;une histoire africaine authentique &lt;/a&gt; permet non seulement de restaurer la dignité des peuples noirs, mais aussi de repenser l’histoire mondiale elle‑même. &lt;/p&gt; &lt;p&gt; Il est un penseur politique et un acteur de la scène panafricaniste : il défend un projet d’Afrique unifiée et fédéralisée, inspiré des idéaux de l’Unité africaine, et critique la division du continent héritée de la colonisation. Ses travaux influencent durablement les mouvements noirs, les études africaines et les réflexions sur la décolonisation des savoirs, tout en restant objet de débats parmi les égyptologues et les historiens. Aujourd’hui, il est souvent présenté comme l’un des grands précurseurs de la réhabilitation de l’Afrique dans l’histoire de l’humanité. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="E169" r:id="rId84" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Frantz_Fanon&quot; title=&quot;Wikipedia&quot;&gt;Frantz FANON&lt;/a&gt; était un penseur majeur de l’anticolonialisme, né en Martinique et devenu psychiatre, essayiste et militant engagé dans la guerre d’indépendance algérienne. Son œuvre cherche &lt;a href=&quot;https://www.youtube.com/watch?v=9hchLgKUSpU&quot; title=&quot;la Philosophie de Frantz FANON par parole de philosophe &quot;&gt;à comprendre comment &lt;/a&gt;  la colonisation détruit psychologiquement et socialement les peuples dominés, tout en fabriquant aussi une image déformée du colonisateur et du colonisé.&lt;/p&gt; &lt;p&gt; Dans Peau noire, masques blancs, il analyse la manière dont le racisme et la domination coloniale produisent un sentiment d’infériorité, des blessures psychiques et une aliénation de soi.  &lt;a href=&quot;https://fondation-frantzfanon.com/&quot; title=&quot;Fondation  Frantz FANON  &quot;&gt;Il montre que le colonisé &lt;/a&gt;  peut finir par intérioriser le regard du dominant, au point de porter un « masque » social pour tenter d’être reconnu dans un monde qui le rejette. &lt;/p&gt; &lt;p&gt; Sa pensée devient encore plus politique dans Les Damnés de la terre, où il défend l’idée que la décolonisation n’est pas seulement un changement administratif, mais une transformation radicale des rapports de pouvoir. Il insiste sur le fait que la colonisation repose elle-même sur la violence, et que la libération des colonisés passe par une rupture profonde avec cet ordre injuste. &lt;/p&gt; &lt;p&gt; Il est lu comme un précurseur des pensées décoloniales et postcoloniales, parce qu’il relie la politique, la psychologie, la culture et le corps vécu des dominés. Sa force est d’avoir montré que la lutte contre le colonialisme ne concerne pas seulement les territoires, mais aussi les esprits, les identités et les façons de penser le monde. &lt;/p&gt; &lt;audio controls title=&quot;Fanon, le phychiatre qui voulait libérer le monde par France Culture&quot;&gt;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/20905-24.05.2025-ITEMA_24146065-2025F23811S0145-NET_MFI_E4CF018B-14D9-469C-9942-543F6B9EFCA5-22.mp3&quot; type=&quot;audio/mpeg&quot;&gt; &lt;/audio&gt;"/>
-    <hyperlink ref="H169" r:id="rId85" display="https://www.laphilo.fr/pho/fanon-mini.webp"/>
-    <hyperlink ref="H184" r:id="rId86" display="https://www.laphilo.fr/pho/zayd-mini.webp"/>
+    <hyperlink ref="E163" r:id="rId79" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/L%C3%A9opold_S%C3%A9dar_Senghor&quot; title=&quot;Wikipedia&quot;&gt;Léopold Sédar SENGHOR&lt;/a&gt; était à la fois un grand poète-philosophe francophone et un homme d’État sénégalais, premier président de la République du Sénégal (1960–1980) et premier Africain membre de l’Académie française. Formé dans le système scolaire français, il incarne une figure hybride, à la croisée de l’Afrique et de la France, de la négritude et de la francophonie. &lt;/p&gt; &lt;p&gt; Au cœur de sa pensée se trouve le concept de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/N%C3%A9gritude&quot;  title=&quot;Négridude par Wikipedia&quot;&gt;« négritude », &lt;/a&gt; qu’il définit comme la reconnaissance du fait d’être noir et l’acceptation de cette identité, de son histoire, de sa culture et de sa destinée. Il en fait une valeur poétique et politique : la négritude vise à restaurer la dignité du peuple noir après la colonisation, en affirmant la beauté de la culture afro‑africaine, de ses langues, de ses rythmes et de son rapport à la vie et à la nature. &lt;/p&gt; &lt;p&gt; Dans sa poésie, il met en avant une sensibilité particulière, une « sensorialité » et une intuition qu’il oppose à la rationalité occidentale jugée plus froide, ce qui fait de ses vers une ode à la terre africaine, aux corps noirs, aux masques, aux danses et aux ancêtres. Des textes comme Femme noire ou Chants d’ombre célèbrent à la fois la femme‑enfant, la femme‑mère, la terre‑Afrique et la mémoire collective, dans une langue riche en images et en musique. &lt;/p&gt; &lt;p&gt; Par‑delà la négritude, il rêve d’une   &lt;a href=&quot;https://www.youtube.com/watch?v=sINJIeY4UKo&quot;  title=&quot;Senghor par RTS&quot;&gt;« Civilisation de l’Universel »,&lt;/a&gt;  c’est‑à‑dire d’un monde où différentes traditions (africaines, européennes, etc.) pourraient se mêler dans un métissage créateur plutôt que s’affronter. Philosophe politique, poète et humaniste, il reste l’une des figures majeures de la littérature francophone, à la fois comme chantre de la fierté noire et comme théoricien d’un dialogue entre cultures. &lt;/p&gt; &lt;audio controls title=&quot;Senghor ‘Tu te languis’ par France Culture&quot;&gt;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/21713-25.11.2025-ITEMA_24321734-2025C53416E0132-ITE_00154728_RSCE-21-996409c1a2c68ce243e4f4ef83e00211.mp3&quot; type=&quot;audio/mpeg&quot;&gt; &lt;/audio&gt;"/>
+    <hyperlink ref="E164" r:id="rId80" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Keiji_Nishitani&quot;  title=&quot;Wikipedia&quot;&gt;Keiji NISHITANI &lt;/a&gt; un philosophe japonais membre de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/%C3%89cole_de_Kyoto&quot;  title=&quot;école de Kyoto par Wikipedia&quot;&gt;l’École de Kyoto, &lt;/a&gt;  au côté de Nishida Kitarō et Tanabe Hajime, et l’un des penseurs modernes les plus originaux sur la religion, le bouddhisme et l’expérience du néant. Il cherche à penser ensemble la crise métaphysique de la modernité occidentale et la voie spirituelle du bouddhisme, notamment le zen et le bouddhisme du Vide (śūnyatā). &lt;/p&gt; &lt;p&gt; Sa réflexion prend comme point de départ le nihilisme moderne, c’est‑à‑dire le sentiment profond que tout est vidé de sens, de valeur et d’origine absolue, auquel il confronte l’expérience bouddhique de la vacuité radicale. Selon lui, la modernité enferme l’homme dans un soi narcissique et isolé, coupé de tout fondement ultime, et ce qui surgit alors n’est pas seulement le doute, mais une « grande incertitude » qui mène au vide de soi‑même. &lt;/p&gt; &lt;p&gt; Il propose alors une  &lt;a href=&quot;https://www.persee.fr/doc/ebisu_1340-3656_2005_num_34_1_1419&quot;  title=&quot;l’un e le tout en question par Persée&quot;&gt;« conversion » spirituelle &lt;/a&gt; : le même néant qui menaçait d’anéantir l’individu peut devenir, lorsque l’on cesse de le fuir, le point de départ d’une nouvelle compréhension du religieux, où le soi s’efface au profit d’une ouverture à l’être tout entier. Pour lui, la religion ne se réduit ni à dogme, ni à institution, ni à simple psychologie, mais à une expérience où le sujet, au cœur de sa plus grande déréliction, découvre que le monde peut être habité de sacrement, de manière « immanemment sainte ». &lt;/p&gt; &lt;p&gt; Il s’inscrit dans une entreprise de « philosophie entre Orient et Occident », où la pensée occidentale rencontre la tradition bouddhique pour repenser ensemble l’être, le mal, la liberté et la responsabilité. À travers des ouvrages comme Religion et néant (Religion and Nothingness), il devient l’une des figures clés du dialogue philosophique et religieux entre Asie et Europe, articulant la crise de la modernité et la possibilité d’une   &lt;a href=&quot;https://www.youtube.com/watch?v=Ak12Fplzo0U&quot;  title=&quot;The void is not the end Nishitani Keiji par NullSOPHY&quot;&gt;renaissance spirituelle &lt;/a&gt; fondée sur la vacuité éclairée. &lt;/p&gt;&#10;&#10;"/>
+    <hyperlink ref="H166" r:id="rId81" display="https://www.laphilo.fr/pho/knkrumah-mini.webp"/>
+    <hyperlink ref="E168" r:id="rId82" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Tran_Duc_Thao&quot; title=&quot; Wikipedia&quot;&gt;Tran Duc THAO&lt;/a&gt; était un philosophe vietnamien  connu pour sa tentative originale d’articuler phénoménologie et marxisme, ainsi que pour son engagement anticolonial et révolutionnaire.  Après la victoire vietnamienne de 1954, il retourne au Vietnam, enseigne à l’université de Hanoï et devient doyen de faculté, avant de connaître des mises à l’écart politiques et une relative marginalisation. &lt;/p&gt; &lt;p&gt; Son  &lt;a href=&quot;https://www.historicalmaterialism.org/figure/tran-duc-thao/&quot;  title=&quot;Tran Duc Thao par Historical materialism &quot;&gt;projet central  &lt;/a&gt; est de produire une synthèse entre phénoménologie et matérialisme dialectique, en partant de l’idée que la phénoménologie permet de saisir &quot;l’expérience vécue&quot; de la domination et du travail. &#10;Il cherche à &quot;réviser&quot; le marxisme pour le rendre attentif à la conscience, au vécu, à la subjectivité, tout en refusant un marxisme mécaniste qui réduirait tout au seul niveau économique. Cette synthèse est mise au service d’un projet politique anticolonial : il s’agit de penser l’émancipation à partir de la vie concrète des colonisés, en montrant le colonialisme comme une forme particulièrement &quot;perfectionnée&quot; du capitalisme. &lt;/p&gt; &lt;p&gt; Il publi en 1951 : &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie_et_mat%C3%A9rialisme_dialectique&quot;  title=&quot;Phénoménologie et matérialisme dialectique par Wikipedia &quot;&gt;&quot;Phénoménologie et matérialisme dialectique&quot; &lt;/a&gt;: Il y soutient que les limites de la phénoménologie ne peuvent être dépassées qu’en intégrant la théorie marxiste du travail et de la société, et que le marxisme a besoin d’une réélaboration phénoménologique pour retrouver &quot;l’inspiration originelle&quot; de Marx. &lt;/p&gt; &lt;p&gt; À partir des années 1960, il développe une théorie matérialiste de la conscience et du langage, en critiquant le structuralisme qui tend à enfermer le langage dans sa seule structure formelle. Il introduit notamment l’idée de &quot;langage de la vie réelle&quot; : un ensemble de significations objectives constituées dans l’activité matérielle des êtres humains, indépendamment de toute conscience individuelle. &lt;/p&gt; &lt;p&gt; Il conçoit la philosophie comme indissociable de la pratique politique : pour lui, la séparation entre théorie et pratique vient d’une compréhension insuffisante de la théorie et  affirme que la libération économique ne suffit pas si elle ne s’accompagne pas de &lt;a href=&quot;https://www.youtube.com/watch?v=NoHrpeGJpr8&quot; title=&quot; GAZA : POURQUOI DISCUTER NE SERT PLUS À RIEN par Padu &quot;&gt;libertés individuelles &lt;/a&gt; effectives (liberté d’expression, de réunion, etc.), distinguant ainsi contenu et forme de la liberté. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E169" r:id="rId83" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cheikh_Anta_Diop&quot; title=&quot;Wikipedia&quot;&gt;Cheikh Anta DIOP&lt;/a&gt; était  un intellectuel sénégalais, historien, anthropologue, physicien et homme politique, considéré comme l’un des fondateurs de  &lt;a href=&quot;http://www.cheikhantadiop.net/&quot; title=&quot;cheikhantadiop &quot;&gt;l’historicité de l’Afrique &lt;/a&gt; et de la pensée afrocentrée. Né à Thieytou au Sénégal, il étudie la physique et la chimie en France, tout en approfondissant l’histoire et l’anthropologie, avant de devenir une figure majeure de la renaissance culturelle africaine dans la seconde moitié du XXᵉ siècle. Il milite aussi activement pour le panafricanisme et l’unification politique du continent, ce qui fait de lui à la fois un savant et un penseur politique engagé.  &lt;/p&gt; &lt;p&gt; Son apport le plus célèbre est la thèse selon laquelle l’Égypte ancienne est une   &lt;a href=&quot;https://www.persee.fr/doc/raipr_0033-9075_1969_num_9_1_1296&quot; title=&quot;civilisations Nègres par persée &quot;&gt;civilisation « nègre », &lt;/a&gt;  c’est‑à‑dire née d’une population d’origine subsaharienne et parente des peuples africains actuels. Dans Nations nègres et culture (1954) puis dans ses travaux ultérieurs, il mobilise des données linguistiques, anthropologiques et historiques pour montrer des parentés profondes entre les cosmo‑gonies égyptiennes et plusieurs traditions africaines (dogon, yoruba, ashanti, etc.), ce qui nourrit l’idée d’une « unité culturelle de l’Afrique noire ». Il entend ainsi retourner les discours racistes de l’époque en affirmant que l’Afrique n’est pas un continent sans histoire, mais que l’Égypte est un centre majeur de l’histoire africaine. &lt;/p&gt; &lt;p&gt; Sur le plan scientifique, il développe une approche pluridisciplinaire qui mêle linguistique, comparaison historique, anthropologie et études physique. Il critique fortement les biais culturels et eurocentrés de l’historiographie et de l’anthropologie coloniales, qui ont minimisé ou occulté l’apport des peuples africains aux civilisations humaines.  Pour lui, reconstituer &lt;a href=&quot;https://www.youtube.com/watch?v=KGlbVk3V9es&quot; title=&quot;conférence de Cheikh Anta Diop par pendanz &quot;&gt;une histoire africaine authentique &lt;/a&gt; permet non seulement de restaurer la dignité des peuples noirs, mais aussi de repenser l’histoire mondiale elle‑même. &lt;/p&gt; &lt;p&gt; Il est un penseur politique et un acteur de la scène panafricaniste : il défend un projet d’Afrique unifiée et fédéralisée, inspiré des idéaux de l’Unité africaine, et critique la division du continent héritée de la colonisation. Ses travaux influencent durablement les mouvements noirs, les études africaines et les réflexions sur la décolonisation des savoirs, tout en restant objet de débats parmi les égyptologues et les historiens. Aujourd’hui, il est souvent présenté comme l’un des grands précurseurs de la réhabilitation de l’Afrique dans l’histoire de l’humanité. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E170" r:id="rId84" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Frantz_Fanon&quot; title=&quot;Wikipedia&quot;&gt;Frantz FANON&lt;/a&gt; était un penseur majeur de l’anticolonialisme, né en Martinique et devenu psychiatre, essayiste et militant engagé dans la guerre d’indépendance algérienne. Son œuvre cherche &lt;a href=&quot;https://www.youtube.com/watch?v=9hchLgKUSpU&quot; title=&quot;la Philosophie de Frantz FANON par parole de philosophe &quot;&gt;à comprendre comment &lt;/a&gt;  la colonisation détruit psychologiquement et socialement les peuples dominés, tout en fabriquant aussi une image déformée du colonisateur et du colonisé.&lt;/p&gt; &lt;p&gt; Dans Peau noire, masques blancs, il analyse la manière dont le racisme et la domination coloniale produisent un sentiment d’infériorité, des blessures psychiques et une aliénation de soi.  &lt;a href=&quot;https://fondation-frantzfanon.com/&quot; title=&quot;Fondation  Frantz FANON  &quot;&gt;Il montre que le colonisé &lt;/a&gt;  peut finir par intérioriser le regard du dominant, au point de porter un « masque » social pour tenter d’être reconnu dans un monde qui le rejette. &lt;/p&gt; &lt;p&gt; Sa pensée devient encore plus politique dans Les Damnés de la terre, où il défend l’idée que la décolonisation n’est pas seulement un changement administratif, mais une transformation radicale des rapports de pouvoir. Il insiste sur le fait que la colonisation repose elle-même sur la violence, et que la libération des colonisés passe par une rupture profonde avec cet ordre injuste. &lt;/p&gt; &lt;p&gt; Il est lu comme un précurseur des pensées décoloniales et postcoloniales, parce qu’il relie la politique, la psychologie, la culture et le corps vécu des dominés. Sa force est d’avoir montré que la lutte contre le colonialisme ne concerne pas seulement les territoires, mais aussi les esprits, les identités et les façons de penser le monde. &lt;/p&gt; &lt;audio controls title=&quot;Fanon, le phychiatre qui voulait libérer le monde par France Culture&quot;&gt;&lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/20905-24.05.2025-ITEMA_24146065-2025F23811S0145-NET_MFI_E4CF018B-14D9-469C-9942-543F6B9EFCA5-22.mp3&quot; type=&quot;audio/mpeg&quot;&gt; &lt;/audio&gt;"/>
+    <hyperlink ref="H170" r:id="rId85" display="https://www.laphilo.fr/pho/fanon-mini.webp"/>
+    <hyperlink ref="H185" r:id="rId86" display="https://www.laphilo.fr/pho/zayd-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>